<commit_message>
Made the Dragon race and standardized more of the things related to stats.
</commit_message>
<xml_diff>
--- a/Design/Tables.xlsx
+++ b/Design/Tables.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="27945" windowHeight="12180" activeTab="1"/>
+    <workbookView windowWidth="27945" windowHeight="11730" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="599" uniqueCount="407">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="592" uniqueCount="401">
   <si>
     <t>1-Handed (base) (5.5 base + 3 stat = 8.5) (8.5 - 4 AC)*2 hands = 9</t>
   </si>
@@ -749,9 +749,6 @@
     <t>XP Reward per Difficulty</t>
   </si>
   <si>
-    <t>Per Level</t>
-  </si>
-  <si>
     <r>
       <rPr>
         <sz val="12"/>
@@ -775,28 +772,6 @@
   <si>
     <r>
       <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <charset val="134"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">7.5 |    </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="4"/>
-        <rFont val="Calibri"/>
-        <charset val="134"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>AoE 6</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
         <sz val="12"/>
         <rFont val="Calibri"/>
         <charset val="134"/>
@@ -813,28 +788,6 @@
         <scheme val="minor"/>
       </rPr>
       <t>AoE 10</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <charset val="134"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> 15 | </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="4"/>
-        <rFont val="Calibri"/>
-        <charset val="134"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>AoE 12</t>
     </r>
   </si>
   <si>
@@ -883,28 +836,6 @@
   <si>
     <r>
       <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <charset val="134"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">5 |    </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="4"/>
-        <rFont val="Calibri"/>
-        <charset val="134"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>AoE 4</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
         <sz val="12"/>
         <rFont val="Calibri"/>
         <charset val="134"/>
@@ -954,28 +885,6 @@
         <charset val="134"/>
         <scheme val="minor"/>
       </rPr>
-      <t xml:space="preserve"> 12.5 | </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="4"/>
-        <rFont val="Calibri"/>
-        <charset val="134"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>AoE 10</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <charset val="134"/>
-        <scheme val="minor"/>
-      </rPr>
       <t xml:space="preserve">10 | </t>
     </r>
     <r>
@@ -987,28 +896,6 @@
         <scheme val="minor"/>
       </rPr>
       <t>AoE 4</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <charset val="134"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">21 | </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="4"/>
-        <rFont val="Calibri"/>
-        <charset val="134"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>AoE 16</t>
     </r>
   </si>
   <si>
@@ -5581,14 +5468,11 @@
         <v>22.5</v>
       </c>
     </row>
-    <row r="15" ht="15.75" spans="2:10">
+    <row r="15" ht="15.75" spans="2:6">
       <c r="B15" s="40"/>
       <c r="D15" s="40"/>
       <c r="E15" s="40"/>
       <c r="F15" s="40"/>
-      <c r="J15" t="s">
-        <v>161</v>
-      </c>
     </row>
     <row r="16" ht="15.75" spans="1:11">
       <c r="A16" s="48" t="s">
@@ -5604,9 +5488,6 @@
         <v>38</v>
       </c>
       <c r="E16" s="50" t="s">
-        <v>39</v>
-      </c>
-      <c r="F16" s="50" t="s">
         <v>40</v>
       </c>
       <c r="H16" s="40"/>
@@ -5630,9 +5511,6 @@
       <c r="E17" s="55">
         <v>0</v>
       </c>
-      <c r="F17" s="55">
-        <v>0</v>
-      </c>
       <c r="H17" s="40"/>
       <c r="K17">
         <v>6</v>
@@ -5646,15 +5524,12 @@
         <v>0</v>
       </c>
       <c r="C18" s="56" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="D18" s="40">
         <v>0</v>
       </c>
-      <c r="E18" s="55" t="s">
-        <v>163</v>
-      </c>
-      <c r="F18" s="55">
+      <c r="E18" s="55">
         <v>-1</v>
       </c>
       <c r="H18" s="57"/>
@@ -5670,16 +5545,16 @@
         <v>0</v>
       </c>
       <c r="C19" s="56" t="s">
-        <v>164</v>
+        <v>162</v>
       </c>
       <c r="D19" s="40">
         <v>0</v>
       </c>
-      <c r="E19" s="55" t="s">
-        <v>165</v>
-      </c>
-      <c r="F19" s="55">
+      <c r="E19" s="55">
         <v>-2</v>
+      </c>
+      <c r="G19">
+        <v>12</v>
       </c>
       <c r="H19" s="58"/>
       <c r="K19" s="70">
@@ -5694,22 +5569,16 @@
         <v>1</v>
       </c>
       <c r="C20" s="61" t="s">
-        <v>166</v>
+        <v>163</v>
       </c>
       <c r="D20" s="62" t="s">
-        <v>167</v>
-      </c>
-      <c r="E20" s="63" t="s">
-        <v>168</v>
-      </c>
-      <c r="F20" s="63">
+        <v>164</v>
+      </c>
+      <c r="E20" s="63">
         <v>-1</v>
       </c>
-      <c r="G20"/>
-      <c r="H20" s="57">
-        <f>5.5*3</f>
-        <v>16.5</v>
-      </c>
+      <c r="H20" s="57"/>
+      <c r="I20"/>
       <c r="J20" s="73"/>
       <c r="K20" s="70">
         <v>6</v>
@@ -5723,15 +5592,12 @@
         <v>1</v>
       </c>
       <c r="C21" s="56" t="s">
-        <v>169</v>
+        <v>165</v>
       </c>
       <c r="D21" s="64" t="s">
-        <v>170</v>
-      </c>
-      <c r="E21" s="55" t="s">
-        <v>171</v>
-      </c>
-      <c r="F21" s="55">
+        <v>166</v>
+      </c>
+      <c r="E21" s="55">
         <v>-2</v>
       </c>
       <c r="H21" s="58"/>
@@ -5750,12 +5616,9 @@
         <v>50</v>
       </c>
       <c r="D22" s="45" t="s">
-        <v>172</v>
-      </c>
-      <c r="E22" s="43" t="s">
-        <v>173</v>
-      </c>
-      <c r="F22" s="43">
+        <v>167</v>
+      </c>
+      <c r="E22" s="43">
         <v>-3</v>
       </c>
       <c r="H22" s="58"/>
@@ -5776,8 +5639,7 @@
       <c r="D23" s="68">
         <v>2</v>
       </c>
-      <c r="E23" s="51"/>
-      <c r="F23" s="50">
+      <c r="E23" s="50">
         <v>3</v>
       </c>
       <c r="G23" s="40"/>
@@ -5801,8 +5663,7 @@
       <c r="D24" s="66">
         <v>4</v>
       </c>
-      <c r="E24" s="45"/>
-      <c r="F24" s="43">
+      <c r="E24" s="43">
         <v>5.5</v>
       </c>
       <c r="G24" s="40"/>
@@ -5864,10 +5725,10 @@
         <v>0</v>
       </c>
       <c r="C28" s="39" t="s">
-        <v>174</v>
+        <v>168</v>
       </c>
       <c r="D28" s="40" t="s">
-        <v>175</v>
+        <v>169</v>
       </c>
       <c r="E28" s="51"/>
       <c r="F28" s="83"/>
@@ -5881,10 +5742,10 @@
         <v>0</v>
       </c>
       <c r="C29" s="84" t="s">
-        <v>176</v>
+        <v>170</v>
       </c>
       <c r="D29" s="85" t="s">
-        <v>177</v>
+        <v>171</v>
       </c>
       <c r="E29" s="40"/>
       <c r="F29" s="41"/>
@@ -5911,16 +5772,16 @@
         <v>1</v>
       </c>
       <c r="C31" s="39" t="s">
-        <v>178</v>
+        <v>172</v>
       </c>
       <c r="D31" s="40" t="s">
-        <v>179</v>
+        <v>173</v>
       </c>
       <c r="E31" s="40" t="s">
         <v>65</v>
       </c>
       <c r="F31" s="41" t="s">
-        <v>180</v>
+        <v>174</v>
       </c>
     </row>
     <row r="32" spans="1:6">
@@ -6045,7 +5906,7 @@
       </c>
       <c r="G39" s="40"/>
       <c r="H39" s="40" t="s">
-        <v>181</v>
+        <v>175</v>
       </c>
       <c r="I39" s="40"/>
       <c r="J39" s="40"/>
@@ -6072,7 +5933,7 @@
         <v>145</v>
       </c>
       <c r="I40" s="50" t="s">
-        <v>182</v>
+        <v>176</v>
       </c>
       <c r="K40" s="58"/>
     </row>
@@ -6224,7 +6085,7 @@
         <v>10</v>
       </c>
       <c r="F46" t="s">
-        <v>183</v>
+        <v>177</v>
       </c>
       <c r="G46" s="39">
         <v>6</v>
@@ -6251,7 +6112,7 @@
         <v>11</v>
       </c>
       <c r="F47" t="s">
-        <v>184</v>
+        <v>178</v>
       </c>
       <c r="G47" s="39">
         <v>7</v>
@@ -6281,7 +6142,7 @@
         <v>11</v>
       </c>
       <c r="F48" t="s">
-        <v>185</v>
+        <v>179</v>
       </c>
       <c r="G48" s="39">
         <v>8</v>
@@ -6311,7 +6172,7 @@
         <v>11</v>
       </c>
       <c r="F49" t="s">
-        <v>186</v>
+        <v>180</v>
       </c>
       <c r="G49" s="39">
         <v>9</v>
@@ -6338,7 +6199,7 @@
         <v>11</v>
       </c>
       <c r="F50" t="s">
-        <v>187</v>
+        <v>181</v>
       </c>
       <c r="G50" s="44">
         <v>10</v>
@@ -6368,7 +6229,7 @@
         <v>12</v>
       </c>
       <c r="F51" t="s">
-        <v>188</v>
+        <v>182</v>
       </c>
       <c r="G51" s="40"/>
       <c r="H51" s="40"/>
@@ -6394,16 +6255,16 @@
         <v>12</v>
       </c>
       <c r="G52" s="96" t="s">
-        <v>189</v>
+        <v>183</v>
       </c>
       <c r="H52" s="96" t="s">
-        <v>190</v>
+        <v>184</v>
       </c>
       <c r="I52" s="103" t="s">
-        <v>191</v>
+        <v>185</v>
       </c>
       <c r="J52" s="104" t="s">
-        <v>192</v>
+        <v>186</v>
       </c>
       <c r="M52" s="58"/>
     </row>
@@ -6424,7 +6285,7 @@
         <v>12</v>
       </c>
       <c r="G53" s="97" t="s">
-        <v>193</v>
+        <v>187</v>
       </c>
       <c r="H53" s="97">
         <v>16</v>
@@ -6455,7 +6316,7 @@
         <v>12</v>
       </c>
       <c r="G54" s="39" t="s">
-        <v>194</v>
+        <v>188</v>
       </c>
       <c r="H54" s="39">
         <v>18</v>
@@ -6482,7 +6343,7 @@
         <v>12</v>
       </c>
       <c r="G55" s="39" t="s">
-        <v>195</v>
+        <v>189</v>
       </c>
       <c r="H55" s="39">
         <v>21</v>
@@ -6509,7 +6370,7 @@
         <v>12</v>
       </c>
       <c r="G56" s="39" t="s">
-        <v>196</v>
+        <v>190</v>
       </c>
       <c r="H56" s="39">
         <v>22</v>
@@ -6536,7 +6397,7 @@
         <v>12</v>
       </c>
       <c r="G57" s="42" t="s">
-        <v>197</v>
+        <v>191</v>
       </c>
       <c r="H57" s="42">
         <v>16</v>
@@ -6563,7 +6424,7 @@
         <v>12</v>
       </c>
       <c r="G58" s="39" t="s">
-        <v>198</v>
+        <v>192</v>
       </c>
       <c r="H58" s="39">
         <v>14</v>
@@ -6590,7 +6451,7 @@
         <v>12</v>
       </c>
       <c r="G59" s="39" t="s">
-        <v>199</v>
+        <v>193</v>
       </c>
       <c r="H59" s="39">
         <v>20</v>
@@ -6615,7 +6476,7 @@
         <v>13</v>
       </c>
       <c r="G60" s="39" t="s">
-        <v>200</v>
+        <v>194</v>
       </c>
       <c r="H60" s="39">
         <v>17</v>
@@ -6640,7 +6501,7 @@
         <v>13</v>
       </c>
       <c r="G61" s="44" t="s">
-        <v>201</v>
+        <v>195</v>
       </c>
       <c r="H61" s="44">
         <v>26</v>
@@ -6683,38 +6544,38 @@
         <v>235.2</v>
       </c>
       <c r="C65" s="105" t="s">
-        <v>202</v>
+        <v>196</v>
       </c>
       <c r="D65" s="105" t="s">
-        <v>203</v>
+        <v>197</v>
       </c>
       <c r="E65" s="105" t="s">
-        <v>204</v>
+        <v>198</v>
       </c>
       <c r="G65" s="40"/>
       <c r="H65" s="106" t="s">
-        <v>205</v>
+        <v>199</v>
       </c>
       <c r="I65" t="s">
-        <v>206</v>
+        <v>200</v>
       </c>
       <c r="J65" s="58"/>
     </row>
     <row r="66" ht="90.75" spans="3:10">
       <c r="C66" s="105" t="s">
-        <v>207</v>
+        <v>201</v>
       </c>
       <c r="E66" s="40"/>
       <c r="F66" s="40"/>
       <c r="G66" s="40"/>
       <c r="H66" s="40" t="s">
-        <v>208</v>
+        <v>202</v>
       </c>
       <c r="I66" t="s">
-        <v>209</v>
+        <v>203</v>
       </c>
       <c r="J66" s="40" t="s">
-        <v>210</v>
+        <v>204</v>
       </c>
     </row>
     <row r="67" spans="5:10">
@@ -6722,13 +6583,13 @@
       <c r="F67" s="40"/>
       <c r="G67" s="40"/>
       <c r="H67" s="40" t="s">
-        <v>208</v>
+        <v>202</v>
       </c>
       <c r="I67" t="s">
-        <v>211</v>
+        <v>205</v>
       </c>
       <c r="J67" s="40" t="s">
-        <v>210</v>
+        <v>204</v>
       </c>
     </row>
     <row r="68" spans="3:10">
@@ -6737,13 +6598,13 @@
       <c r="F68" s="40"/>
       <c r="G68" s="40"/>
       <c r="H68" s="40" t="s">
-        <v>208</v>
+        <v>202</v>
       </c>
       <c r="I68" t="s">
-        <v>212</v>
+        <v>206</v>
       </c>
       <c r="J68" s="40" t="s">
-        <v>213</v>
+        <v>207</v>
       </c>
     </row>
     <row r="69" ht="13" customHeight="1" spans="5:10">
@@ -6751,13 +6612,13 @@
       <c r="F69" s="40"/>
       <c r="G69" s="40"/>
       <c r="H69" s="40" t="s">
-        <v>214</v>
+        <v>208</v>
       </c>
       <c r="I69" s="106" t="s">
-        <v>215</v>
+        <v>209</v>
       </c>
       <c r="J69" s="40" t="s">
-        <v>213</v>
+        <v>207</v>
       </c>
     </row>
     <row r="70" spans="5:10">
@@ -6765,13 +6626,13 @@
       <c r="F70" s="40"/>
       <c r="G70" s="40"/>
       <c r="H70" s="40" t="s">
-        <v>216</v>
+        <v>210</v>
       </c>
       <c r="I70" s="106" t="s">
-        <v>217</v>
+        <v>211</v>
       </c>
       <c r="J70" s="40" t="s">
-        <v>218</v>
+        <v>212</v>
       </c>
     </row>
     <row r="71" ht="15.75" spans="1:14">
@@ -6804,7 +6665,7 @@
       <c r="A73" s="40"/>
       <c r="F73" s="40"/>
       <c r="G73" s="111" t="s">
-        <v>193</v>
+        <v>187</v>
       </c>
       <c r="H73" s="111"/>
       <c r="I73" s="111"/>
@@ -6817,7 +6678,7 @@
       <c r="A74" s="40"/>
       <c r="F74" s="40"/>
       <c r="G74" s="40" t="s">
-        <v>194</v>
+        <v>188</v>
       </c>
       <c r="H74" s="40"/>
       <c r="I74" s="40"/>
@@ -6831,7 +6692,7 @@
       <c r="A75" s="40"/>
       <c r="F75" s="40"/>
       <c r="G75" s="40" t="s">
-        <v>195</v>
+        <v>189</v>
       </c>
       <c r="H75" s="40"/>
       <c r="I75" s="40"/>
@@ -6845,7 +6706,7 @@
       <c r="A76" s="40"/>
       <c r="F76" s="40"/>
       <c r="G76" s="40" t="s">
-        <v>196</v>
+        <v>190</v>
       </c>
       <c r="H76" s="40"/>
       <c r="I76" s="40"/>
@@ -6858,7 +6719,7 @@
       <c r="A77" s="108"/>
       <c r="F77" s="40"/>
       <c r="G77" s="112" t="s">
-        <v>197</v>
+        <v>191</v>
       </c>
       <c r="H77" s="112"/>
       <c r="I77" s="112"/>
@@ -6872,7 +6733,7 @@
       <c r="A78" s="40"/>
       <c r="F78" s="40"/>
       <c r="G78" s="40" t="s">
-        <v>198</v>
+        <v>192</v>
       </c>
       <c r="H78" s="40"/>
       <c r="I78" s="40"/>
@@ -6885,7 +6746,7 @@
       <c r="A79" s="40"/>
       <c r="F79" s="40"/>
       <c r="G79" s="40" t="s">
-        <v>200</v>
+        <v>194</v>
       </c>
       <c r="H79" s="40"/>
       <c r="I79" s="40"/>
@@ -6899,7 +6760,7 @@
       <c r="A80" s="40"/>
       <c r="F80" s="40"/>
       <c r="G80" s="40" t="s">
-        <v>199</v>
+        <v>193</v>
       </c>
       <c r="H80" s="40"/>
       <c r="I80" s="40"/>
@@ -6913,7 +6774,7 @@
       <c r="A81" s="40"/>
       <c r="F81" s="40"/>
       <c r="G81" s="40" t="s">
-        <v>201</v>
+        <v>195</v>
       </c>
       <c r="H81" s="40"/>
       <c r="I81" s="40"/>
@@ -7202,31 +7063,31 @@
   <sheetData>
     <row r="1" spans="1:9">
       <c r="A1" s="2" t="s">
+        <v>213</v>
+      </c>
+      <c r="B1" s="3" t="s">
+        <v>214</v>
+      </c>
+      <c r="C1" s="3" t="s">
+        <v>215</v>
+      </c>
+      <c r="D1" s="3" t="s">
+        <v>216</v>
+      </c>
+      <c r="E1" s="3" t="s">
+        <v>217</v>
+      </c>
+      <c r="F1" s="3" t="s">
+        <v>218</v>
+      </c>
+      <c r="G1" s="3" t="s">
         <v>219</v>
       </c>
-      <c r="B1" s="3" t="s">
+      <c r="H1" s="3" t="s">
         <v>220</v>
       </c>
-      <c r="C1" s="3" t="s">
+      <c r="I1" s="16" t="s">
         <v>221</v>
-      </c>
-      <c r="D1" s="3" t="s">
-        <v>222</v>
-      </c>
-      <c r="E1" s="3" t="s">
-        <v>223</v>
-      </c>
-      <c r="F1" s="3" t="s">
-        <v>224</v>
-      </c>
-      <c r="G1" s="3" t="s">
-        <v>225</v>
-      </c>
-      <c r="H1" s="3" t="s">
-        <v>226</v>
-      </c>
-      <c r="I1" s="16" t="s">
-        <v>227</v>
       </c>
     </row>
     <row r="2" spans="1:9">
@@ -7234,28 +7095,28 @@
         <v>0</v>
       </c>
       <c r="B2" s="5" t="s">
-        <v>228</v>
+        <v>222</v>
       </c>
       <c r="C2" s="6" t="s">
-        <v>229</v>
+        <v>223</v>
       </c>
       <c r="D2" s="6" t="s">
-        <v>228</v>
+        <v>222</v>
       </c>
       <c r="E2" s="5" t="s">
-        <v>228</v>
+        <v>222</v>
       </c>
       <c r="F2" s="6" t="s">
-        <v>228</v>
+        <v>222</v>
       </c>
       <c r="G2" s="6" t="s">
-        <v>229</v>
+        <v>223</v>
       </c>
       <c r="H2" s="6" t="s">
-        <v>230</v>
+        <v>224</v>
       </c>
       <c r="I2" s="6" t="s">
-        <v>230</v>
+        <v>224</v>
       </c>
     </row>
     <row r="3" spans="1:9">
@@ -7263,28 +7124,28 @@
         <v>1</v>
       </c>
       <c r="B3" s="5" t="s">
-        <v>231</v>
+        <v>225</v>
       </c>
       <c r="C3" s="6" t="s">
-        <v>232</v>
+        <v>226</v>
       </c>
       <c r="D3" s="6" t="s">
-        <v>231</v>
+        <v>225</v>
       </c>
       <c r="E3" s="5" t="s">
-        <v>233</v>
+        <v>227</v>
       </c>
       <c r="F3" s="6" t="s">
-        <v>231</v>
+        <v>225</v>
       </c>
       <c r="G3" s="6" t="s">
-        <v>232</v>
+        <v>226</v>
       </c>
       <c r="H3" s="6" t="s">
-        <v>234</v>
+        <v>228</v>
       </c>
       <c r="I3" s="6" t="s">
-        <v>234</v>
+        <v>228</v>
       </c>
     </row>
     <row r="4" spans="1:9">
@@ -7292,28 +7153,28 @@
         <v>2</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>235</v>
+        <v>229</v>
       </c>
       <c r="C4" s="6" t="s">
-        <v>236</v>
+        <v>230</v>
       </c>
       <c r="D4" s="6" t="s">
-        <v>235</v>
+        <v>229</v>
       </c>
       <c r="E4" s="5" t="s">
-        <v>235</v>
+        <v>229</v>
       </c>
       <c r="F4" s="6" t="s">
-        <v>235</v>
+        <v>229</v>
       </c>
       <c r="G4" s="6" t="s">
-        <v>236</v>
+        <v>230</v>
       </c>
       <c r="H4" s="6" t="s">
-        <v>237</v>
+        <v>231</v>
       </c>
       <c r="I4" s="6" t="s">
-        <v>237</v>
+        <v>231</v>
       </c>
     </row>
     <row r="5" spans="1:9">
@@ -7321,28 +7182,28 @@
         <v>3</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>238</v>
+        <v>232</v>
       </c>
       <c r="C5" s="6" t="s">
-        <v>239</v>
+        <v>233</v>
       </c>
       <c r="D5" s="6" t="s">
-        <v>240</v>
+        <v>234</v>
       </c>
       <c r="E5" s="5" t="s">
-        <v>240</v>
+        <v>234</v>
       </c>
       <c r="F5" s="6" t="s">
-        <v>240</v>
+        <v>234</v>
       </c>
       <c r="G5" s="6" t="s">
-        <v>239</v>
+        <v>233</v>
       </c>
       <c r="H5" s="6" t="s">
-        <v>241</v>
+        <v>235</v>
       </c>
       <c r="I5" s="6" t="s">
-        <v>242</v>
+        <v>236</v>
       </c>
     </row>
     <row r="6" spans="1:9">
@@ -7350,28 +7211,28 @@
         <v>4</v>
       </c>
       <c r="B6" s="5" t="s">
+        <v>237</v>
+      </c>
+      <c r="C6" s="6" t="s">
+        <v>238</v>
+      </c>
+      <c r="D6" s="6" t="s">
+        <v>239</v>
+      </c>
+      <c r="E6" s="5" t="s">
+        <v>240</v>
+      </c>
+      <c r="F6" s="6" t="s">
+        <v>241</v>
+      </c>
+      <c r="G6" s="6" t="s">
+        <v>238</v>
+      </c>
+      <c r="H6" s="6" t="s">
+        <v>242</v>
+      </c>
+      <c r="I6" s="6" t="s">
         <v>243</v>
-      </c>
-      <c r="C6" s="6" t="s">
-        <v>244</v>
-      </c>
-      <c r="D6" s="6" t="s">
-        <v>245</v>
-      </c>
-      <c r="E6" s="5" t="s">
-        <v>246</v>
-      </c>
-      <c r="F6" s="6" t="s">
-        <v>247</v>
-      </c>
-      <c r="G6" s="6" t="s">
-        <v>244</v>
-      </c>
-      <c r="H6" s="6" t="s">
-        <v>248</v>
-      </c>
-      <c r="I6" s="6" t="s">
-        <v>249</v>
       </c>
     </row>
     <row r="7" spans="1:9">
@@ -7379,28 +7240,28 @@
         <v>5</v>
       </c>
       <c r="B7" s="5" t="s">
+        <v>244</v>
+      </c>
+      <c r="C7" s="6" t="s">
+        <v>245</v>
+      </c>
+      <c r="D7" s="6" t="s">
+        <v>246</v>
+      </c>
+      <c r="E7" s="5" t="s">
+        <v>247</v>
+      </c>
+      <c r="F7" s="6" t="s">
+        <v>248</v>
+      </c>
+      <c r="G7" s="6" t="s">
+        <v>245</v>
+      </c>
+      <c r="H7" s="6" t="s">
+        <v>249</v>
+      </c>
+      <c r="I7" s="6" t="s">
         <v>250</v>
-      </c>
-      <c r="C7" s="6" t="s">
-        <v>251</v>
-      </c>
-      <c r="D7" s="6" t="s">
-        <v>252</v>
-      </c>
-      <c r="E7" s="5" t="s">
-        <v>253</v>
-      </c>
-      <c r="F7" s="6" t="s">
-        <v>254</v>
-      </c>
-      <c r="G7" s="6" t="s">
-        <v>251</v>
-      </c>
-      <c r="H7" s="6" t="s">
-        <v>255</v>
-      </c>
-      <c r="I7" s="6" t="s">
-        <v>256</v>
       </c>
     </row>
     <row r="8" spans="1:9">
@@ -7408,28 +7269,28 @@
         <v>6</v>
       </c>
       <c r="B8" s="5" t="s">
+        <v>251</v>
+      </c>
+      <c r="C8" s="6" t="s">
+        <v>252</v>
+      </c>
+      <c r="D8" s="6" t="s">
+        <v>253</v>
+      </c>
+      <c r="E8" s="5" t="s">
+        <v>254</v>
+      </c>
+      <c r="F8" s="6" t="s">
+        <v>255</v>
+      </c>
+      <c r="G8" s="6" t="s">
+        <v>256</v>
+      </c>
+      <c r="H8" s="6" t="s">
         <v>257</v>
       </c>
-      <c r="C8" s="6" t="s">
+      <c r="I8" s="6" t="s">
         <v>258</v>
-      </c>
-      <c r="D8" s="6" t="s">
-        <v>259</v>
-      </c>
-      <c r="E8" s="5" t="s">
-        <v>260</v>
-      </c>
-      <c r="F8" s="6" t="s">
-        <v>261</v>
-      </c>
-      <c r="G8" s="6" t="s">
-        <v>262</v>
-      </c>
-      <c r="H8" s="6" t="s">
-        <v>263</v>
-      </c>
-      <c r="I8" s="6" t="s">
-        <v>264</v>
       </c>
     </row>
     <row r="9" spans="1:9">
@@ -7437,28 +7298,28 @@
         <v>7</v>
       </c>
       <c r="B9" s="5" t="s">
+        <v>259</v>
+      </c>
+      <c r="C9" s="6" t="s">
+        <v>260</v>
+      </c>
+      <c r="D9" s="6" t="s">
+        <v>261</v>
+      </c>
+      <c r="E9" s="5" t="s">
+        <v>262</v>
+      </c>
+      <c r="F9" s="6" t="s">
+        <v>263</v>
+      </c>
+      <c r="G9" s="6" t="s">
+        <v>264</v>
+      </c>
+      <c r="H9" s="6" t="s">
         <v>265</v>
       </c>
-      <c r="C9" s="6" t="s">
+      <c r="I9" s="6" t="s">
         <v>266</v>
-      </c>
-      <c r="D9" s="6" t="s">
-        <v>267</v>
-      </c>
-      <c r="E9" s="5" t="s">
-        <v>268</v>
-      </c>
-      <c r="F9" s="6" t="s">
-        <v>269</v>
-      </c>
-      <c r="G9" s="6" t="s">
-        <v>270</v>
-      </c>
-      <c r="H9" s="6" t="s">
-        <v>271</v>
-      </c>
-      <c r="I9" s="6" t="s">
-        <v>272</v>
       </c>
     </row>
     <row r="10" spans="1:9">
@@ -7466,28 +7327,28 @@
         <v>8</v>
       </c>
       <c r="B10" s="5" t="s">
+        <v>267</v>
+      </c>
+      <c r="C10" s="6" t="s">
+        <v>268</v>
+      </c>
+      <c r="D10" s="6" t="s">
+        <v>269</v>
+      </c>
+      <c r="E10" s="5" t="s">
+        <v>270</v>
+      </c>
+      <c r="F10" s="6" t="s">
+        <v>271</v>
+      </c>
+      <c r="G10" s="6" t="s">
+        <v>272</v>
+      </c>
+      <c r="H10" s="6" t="s">
         <v>273</v>
       </c>
-      <c r="C10" s="6" t="s">
+      <c r="I10" s="6" t="s">
         <v>274</v>
-      </c>
-      <c r="D10" s="6" t="s">
-        <v>275</v>
-      </c>
-      <c r="E10" s="5" t="s">
-        <v>276</v>
-      </c>
-      <c r="F10" s="6" t="s">
-        <v>277</v>
-      </c>
-      <c r="G10" s="6" t="s">
-        <v>278</v>
-      </c>
-      <c r="H10" s="6" t="s">
-        <v>279</v>
-      </c>
-      <c r="I10" s="6" t="s">
-        <v>280</v>
       </c>
     </row>
     <row r="11" spans="1:9">
@@ -7495,28 +7356,28 @@
         <v>9</v>
       </c>
       <c r="B11" s="5" t="s">
+        <v>275</v>
+      </c>
+      <c r="C11" s="6" t="s">
+        <v>276</v>
+      </c>
+      <c r="D11" s="6" t="s">
+        <v>277</v>
+      </c>
+      <c r="E11" s="5" t="s">
+        <v>278</v>
+      </c>
+      <c r="F11" s="6" t="s">
+        <v>279</v>
+      </c>
+      <c r="G11" s="6" t="s">
+        <v>280</v>
+      </c>
+      <c r="H11" s="6" t="s">
         <v>281</v>
       </c>
-      <c r="C11" s="6" t="s">
+      <c r="I11" s="6" t="s">
         <v>282</v>
-      </c>
-      <c r="D11" s="6" t="s">
-        <v>283</v>
-      </c>
-      <c r="E11" s="5" t="s">
-        <v>284</v>
-      </c>
-      <c r="F11" s="6" t="s">
-        <v>285</v>
-      </c>
-      <c r="G11" s="6" t="s">
-        <v>286</v>
-      </c>
-      <c r="H11" s="6" t="s">
-        <v>287</v>
-      </c>
-      <c r="I11" s="6" t="s">
-        <v>288</v>
       </c>
     </row>
     <row r="12" spans="1:9">
@@ -7524,28 +7385,28 @@
         <v>10</v>
       </c>
       <c r="B12" s="5" t="s">
+        <v>283</v>
+      </c>
+      <c r="C12" s="6" t="s">
+        <v>284</v>
+      </c>
+      <c r="D12" s="6" t="s">
+        <v>285</v>
+      </c>
+      <c r="E12" s="5" t="s">
+        <v>286</v>
+      </c>
+      <c r="F12" s="6" t="s">
+        <v>287</v>
+      </c>
+      <c r="G12" s="6" t="s">
+        <v>288</v>
+      </c>
+      <c r="H12" s="6" t="s">
         <v>289</v>
       </c>
-      <c r="C12" s="6" t="s">
+      <c r="I12" s="6" t="s">
         <v>290</v>
-      </c>
-      <c r="D12" s="6" t="s">
-        <v>291</v>
-      </c>
-      <c r="E12" s="5" t="s">
-        <v>292</v>
-      </c>
-      <c r="F12" s="6" t="s">
-        <v>293</v>
-      </c>
-      <c r="G12" s="6" t="s">
-        <v>294</v>
-      </c>
-      <c r="H12" s="6" t="s">
-        <v>295</v>
-      </c>
-      <c r="I12" s="6" t="s">
-        <v>296</v>
       </c>
     </row>
     <row r="13" spans="1:9">
@@ -7553,28 +7414,28 @@
         <v>11</v>
       </c>
       <c r="B13" s="5" t="s">
-        <v>297</v>
+        <v>291</v>
       </c>
       <c r="C13" s="6" t="s">
+        <v>288</v>
+      </c>
+      <c r="D13" s="6" t="s">
+        <v>292</v>
+      </c>
+      <c r="E13" s="5" t="s">
+        <v>293</v>
+      </c>
+      <c r="F13" s="6" t="s">
         <v>294</v>
       </c>
-      <c r="D13" s="6" t="s">
-        <v>298</v>
-      </c>
-      <c r="E13" s="5" t="s">
-        <v>299</v>
-      </c>
-      <c r="F13" s="6" t="s">
-        <v>300</v>
-      </c>
       <c r="G13" s="6" t="s">
-        <v>294</v>
+        <v>288</v>
       </c>
       <c r="H13" s="6" t="s">
-        <v>301</v>
+        <v>295</v>
       </c>
       <c r="I13" s="6" t="s">
-        <v>302</v>
+        <v>296</v>
       </c>
     </row>
     <row r="14" ht="19.5" spans="1:9">
@@ -7582,33 +7443,33 @@
         <v>12</v>
       </c>
       <c r="B14" s="5" t="s">
-        <v>303</v>
+        <v>297</v>
       </c>
       <c r="C14" s="6" t="s">
-        <v>294</v>
+        <v>288</v>
       </c>
       <c r="D14" s="6" t="s">
-        <v>302</v>
+        <v>296</v>
       </c>
       <c r="E14" s="5" t="s">
-        <v>304</v>
+        <v>298</v>
       </c>
       <c r="F14" s="6" t="s">
-        <v>305</v>
+        <v>299</v>
       </c>
       <c r="G14" s="6" t="s">
-        <v>294</v>
+        <v>288</v>
       </c>
       <c r="H14" s="6" t="s">
-        <v>306</v>
+        <v>300</v>
       </c>
       <c r="I14" s="6" t="s">
-        <v>302</v>
+        <v>296</v>
       </c>
     </row>
     <row r="15" ht="19.5" spans="1:9">
       <c r="A15" s="8" t="s">
-        <v>307</v>
+        <v>301</v>
       </c>
       <c r="B15" s="9" t="s">
         <v>4</v>
@@ -7640,34 +7501,34 @@
     </row>
     <row r="18" spans="1:10">
       <c r="A18" s="2" t="s">
+        <v>302</v>
+      </c>
+      <c r="B18" s="3" t="s">
+        <v>303</v>
+      </c>
+      <c r="C18" s="3" t="s">
+        <v>304</v>
+      </c>
+      <c r="D18" s="3" t="s">
+        <v>305</v>
+      </c>
+      <c r="E18" s="3" t="s">
+        <v>306</v>
+      </c>
+      <c r="F18" s="3" t="s">
+        <v>307</v>
+      </c>
+      <c r="G18" s="3" t="s">
         <v>308</v>
       </c>
-      <c r="B18" s="3" t="s">
+      <c r="H18" s="3" t="s">
         <v>309</v>
       </c>
-      <c r="C18" s="3" t="s">
+      <c r="I18" s="3" t="s">
         <v>310</v>
       </c>
-      <c r="D18" s="3" t="s">
+      <c r="J18" s="3" t="s">
         <v>311</v>
-      </c>
-      <c r="E18" s="3" t="s">
-        <v>312</v>
-      </c>
-      <c r="F18" s="3" t="s">
-        <v>313</v>
-      </c>
-      <c r="G18" s="3" t="s">
-        <v>314</v>
-      </c>
-      <c r="H18" s="3" t="s">
-        <v>315</v>
-      </c>
-      <c r="I18" s="3" t="s">
-        <v>316</v>
-      </c>
-      <c r="J18" s="3" t="s">
-        <v>317</v>
       </c>
     </row>
     <row r="19" spans="1:10">
@@ -7675,31 +7536,31 @@
         <v>0</v>
       </c>
       <c r="B19" s="5" t="s">
-        <v>318</v>
+        <v>312</v>
       </c>
       <c r="C19" s="5" t="s">
-        <v>319</v>
+        <v>313</v>
       </c>
       <c r="D19" s="6" t="s">
-        <v>318</v>
+        <v>312</v>
       </c>
       <c r="E19" s="6" t="s">
-        <v>318</v>
+        <v>312</v>
       </c>
       <c r="F19" s="5" t="s">
-        <v>318</v>
+        <v>312</v>
       </c>
       <c r="G19" s="11" t="s">
-        <v>318</v>
+        <v>312</v>
       </c>
       <c r="H19" s="6" t="s">
-        <v>319</v>
+        <v>313</v>
       </c>
       <c r="I19" s="5" t="s">
-        <v>320</v>
+        <v>314</v>
       </c>
       <c r="J19" s="6" t="s">
-        <v>320</v>
+        <v>314</v>
       </c>
     </row>
     <row r="20" spans="1:10">
@@ -7707,31 +7568,31 @@
         <v>1</v>
       </c>
       <c r="B20" s="5" t="s">
-        <v>321</v>
+        <v>315</v>
       </c>
       <c r="C20" s="5" t="s">
-        <v>322</v>
+        <v>316</v>
       </c>
       <c r="D20" s="6" t="s">
-        <v>321</v>
+        <v>315</v>
       </c>
       <c r="E20" s="6" t="s">
-        <v>321</v>
+        <v>315</v>
       </c>
       <c r="F20" s="5" t="s">
-        <v>323</v>
+        <v>317</v>
       </c>
       <c r="G20" s="11" t="s">
-        <v>323</v>
+        <v>317</v>
       </c>
       <c r="H20" s="6" t="s">
-        <v>322</v>
+        <v>316</v>
       </c>
       <c r="I20" s="5" t="s">
-        <v>324</v>
+        <v>318</v>
       </c>
       <c r="J20" s="6" t="s">
-        <v>325</v>
+        <v>319</v>
       </c>
     </row>
     <row r="21" spans="1:10">
@@ -7739,31 +7600,31 @@
         <v>2</v>
       </c>
       <c r="B21" s="5" t="s">
-        <v>326</v>
+        <v>320</v>
       </c>
       <c r="C21" s="5" t="s">
-        <v>327</v>
+        <v>321</v>
       </c>
       <c r="D21" s="6" t="s">
-        <v>326</v>
+        <v>320</v>
       </c>
       <c r="E21" s="6" t="s">
-        <v>326</v>
+        <v>320</v>
       </c>
       <c r="F21" s="5" t="s">
-        <v>326</v>
+        <v>320</v>
       </c>
       <c r="G21" s="11" t="s">
-        <v>328</v>
+        <v>322</v>
       </c>
       <c r="H21" s="6" t="s">
-        <v>327</v>
+        <v>321</v>
       </c>
       <c r="I21" s="5" t="s">
-        <v>329</v>
+        <v>323</v>
       </c>
       <c r="J21" s="6" t="s">
-        <v>329</v>
+        <v>323</v>
       </c>
     </row>
     <row r="22" spans="1:10">
@@ -7771,31 +7632,31 @@
         <v>3</v>
       </c>
       <c r="B22" s="5" t="s">
-        <v>330</v>
+        <v>324</v>
       </c>
       <c r="C22" s="5" t="s">
-        <v>331</v>
+        <v>325</v>
       </c>
       <c r="D22" s="6" t="s">
-        <v>330</v>
+        <v>324</v>
       </c>
       <c r="E22" s="6" t="s">
-        <v>330</v>
+        <v>324</v>
       </c>
       <c r="F22" s="5" t="s">
-        <v>330</v>
+        <v>324</v>
       </c>
       <c r="G22" s="11" t="s">
-        <v>332</v>
+        <v>326</v>
       </c>
       <c r="H22" s="6" t="s">
-        <v>331</v>
+        <v>325</v>
       </c>
       <c r="I22" s="5" t="s">
-        <v>333</v>
+        <v>327</v>
       </c>
       <c r="J22" s="6" t="s">
-        <v>334</v>
+        <v>328</v>
       </c>
     </row>
     <row r="23" spans="1:10">
@@ -7803,31 +7664,31 @@
         <v>4</v>
       </c>
       <c r="B23" s="5" t="s">
-        <v>335</v>
+        <v>329</v>
       </c>
       <c r="C23" s="5" t="s">
-        <v>336</v>
+        <v>330</v>
       </c>
       <c r="D23" s="6" t="s">
-        <v>335</v>
+        <v>329</v>
       </c>
       <c r="E23" s="6" t="s">
-        <v>335</v>
+        <v>329</v>
       </c>
       <c r="F23" s="5" t="s">
-        <v>337</v>
+        <v>331</v>
       </c>
       <c r="G23" s="11" t="s">
-        <v>338</v>
+        <v>332</v>
       </c>
       <c r="H23" s="6" t="s">
-        <v>339</v>
+        <v>333</v>
       </c>
       <c r="I23" s="5" t="s">
-        <v>340</v>
+        <v>334</v>
       </c>
       <c r="J23" s="6" t="s">
-        <v>228</v>
+        <v>222</v>
       </c>
     </row>
     <row r="24" spans="1:10">
@@ -7835,31 +7696,31 @@
         <v>5</v>
       </c>
       <c r="B24" s="13" t="s">
-        <v>230</v>
+        <v>224</v>
       </c>
       <c r="C24" s="13" t="s">
-        <v>341</v>
+        <v>335</v>
       </c>
       <c r="D24" s="14" t="s">
-        <v>230</v>
+        <v>224</v>
       </c>
       <c r="E24" s="14" t="s">
-        <v>230</v>
+        <v>224</v>
       </c>
       <c r="F24" s="13" t="s">
-        <v>342</v>
+        <v>336</v>
       </c>
       <c r="G24" s="15" t="s">
-        <v>343</v>
+        <v>337</v>
       </c>
       <c r="H24" s="14" t="s">
-        <v>341</v>
+        <v>335</v>
       </c>
       <c r="I24" s="13" t="s">
-        <v>344</v>
+        <v>338</v>
       </c>
       <c r="J24" s="14" t="s">
-        <v>345</v>
+        <v>339</v>
       </c>
     </row>
     <row r="25" spans="1:10">
@@ -7867,31 +7728,31 @@
         <v>6</v>
       </c>
       <c r="B25" s="5" t="s">
-        <v>234</v>
+        <v>228</v>
       </c>
       <c r="C25" s="5" t="s">
-        <v>346</v>
+        <v>340</v>
       </c>
       <c r="D25" s="6" t="s">
-        <v>234</v>
+        <v>228</v>
       </c>
       <c r="E25" s="6" t="s">
-        <v>347</v>
+        <v>341</v>
       </c>
       <c r="F25" s="5" t="s">
-        <v>348</v>
+        <v>342</v>
       </c>
       <c r="G25" s="11" t="s">
-        <v>349</v>
+        <v>343</v>
       </c>
       <c r="H25" s="6" t="s">
-        <v>346</v>
+        <v>340</v>
       </c>
       <c r="I25" s="5" t="s">
-        <v>350</v>
+        <v>344</v>
       </c>
       <c r="J25" s="6" t="s">
-        <v>351</v>
+        <v>345</v>
       </c>
     </row>
     <row r="26" spans="1:10">
@@ -7899,31 +7760,31 @@
         <v>7</v>
       </c>
       <c r="B26" s="5" t="s">
-        <v>237</v>
+        <v>231</v>
       </c>
       <c r="C26" s="5" t="s">
+        <v>346</v>
+      </c>
+      <c r="D26" s="6" t="s">
+        <v>231</v>
+      </c>
+      <c r="E26" s="6" t="s">
+        <v>347</v>
+      </c>
+      <c r="F26" s="5" t="s">
+        <v>348</v>
+      </c>
+      <c r="G26" s="11" t="s">
+        <v>349</v>
+      </c>
+      <c r="H26" s="6" t="s">
+        <v>350</v>
+      </c>
+      <c r="I26" s="5" t="s">
+        <v>351</v>
+      </c>
+      <c r="J26" s="6" t="s">
         <v>352</v>
-      </c>
-      <c r="D26" s="6" t="s">
-        <v>237</v>
-      </c>
-      <c r="E26" s="6" t="s">
-        <v>353</v>
-      </c>
-      <c r="F26" s="5" t="s">
-        <v>354</v>
-      </c>
-      <c r="G26" s="11" t="s">
-        <v>355</v>
-      </c>
-      <c r="H26" s="6" t="s">
-        <v>356</v>
-      </c>
-      <c r="I26" s="5" t="s">
-        <v>357</v>
-      </c>
-      <c r="J26" s="6" t="s">
-        <v>358</v>
       </c>
     </row>
     <row r="27" spans="1:10">
@@ -7931,31 +7792,31 @@
         <v>8</v>
       </c>
       <c r="B27" s="5" t="s">
-        <v>242</v>
+        <v>236</v>
       </c>
       <c r="C27" s="5" t="s">
+        <v>353</v>
+      </c>
+      <c r="D27" s="6" t="s">
+        <v>354</v>
+      </c>
+      <c r="E27" s="6" t="s">
+        <v>355</v>
+      </c>
+      <c r="F27" s="5" t="s">
+        <v>356</v>
+      </c>
+      <c r="G27" s="11" t="s">
+        <v>357</v>
+      </c>
+      <c r="H27" s="6" t="s">
+        <v>358</v>
+      </c>
+      <c r="I27" s="5" t="s">
         <v>359</v>
       </c>
-      <c r="D27" s="6" t="s">
+      <c r="J27" s="6" t="s">
         <v>360</v>
-      </c>
-      <c r="E27" s="6" t="s">
-        <v>361</v>
-      </c>
-      <c r="F27" s="5" t="s">
-        <v>362</v>
-      </c>
-      <c r="G27" s="11" t="s">
-        <v>363</v>
-      </c>
-      <c r="H27" s="6" t="s">
-        <v>364</v>
-      </c>
-      <c r="I27" s="5" t="s">
-        <v>365</v>
-      </c>
-      <c r="J27" s="6" t="s">
-        <v>366</v>
       </c>
     </row>
     <row r="28" spans="1:10">
@@ -7963,31 +7824,31 @@
         <v>9</v>
       </c>
       <c r="B28" s="5" t="s">
-        <v>249</v>
+        <v>243</v>
       </c>
       <c r="C28" s="5" t="s">
+        <v>361</v>
+      </c>
+      <c r="D28" s="6" t="s">
+        <v>242</v>
+      </c>
+      <c r="E28" s="6" t="s">
+        <v>362</v>
+      </c>
+      <c r="F28" s="5" t="s">
+        <v>363</v>
+      </c>
+      <c r="G28" s="11" t="s">
+        <v>364</v>
+      </c>
+      <c r="H28" s="6" t="s">
+        <v>365</v>
+      </c>
+      <c r="I28" s="5" t="s">
+        <v>366</v>
+      </c>
+      <c r="J28" s="6" t="s">
         <v>367</v>
-      </c>
-      <c r="D28" s="6" t="s">
-        <v>248</v>
-      </c>
-      <c r="E28" s="6" t="s">
-        <v>368</v>
-      </c>
-      <c r="F28" s="5" t="s">
-        <v>369</v>
-      </c>
-      <c r="G28" s="11" t="s">
-        <v>370</v>
-      </c>
-      <c r="H28" s="6" t="s">
-        <v>371</v>
-      </c>
-      <c r="I28" s="5" t="s">
-        <v>372</v>
-      </c>
-      <c r="J28" s="6" t="s">
-        <v>373</v>
       </c>
     </row>
     <row r="29" spans="1:10">
@@ -7995,31 +7856,31 @@
         <v>10</v>
       </c>
       <c r="B29" s="5" t="s">
+        <v>368</v>
+      </c>
+      <c r="C29" s="5" t="s">
+        <v>369</v>
+      </c>
+      <c r="D29" s="6" t="s">
+        <v>249</v>
+      </c>
+      <c r="E29" s="6" t="s">
+        <v>370</v>
+      </c>
+      <c r="F29" s="5" t="s">
+        <v>371</v>
+      </c>
+      <c r="G29" s="11" t="s">
+        <v>372</v>
+      </c>
+      <c r="H29" s="6" t="s">
+        <v>373</v>
+      </c>
+      <c r="I29" s="5" t="s">
         <v>374</v>
       </c>
-      <c r="C29" s="5" t="s">
+      <c r="J29" s="6" t="s">
         <v>375</v>
-      </c>
-      <c r="D29" s="6" t="s">
-        <v>255</v>
-      </c>
-      <c r="E29" s="6" t="s">
-        <v>376</v>
-      </c>
-      <c r="F29" s="5" t="s">
-        <v>377</v>
-      </c>
-      <c r="G29" s="11" t="s">
-        <v>378</v>
-      </c>
-      <c r="H29" s="6" t="s">
-        <v>379</v>
-      </c>
-      <c r="I29" s="5" t="s">
-        <v>380</v>
-      </c>
-      <c r="J29" s="6" t="s">
-        <v>381</v>
       </c>
     </row>
     <row r="30" spans="1:10">
@@ -8027,31 +7888,31 @@
         <v>11</v>
       </c>
       <c r="B30" s="5" t="s">
+        <v>376</v>
+      </c>
+      <c r="C30" s="5" t="s">
+        <v>377</v>
+      </c>
+      <c r="D30" s="6" t="s">
+        <v>378</v>
+      </c>
+      <c r="E30" s="6" t="s">
+        <v>379</v>
+      </c>
+      <c r="F30" s="5" t="s">
+        <v>380</v>
+      </c>
+      <c r="G30" s="11" t="s">
+        <v>381</v>
+      </c>
+      <c r="H30" s="6" t="s">
         <v>382</v>
       </c>
-      <c r="C30" s="5" t="s">
+      <c r="I30" s="5" t="s">
         <v>383</v>
       </c>
-      <c r="D30" s="6" t="s">
+      <c r="J30" s="6" t="s">
         <v>384</v>
-      </c>
-      <c r="E30" s="6" t="s">
-        <v>385</v>
-      </c>
-      <c r="F30" s="5" t="s">
-        <v>386</v>
-      </c>
-      <c r="G30" s="11" t="s">
-        <v>387</v>
-      </c>
-      <c r="H30" s="6" t="s">
-        <v>388</v>
-      </c>
-      <c r="I30" s="5" t="s">
-        <v>389</v>
-      </c>
-      <c r="J30" s="6" t="s">
-        <v>390</v>
       </c>
     </row>
     <row r="31" spans="1:10">
@@ -8059,63 +7920,63 @@
         <v>12</v>
       </c>
       <c r="B31" s="5" t="s">
-        <v>272</v>
+        <v>266</v>
       </c>
       <c r="C31" s="5" t="s">
+        <v>385</v>
+      </c>
+      <c r="D31" s="6" t="s">
+        <v>386</v>
+      </c>
+      <c r="E31" s="6" t="s">
+        <v>387</v>
+      </c>
+      <c r="F31" s="5" t="s">
+        <v>388</v>
+      </c>
+      <c r="G31" s="11" t="s">
+        <v>389</v>
+      </c>
+      <c r="H31" s="6" t="s">
+        <v>390</v>
+      </c>
+      <c r="I31" s="5" t="s">
         <v>391</v>
       </c>
-      <c r="D31" s="6" t="s">
+      <c r="J31" s="6" t="s">
         <v>392</v>
-      </c>
-      <c r="E31" s="6" t="s">
-        <v>393</v>
-      </c>
-      <c r="F31" s="5" t="s">
-        <v>394</v>
-      </c>
-      <c r="G31" s="11" t="s">
-        <v>395</v>
-      </c>
-      <c r="H31" s="6" t="s">
-        <v>396</v>
-      </c>
-      <c r="I31" s="5" t="s">
-        <v>397</v>
-      </c>
-      <c r="J31" s="6" t="s">
-        <v>398</v>
       </c>
     </row>
     <row r="32" spans="1:10">
       <c r="A32" s="8" t="s">
+        <v>393</v>
+      </c>
+      <c r="B32" s="8" t="s">
+        <v>394</v>
+      </c>
+      <c r="C32" s="3" t="s">
+        <v>395</v>
+      </c>
+      <c r="D32" s="8" t="s">
+        <v>396</v>
+      </c>
+      <c r="E32" s="8" t="s">
+        <v>397</v>
+      </c>
+      <c r="F32" s="8" t="s">
+        <v>398</v>
+      </c>
+      <c r="G32" s="8" t="s">
+        <v>308</v>
+      </c>
+      <c r="H32" s="8" t="s">
+        <v>309</v>
+      </c>
+      <c r="I32" s="8" t="s">
         <v>399</v>
       </c>
-      <c r="B32" s="8" t="s">
+      <c r="J32" s="8" t="s">
         <v>400</v>
-      </c>
-      <c r="C32" s="3" t="s">
-        <v>401</v>
-      </c>
-      <c r="D32" s="8" t="s">
-        <v>402</v>
-      </c>
-      <c r="E32" s="8" t="s">
-        <v>403</v>
-      </c>
-      <c r="F32" s="8" t="s">
-        <v>404</v>
-      </c>
-      <c r="G32" s="8" t="s">
-        <v>314</v>
-      </c>
-      <c r="H32" s="8" t="s">
-        <v>315</v>
-      </c>
-      <c r="I32" s="8" t="s">
-        <v>405</v>
-      </c>
-      <c r="J32" s="8" t="s">
-        <v>406</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Made some new calculations for epic monsters and based on their action points (degree). It's a mess but it seems the calculations are fine. THe final number in the monster stat block is not working.
</commit_message>
<xml_diff>
--- a/Design/Tables.xlsx
+++ b/Design/Tables.xlsx
@@ -1,10 +1,10 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:dbsheet="http://web.wps.cn/et/2021/dbsheet">
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="27945" windowHeight="11730" activeTab="1"/>
+    <workbookView windowWidth="28800" windowHeight="12300" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -2855,11 +2855,11 @@
     <xf numFmtId="0" fontId="16" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -2965,7 +2965,7 @@
     <cellStyle name="Percent" xfId="3" builtinId="5"/>
     <cellStyle name="Comma [0]" xfId="4" builtinId="6"/>
     <cellStyle name="Currency [0]" xfId="5" builtinId="7"/>
-    <cellStyle name="Hyperlink" xfId="6" builtinId="8"/>
+    <cellStyle name="Link" xfId="6" builtinId="8"/>
     <cellStyle name="Followed Hyperlink" xfId="7" builtinId="9"/>
     <cellStyle name="Note" xfId="8" builtinId="10"/>
     <cellStyle name="Warning Text" xfId="9" builtinId="11"/>
@@ -5554,9 +5554,12 @@
         <v>-2</v>
       </c>
       <c r="G19">
-        <v>12</v>
-      </c>
-      <c r="H19" s="58"/>
+        <v>15.5</v>
+      </c>
+      <c r="H19" s="58">
+        <f>5.5*3</f>
+        <v>16.5</v>
+      </c>
       <c r="K19" s="70">
         <v>5</v>
       </c>
@@ -5578,7 +5581,6 @@
         <v>-1</v>
       </c>
       <c r="H20" s="57"/>
-      <c r="I20"/>
       <c r="J20" s="73"/>
       <c r="K20" s="70">
         <v>6</v>
@@ -6042,9 +6044,7 @@
       <c r="K44" s="58"/>
     </row>
     <row r="45" ht="15.75" spans="1:11">
-      <c r="A45" s="72" t="s">
-        <v>102</v>
-      </c>
+      <c r="A45" s="72"/>
       <c r="B45" s="39">
         <v>150</v>
       </c>
@@ -6070,7 +6070,7 @@
     </row>
     <row r="46" ht="15.75" spans="1:11">
       <c r="A46" s="72" t="s">
-        <v>106</v>
+        <v>102</v>
       </c>
       <c r="B46" s="39">
         <v>175</v>
@@ -6098,7 +6098,10 @@
       </c>
       <c r="K46" s="58"/>
     </row>
-    <row r="47" ht="15.75" spans="2:11">
+    <row r="47" ht="15.75" spans="1:11">
+      <c r="A47" s="72" t="s">
+        <v>106</v>
+      </c>
       <c r="B47" s="39">
         <v>200</v>
       </c>
@@ -6126,9 +6129,7 @@
       <c r="K47" s="58"/>
     </row>
     <row r="48" ht="15.75" spans="1:11">
-      <c r="A48" s="72" t="s">
-        <v>109</v>
-      </c>
+      <c r="A48" s="72"/>
       <c r="B48" s="52">
         <v>225</v>
       </c>
@@ -6157,7 +6158,7 @@
     </row>
     <row r="49" ht="15.75" spans="1:11">
       <c r="A49" s="72" t="s">
-        <v>113</v>
+        <v>109</v>
       </c>
       <c r="B49" s="39">
         <v>250</v>
@@ -6185,7 +6186,10 @@
       </c>
       <c r="K49" s="58"/>
     </row>
-    <row r="50" ht="16.5" spans="2:11">
+    <row r="50" ht="16.5" spans="1:11">
+      <c r="A50" s="72" t="s">
+        <v>113</v>
+      </c>
       <c r="B50" s="39">
         <v>275</v>
       </c>
@@ -6213,10 +6217,8 @@
       <c r="K50" s="58"/>
     </row>
     <row r="51" ht="16.5" spans="1:13">
-      <c r="A51" s="94" t="s">
-        <v>115</v>
-      </c>
-      <c r="B51" s="95">
+      <c r="A51" s="72"/>
+      <c r="B51" s="94">
         <v>300</v>
       </c>
       <c r="C51" s="40">
@@ -6239,10 +6241,10 @@
       <c r="M51" s="58"/>
     </row>
     <row r="52" ht="16.5" spans="1:13">
-      <c r="A52" s="94" t="s">
-        <v>117</v>
-      </c>
-      <c r="B52" s="95">
+      <c r="A52" s="95" t="s">
+        <v>115</v>
+      </c>
+      <c r="B52" s="94">
         <v>325</v>
       </c>
       <c r="C52" s="40">
@@ -6269,8 +6271,8 @@
       <c r="M52" s="58"/>
     </row>
     <row r="53" ht="15.75" spans="1:13">
-      <c r="A53" s="72" t="s">
-        <v>120</v>
+      <c r="A53" s="95" t="s">
+        <v>117</v>
       </c>
       <c r="B53" s="39">
         <v>350</v>
@@ -6300,9 +6302,7 @@
       <c r="M53" s="58"/>
     </row>
     <row r="54" ht="16.5" spans="1:10">
-      <c r="A54" s="72" t="s">
-        <v>123</v>
-      </c>
+      <c r="A54" s="95"/>
       <c r="B54" s="65">
         <v>375</v>
       </c>
@@ -6329,7 +6329,10 @@
         <v>32</v>
       </c>
     </row>
-    <row r="55" spans="2:10">
+    <row r="55" ht="15.75" spans="1:10">
+      <c r="A55" s="72" t="s">
+        <v>120</v>
+      </c>
       <c r="B55" s="39">
         <v>400</v>
       </c>
@@ -6356,7 +6359,8 @@
         <v>31</v>
       </c>
     </row>
-    <row r="56" spans="2:10">
+    <row r="56" ht="15.75" spans="1:10">
+      <c r="A56" s="72"/>
       <c r="B56" s="39">
         <v>425</v>
       </c>
@@ -6383,7 +6387,10 @@
         <v>32</v>
       </c>
     </row>
-    <row r="57" spans="2:10">
+    <row r="57" ht="15.75" spans="1:10">
+      <c r="A57" s="72" t="s">
+        <v>123</v>
+      </c>
       <c r="B57" s="39">
         <v>450</v>
       </c>
@@ -6410,7 +6417,8 @@
         <v>32</v>
       </c>
     </row>
-    <row r="58" spans="2:10">
+    <row r="58" ht="15.75" spans="1:10">
+      <c r="A58" s="72"/>
       <c r="B58" s="39">
         <v>475</v>
       </c>
@@ -6444,7 +6452,7 @@
       <c r="C59" s="40">
         <v>105</v>
       </c>
-      <c r="D59" s="95" t="s">
+      <c r="D59" s="94" t="s">
         <v>136</v>
       </c>
       <c r="E59" s="41">
@@ -6464,12 +6472,13 @@
         <v>32</v>
       </c>
     </row>
-    <row r="60" ht="15.75" spans="2:10">
+    <row r="60" ht="15.75" spans="1:10">
+      <c r="A60" s="72"/>
       <c r="B60" s="52">
         <v>600</v>
       </c>
-      <c r="C60" s="95"/>
-      <c r="D60" s="95">
+      <c r="C60" s="94"/>
+      <c r="D60" s="94">
         <v>14.5</v>
       </c>
       <c r="E60" s="41">
@@ -6493,8 +6502,8 @@
       <c r="B61" s="52">
         <v>750</v>
       </c>
-      <c r="C61" s="95"/>
-      <c r="D61" s="95">
+      <c r="C61" s="94"/>
+      <c r="D61" s="94">
         <v>15</v>
       </c>
       <c r="E61" s="41">

</xml_diff>

<commit_message>
Made some more polish
</commit_message>
<xml_diff>
--- a/Design/Tables.xlsx
+++ b/Design/Tables.xlsx
@@ -1,10 +1,10 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:dbsheet="http://web.wps.cn/et/2021/dbsheet">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="28800" windowHeight="12300" activeTab="1"/>
+    <workbookView windowWidth="27945" windowHeight="11730" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -2965,7 +2965,7 @@
     <cellStyle name="Percent" xfId="3" builtinId="5"/>
     <cellStyle name="Comma [0]" xfId="4" builtinId="6"/>
     <cellStyle name="Currency [0]" xfId="5" builtinId="7"/>
-    <cellStyle name="Link" xfId="6" builtinId="8"/>
+    <cellStyle name="Hyperlink" xfId="6" builtinId="8"/>
     <cellStyle name="Followed Hyperlink" xfId="7" builtinId="9"/>
     <cellStyle name="Note" xfId="8" builtinId="10"/>
     <cellStyle name="Warning Text" xfId="9" builtinId="11"/>
@@ -5474,7 +5474,7 @@
       <c r="E15" s="40"/>
       <c r="F15" s="40"/>
     </row>
-    <row r="16" ht="15.75" spans="1:11">
+    <row r="16" ht="15.75" spans="1:8">
       <c r="A16" s="48" t="s">
         <v>34</v>
       </c>
@@ -5491,11 +5491,8 @@
         <v>40</v>
       </c>
       <c r="H16" s="40"/>
-      <c r="K16">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="17" ht="15.75" spans="1:11">
+    </row>
+    <row r="17" ht="15.75" spans="1:8">
       <c r="A17" s="52">
         <v>0</v>
       </c>
@@ -5512,9 +5509,6 @@
         <v>0</v>
       </c>
       <c r="H17" s="40"/>
-      <c r="K17">
-        <v>6</v>
-      </c>
     </row>
     <row r="18" ht="15.75" spans="1:11">
       <c r="A18" s="52">
@@ -5533,9 +5527,7 @@
         <v>-1</v>
       </c>
       <c r="H18" s="57"/>
-      <c r="K18" s="70">
-        <v>4</v>
-      </c>
+      <c r="K18" s="70"/>
     </row>
     <row r="19" ht="15.75" spans="1:11">
       <c r="A19" s="52">
@@ -5553,16 +5545,8 @@
       <c r="E19" s="55">
         <v>-2</v>
       </c>
-      <c r="G19">
-        <v>15.5</v>
-      </c>
-      <c r="H19" s="58">
-        <f>5.5*3</f>
-        <v>16.5</v>
-      </c>
-      <c r="K19" s="70">
-        <v>5</v>
-      </c>
+      <c r="H19" s="58"/>
+      <c r="K19" s="70"/>
     </row>
     <row r="20" ht="15.75" spans="1:11">
       <c r="A20" s="59">
@@ -5582,9 +5566,7 @@
       </c>
       <c r="H20" s="57"/>
       <c r="J20" s="73"/>
-      <c r="K20" s="70">
-        <v>6</v>
-      </c>
+      <c r="K20" s="70"/>
     </row>
     <row r="21" ht="15.75" spans="1:11">
       <c r="A21" s="52">
@@ -5603,9 +5585,7 @@
         <v>-2</v>
       </c>
       <c r="H21" s="58"/>
-      <c r="K21" s="70">
-        <v>4</v>
-      </c>
+      <c r="K21" s="70"/>
     </row>
     <row r="22" ht="16.5" spans="1:11">
       <c r="A22" s="65">
@@ -5624,9 +5604,7 @@
         <v>-3</v>
       </c>
       <c r="H22" s="58"/>
-      <c r="K22" s="70">
-        <v>5</v>
-      </c>
+      <c r="K22" s="70"/>
     </row>
     <row r="23" ht="15.75" spans="1:11">
       <c r="A23" s="67">
@@ -5648,9 +5626,7 @@
       <c r="H23" s="70"/>
       <c r="I23" s="70"/>
       <c r="J23" s="70"/>
-      <c r="K23" s="70">
-        <v>5</v>
-      </c>
+      <c r="K23" s="70"/>
     </row>
     <row r="24" ht="16.5" spans="1:11">
       <c r="A24" s="65">
@@ -5672,9 +5648,7 @@
       <c r="H24" s="70"/>
       <c r="I24" s="70"/>
       <c r="J24" s="70"/>
-      <c r="K24" s="70">
-        <v>6</v>
-      </c>
+      <c r="K24" s="70"/>
     </row>
     <row r="25" ht="16.5" spans="1:11">
       <c r="A25" s="72"/>
@@ -5687,12 +5661,9 @@
       <c r="H25" s="40"/>
       <c r="I25" s="70"/>
       <c r="J25" s="70"/>
-      <c r="K25" s="99">
-        <f>46/9</f>
-        <v>5.11111111111111</v>
-      </c>
-    </row>
-    <row r="26" ht="15.75" spans="1:11">
+      <c r="K25" s="99"/>
+    </row>
+    <row r="26" spans="1:11">
       <c r="A26" s="74"/>
       <c r="B26" s="51"/>
       <c r="C26" s="75" t="s">
@@ -5802,7 +5773,7 @@
       <c r="E32" s="40"/>
       <c r="F32" s="41"/>
     </row>
-    <row r="33" ht="15.75" spans="1:6">
+    <row r="33" spans="1:6">
       <c r="A33" s="44">
         <v>1</v>
       </c>
@@ -5872,7 +5843,7 @@
       <c r="J37" s="40"/>
       <c r="K37" s="58"/>
     </row>
-    <row r="38" ht="16.5" spans="1:12">
+    <row r="38" ht="16.5" spans="1:11">
       <c r="A38" s="58"/>
       <c r="C38" s="67" t="s">
         <v>82</v>
@@ -5883,14 +5854,7 @@
       <c r="H38" s="72"/>
       <c r="I38" s="58"/>
       <c r="J38" s="40"/>
-      <c r="K38" s="58">
-        <f>550+225</f>
-        <v>775</v>
-      </c>
-      <c r="L38">
-        <f>150*5+200</f>
-        <v>950</v>
-      </c>
+      <c r="K38" s="58"/>
     </row>
     <row r="39" ht="16.5" spans="1:11">
       <c r="A39" s="72"/>

</xml_diff>

<commit_message>
Worked on book creator.
</commit_message>
<xml_diff>
--- a/Design/Tables.xlsx
+++ b/Design/Tables.xlsx
@@ -4,10 +4,11 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="28800" windowHeight="12300"/>
+    <workbookView windowWidth="27630" windowHeight="12900" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="Standard" sheetId="3" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="4" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -27,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="146" uniqueCount="123">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="233" uniqueCount="144">
   <si>
     <t>1-Handed (base) (5.5 base + 3 stat = 8.5) (8.5 - 4 AC)*2 hands = 9</t>
   </si>
@@ -554,6 +555,69 @@
   <si>
     <t>Hard</t>
   </si>
+  <si>
+    <t>Cleric</t>
+  </si>
+  <si>
+    <t>Druid</t>
+  </si>
+  <si>
+    <t>Hunter</t>
+  </si>
+  <si>
+    <t>Rogue</t>
+  </si>
+  <si>
+    <t>Warlock</t>
+  </si>
+  <si>
+    <t>Warrior</t>
+  </si>
+  <si>
+    <t>Wizard</t>
+  </si>
+  <si>
+    <t>Artificer</t>
+  </si>
+  <si>
+    <t>Knight</t>
+  </si>
+  <si>
+    <t>Sorcerer</t>
+  </si>
+  <si>
+    <t>Swashbuckler</t>
+  </si>
+  <si>
+    <t>Minor</t>
+  </si>
+  <si>
+    <t>Spec (Minor)</t>
+  </si>
+  <si>
+    <t>Spec (Keystone)</t>
+  </si>
+  <si>
+    <t>Keystone</t>
+  </si>
+  <si>
+    <t>Other</t>
+  </si>
+  <si>
+    <t>Upgrade</t>
+  </si>
+  <si>
+    <t>Util</t>
+  </si>
+  <si>
+    <t>Other     ]</t>
+  </si>
+  <si>
+    <t>[     Other</t>
+  </si>
+  <si>
+    <t>Ult</t>
+  </si>
 </sst>
 </file>
 
@@ -565,7 +629,7 @@
     <numFmt numFmtId="176" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
     <numFmt numFmtId="177" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
   </numFmts>
-  <fonts count="36">
+  <fonts count="41">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -575,8 +639,53 @@
     </font>
     <font>
       <b/>
+      <sz val="14"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="14"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="13"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="13"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="13"/>
+      <color theme="4" tint="-0.25"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="12"/>
       <color theme="9" tint="-0.249977111117893"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color theme="1"/>
       <name val="Calibri"/>
       <charset val="134"/>
       <scheme val="minor"/>
@@ -622,13 +731,6 @@
       <b/>
       <sz val="12"/>
       <color rgb="FF00B0F0"/>
-      <name val="Calibri"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="12"/>
-      <color theme="1"/>
       <name val="Calibri"/>
       <charset val="134"/>
       <scheme val="minor"/>
@@ -1045,6 +1147,43 @@
       <diagonal/>
     </border>
     <border>
+      <left/>
+      <right/>
+      <top style="medium">
+        <color auto="1"/>
+      </top>
+      <bottom style="medium">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color auto="1"/>
+      </left>
+      <right style="medium">
+        <color auto="1"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color auto="1"/>
+      </left>
+      <right style="medium">
+        <color auto="1"/>
+      </right>
+      <top style="medium">
+        <color auto="1"/>
+      </top>
+      <bottom style="medium">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
       <left style="medium">
         <color auto="1"/>
       </left>
@@ -1079,17 +1218,6 @@
       <left style="medium">
         <color auto="1"/>
       </left>
-      <right/>
-      <top style="medium">
-        <color auto="1"/>
-      </top>
-      <bottom style="medium">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
       <right/>
       <top style="medium">
         <color auto="1"/>
@@ -1182,32 +1310,6 @@
         <color auto="1"/>
       </right>
       <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="medium">
-        <color auto="1"/>
-      </left>
-      <right style="medium">
-        <color auto="1"/>
-      </right>
-      <top/>
-      <bottom style="medium">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="medium">
-        <color auto="1"/>
-      </left>
-      <right style="medium">
-        <color auto="1"/>
-      </right>
-      <top style="medium">
-        <color auto="1"/>
-      </top>
       <bottom style="medium">
         <color auto="1"/>
       </bottom>
@@ -1331,137 +1433,137 @@
     <xf numFmtId="42" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="16" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="17" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="17" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="18" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="23" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="4" borderId="19" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="5" borderId="20" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="5" borderId="19" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="6" borderId="21" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="0" borderId="22" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="0" borderId="23" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="30" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="31" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="32" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="33" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="34" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="34" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="33" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="33" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="34" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="34" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="33" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="33" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="34" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="34" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="33" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="33" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="34" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="34" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="33" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="33" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="34" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="34" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="33" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="33" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="34" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="34" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="33" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="17" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="17" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="0" borderId="18" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="4" borderId="19" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="5" borderId="20" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="31" fillId="5" borderId="19" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="32" fillId="6" borderId="21" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="33" fillId="0" borderId="22" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="34" fillId="0" borderId="23" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="35" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="36" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="37" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="38" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="39" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="39" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="38" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="38" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="39" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="39" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="38" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="38" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="39" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="39" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="38" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="38" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="39" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="39" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="38" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="38" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="39" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="39" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="38" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="38" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="39" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="39" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="38" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="98">
+  <cellXfs count="108">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -1471,262 +1573,292 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="16" fontId="0" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="16" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="13" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -1735,37 +1867,37 @@
     <xf numFmtId="16" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="16" fontId="0" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1" quotePrefix="1">
+    <xf numFmtId="16" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1" quotePrefix="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1" quotePrefix="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1" applyAlignment="1" quotePrefix="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1" quotePrefix="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1" applyAlignment="1" quotePrefix="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1" quotePrefix="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -1781,7 +1913,7 @@
     <cellStyle name="Note" xfId="8" builtinId="10"/>
     <cellStyle name="Warning Text" xfId="9" builtinId="11"/>
     <cellStyle name="Title" xfId="10" builtinId="15"/>
-    <cellStyle name="CExplanatory Text" xfId="11" builtinId="53"/>
+    <cellStyle name="Explanatory Text" xfId="11" builtinId="53"/>
     <cellStyle name="Heading 1" xfId="12" builtinId="16"/>
     <cellStyle name="Heading 2" xfId="13" builtinId="17"/>
     <cellStyle name="Heading 3" xfId="14" builtinId="18"/>
@@ -2117,229 +2249,229 @@
   </cols>
   <sheetData>
     <row r="2" ht="15.75"/>
-    <row r="3" ht="16.5" spans="2:14">
-      <c r="B3" s="1" t="s">
+    <row r="3" ht="16.5" spans="1:14">
+      <c r="B3" s="11" t="s">
         <v>0</v>
       </c>
-      <c r="C3" s="2"/>
-      <c r="D3" s="3"/>
-      <c r="E3" s="4" t="s">
+      <c r="C3" s="12"/>
+      <c r="D3" s="13"/>
+      <c r="E3" s="14" t="s">
         <v>1</v>
       </c>
-      <c r="F3" s="5"/>
-      <c r="G3" s="6"/>
-      <c r="L3" s="53" t="s">
+      <c r="F3" s="15"/>
+      <c r="G3" s="16"/>
+      <c r="L3" s="17" t="s">
         <v>2</v>
       </c>
-      <c r="M3" s="41" t="s">
+      <c r="M3" s="18" t="s">
         <v>3</v>
       </c>
-      <c r="N3" s="53"/>
-    </row>
-    <row r="4" ht="15.75" spans="2:14">
-      <c r="B4" s="7" t="s">
+      <c r="N3" s="17"/>
+    </row>
+    <row r="4" ht="15.75" spans="1:14">
+      <c r="B4" s="19" t="s">
         <v>4</v>
       </c>
-      <c r="C4" s="8" t="s">
+      <c r="C4" s="20" t="s">
         <v>5</v>
       </c>
-      <c r="D4" s="9" t="s">
+      <c r="D4" s="21" t="s">
         <v>6</v>
       </c>
-      <c r="E4" s="8"/>
-      <c r="F4" s="8"/>
-      <c r="G4" s="8"/>
-      <c r="L4" s="53" t="s">
+      <c r="E4" s="20"/>
+      <c r="F4" s="20"/>
+      <c r="G4" s="20"/>
+      <c r="L4" s="17" t="s">
         <v>7</v>
       </c>
-      <c r="M4" s="41" t="s">
+      <c r="M4" s="18" t="s">
         <v>8</v>
       </c>
-      <c r="N4" s="53"/>
-    </row>
-    <row r="5" ht="15.75" spans="2:14">
-      <c r="B5" s="7" t="s">
+      <c r="N4" s="17"/>
+    </row>
+    <row r="5" ht="15.75" spans="1:14">
+      <c r="B5" s="19" t="s">
         <v>9</v>
       </c>
-      <c r="C5" s="8" t="s">
+      <c r="C5" s="20" t="s">
         <v>10</v>
       </c>
-      <c r="D5" s="9" t="s">
+      <c r="D5" s="21" t="s">
         <v>11</v>
       </c>
-      <c r="E5" s="8"/>
-      <c r="F5" s="8"/>
-      <c r="G5" s="8"/>
-      <c r="L5" s="53" t="s">
+      <c r="E5" s="20"/>
+      <c r="F5" s="20"/>
+      <c r="G5" s="20"/>
+      <c r="L5" s="17" t="s">
         <v>12</v>
       </c>
-      <c r="M5" s="41" t="s">
+      <c r="M5" s="18" t="s">
         <v>13</v>
       </c>
-      <c r="N5" s="41"/>
-    </row>
-    <row r="6" ht="16.5" spans="2:14">
-      <c r="B6" s="10" t="s">
+      <c r="N5" s="18"/>
+    </row>
+    <row r="6" ht="16.5" spans="1:14">
+      <c r="B6" s="22" t="s">
         <v>14</v>
       </c>
-      <c r="C6" s="11" t="s">
+      <c r="C6" s="23" t="s">
         <v>15</v>
       </c>
-      <c r="D6" s="12"/>
-      <c r="E6" s="8"/>
-      <c r="F6" s="8"/>
-      <c r="G6" s="8"/>
-      <c r="L6" s="53" t="s">
+      <c r="D6" s="24"/>
+      <c r="E6" s="20"/>
+      <c r="F6" s="20"/>
+      <c r="G6" s="20"/>
+      <c r="L6" s="17" t="s">
         <v>16</v>
       </c>
-      <c r="M6" s="41" t="s">
+      <c r="M6" s="18" t="s">
         <v>17</v>
       </c>
-      <c r="N6" s="41"/>
-    </row>
-    <row r="7" ht="16.5" spans="5:14">
-      <c r="E7" s="8"/>
-      <c r="F7" s="8"/>
-      <c r="G7" s="8"/>
-      <c r="L7" s="81" t="s">
+      <c r="N6" s="18"/>
+    </row>
+    <row r="7" ht="16.5" spans="1:14">
+      <c r="E7" s="20"/>
+      <c r="F7" s="20"/>
+      <c r="G7" s="20"/>
+      <c r="L7" s="25" t="s">
         <v>18</v>
       </c>
-      <c r="M7" s="41" t="s">
+      <c r="M7" s="18" t="s">
         <v>19</v>
       </c>
-      <c r="N7" s="41"/>
-    </row>
-    <row r="8" ht="16.5" spans="3:14">
-      <c r="C8" s="13" t="s">
+      <c r="N7" s="18"/>
+    </row>
+    <row r="8" ht="16.5" spans="1:14">
+      <c r="C8" s="26" t="s">
         <v>20</v>
       </c>
-      <c r="D8" s="14"/>
-      <c r="E8" s="14"/>
-      <c r="F8" s="15"/>
-      <c r="G8" s="16"/>
-      <c r="L8" s="81" t="s">
+      <c r="D8" s="27"/>
+      <c r="E8" s="27"/>
+      <c r="F8" s="28"/>
+      <c r="G8" s="29"/>
+      <c r="L8" s="25" t="s">
         <v>21</v>
       </c>
-      <c r="M8" s="81"/>
-      <c r="N8" s="53"/>
-    </row>
-    <row r="9" spans="1:9">
-      <c r="A9" s="17" t="s">
+      <c r="M8" s="25"/>
+      <c r="N8" s="17"/>
+    </row>
+    <row r="9" spans="1:14">
+      <c r="A9" s="30" t="s">
         <v>22</v>
       </c>
-      <c r="B9" s="18" t="s">
+      <c r="B9" s="31" t="s">
         <v>23</v>
       </c>
-      <c r="C9" s="19" t="s">
+      <c r="C9" s="32" t="s">
         <v>24</v>
       </c>
-      <c r="D9" s="19" t="s">
+      <c r="D9" s="32" t="s">
         <v>25</v>
       </c>
-      <c r="E9" s="20" t="s">
+      <c r="E9" s="33" t="s">
         <v>26</v>
       </c>
-      <c r="F9" s="18" t="s">
+      <c r="F9" s="31" t="s">
         <v>23</v>
       </c>
-      <c r="G9" s="19" t="s">
+      <c r="G9" s="32" t="s">
         <v>24</v>
       </c>
-      <c r="H9" s="19" t="s">
+      <c r="H9" s="32" t="s">
         <v>25</v>
       </c>
-      <c r="I9" s="20" t="s">
+      <c r="I9" s="33" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="10" spans="1:9">
-      <c r="A10" s="98" t="s">
+    <row r="10" spans="1:14">
+      <c r="A10" s="108" t="s">
         <v>28</v>
       </c>
-      <c r="B10" s="22">
+      <c r="B10" s="35">
         <v>5.5</v>
       </c>
-      <c r="C10" s="99" t="s">
+      <c r="C10" s="109" t="s">
         <v>29</v>
       </c>
-      <c r="D10" s="23">
+      <c r="D10" s="36">
         <v>-4</v>
       </c>
-      <c r="E10" s="24">
+      <c r="E10" s="37">
         <v>9</v>
       </c>
-      <c r="F10" s="25">
+      <c r="F10" s="38">
         <v>10.5</v>
       </c>
-      <c r="G10" s="99" t="s">
+      <c r="G10" s="109" t="s">
         <v>29</v>
       </c>
-      <c r="H10" s="23">
+      <c r="H10" s="36">
         <v>-4</v>
       </c>
-      <c r="I10" s="24">
+      <c r="I10" s="37">
         <v>9.5</v>
       </c>
     </row>
-    <row r="11" spans="1:9">
-      <c r="A11" s="98" t="s">
+    <row r="11" spans="1:14">
+      <c r="A11" s="108" t="s">
         <v>30</v>
       </c>
-      <c r="B11" s="22">
+      <c r="B11" s="35">
         <v>5.5</v>
       </c>
-      <c r="C11" s="99" t="s">
+      <c r="C11" s="109" t="s">
         <v>31</v>
       </c>
-      <c r="D11" s="23">
+      <c r="D11" s="36">
         <v>-4</v>
       </c>
-      <c r="E11" s="24">
+      <c r="E11" s="37">
         <v>11</v>
       </c>
-      <c r="F11" s="25">
+      <c r="F11" s="38">
         <v>10.5</v>
       </c>
-      <c r="G11" s="99" t="s">
+      <c r="G11" s="109" t="s">
         <v>31</v>
       </c>
-      <c r="H11" s="23">
+      <c r="H11" s="36">
         <v>-4</v>
       </c>
-      <c r="I11" s="24">
+      <c r="I11" s="37">
         <v>10.5</v>
       </c>
     </row>
-    <row r="12" ht="15.75" spans="1:9">
-      <c r="A12" s="100" t="s">
+    <row r="12" ht="15.75" spans="1:14">
+      <c r="A12" s="110" t="s">
         <v>32</v>
       </c>
-      <c r="B12" s="27">
+      <c r="B12" s="40">
         <v>5.5</v>
       </c>
-      <c r="C12" s="101" t="s">
+      <c r="C12" s="111" t="s">
         <v>33</v>
       </c>
-      <c r="D12" s="28">
+      <c r="D12" s="41">
         <v>-5</v>
       </c>
-      <c r="E12" s="29">
+      <c r="E12" s="42">
         <v>11</v>
       </c>
-      <c r="F12" s="30">
+      <c r="F12" s="43">
         <v>10.5</v>
       </c>
-      <c r="G12" s="101" t="s">
+      <c r="G12" s="111" t="s">
         <v>33</v>
       </c>
-      <c r="H12" s="28">
+      <c r="H12" s="41">
         <v>-5</v>
       </c>
-      <c r="I12" s="29">
+      <c r="I12" s="42">
         <v>11.5</v>
       </c>
     </row>
-    <row r="14" spans="2:4">
+    <row r="14" spans="1:14">
       <c r="B14">
         <v>16.5</v>
       </c>
@@ -2352,1531 +2484,1531 @@
         <v>22.5</v>
       </c>
     </row>
-    <row r="15" ht="15.75" spans="2:6">
-      <c r="B15" s="23"/>
-      <c r="D15" s="23"/>
-      <c r="E15" s="23"/>
-      <c r="F15" s="23"/>
-    </row>
-    <row r="16" ht="15.75" spans="1:8">
-      <c r="A16" s="31" t="s">
+    <row r="15" ht="15.75" spans="1:14">
+      <c r="B15" s="36"/>
+      <c r="D15" s="36"/>
+      <c r="E15" s="36"/>
+      <c r="F15" s="36"/>
+    </row>
+    <row r="16" ht="15.75" spans="1:14">
+      <c r="A16" s="44" t="s">
         <v>34</v>
       </c>
-      <c r="B16" s="32" t="s">
+      <c r="B16" s="45" t="s">
         <v>35</v>
       </c>
-      <c r="C16" s="33" t="s">
+      <c r="C16" s="46" t="s">
         <v>36</v>
       </c>
-      <c r="D16" s="34" t="s">
+      <c r="D16" s="47" t="s">
         <v>37</v>
       </c>
-      <c r="E16" s="33" t="s">
+      <c r="E16" s="46" t="s">
         <v>38</v>
       </c>
-      <c r="H16" s="23"/>
-    </row>
-    <row r="17" ht="15.75" spans="1:8">
-      <c r="A17" s="35">
+      <c r="H16" s="36"/>
+    </row>
+    <row r="17" ht="15.75" spans="1:12">
+      <c r="A17" s="48">
         <v>0</v>
       </c>
-      <c r="B17" s="36">
+      <c r="B17" s="49">
         <v>0</v>
       </c>
-      <c r="C17" s="37">
+      <c r="C17" s="50">
         <v>0</v>
       </c>
-      <c r="D17" s="23">
+      <c r="D17" s="36">
         <v>0</v>
       </c>
-      <c r="E17" s="38">
+      <c r="E17" s="51">
         <v>0</v>
       </c>
-      <c r="H17" s="23"/>
-    </row>
-    <row r="18" ht="15.75" spans="1:11">
-      <c r="A18" s="35">
+      <c r="H17" s="36"/>
+    </row>
+    <row r="18" ht="15.75" spans="1:12">
+      <c r="A18" s="48">
         <v>0.5</v>
       </c>
-      <c r="B18" s="36">
+      <c r="B18" s="49">
         <v>0</v>
       </c>
-      <c r="C18" s="39" t="s">
+      <c r="C18" s="52" t="s">
         <v>39</v>
       </c>
-      <c r="D18" s="23">
+      <c r="D18" s="36">
         <v>0</v>
       </c>
-      <c r="E18" s="38">
+      <c r="E18" s="51">
         <v>-1</v>
       </c>
-      <c r="H18" s="40"/>
-      <c r="K18" s="53"/>
-    </row>
-    <row r="19" ht="15.75" spans="1:11">
-      <c r="A19" s="35">
+      <c r="H18" s="53"/>
+      <c r="K18" s="17"/>
+    </row>
+    <row r="19" ht="15.75" spans="1:12">
+      <c r="A19" s="48">
         <v>1</v>
       </c>
-      <c r="B19" s="36">
+      <c r="B19" s="49">
         <v>0</v>
       </c>
-      <c r="C19" s="39" t="s">
+      <c r="C19" s="52" t="s">
         <v>40</v>
       </c>
-      <c r="D19" s="23">
+      <c r="D19" s="36">
         <v>0</v>
       </c>
-      <c r="E19" s="38">
+      <c r="E19" s="51">
         <v>-2</v>
       </c>
-      <c r="H19" s="41"/>
-      <c r="K19" s="53"/>
-    </row>
-    <row r="20" ht="15.75" spans="1:11">
-      <c r="A20" s="42">
+      <c r="H19" s="18"/>
+      <c r="K19" s="17"/>
+    </row>
+    <row r="20" ht="15.75" spans="1:12">
+      <c r="A20" s="54">
         <v>0</v>
       </c>
-      <c r="B20" s="43">
+      <c r="B20" s="55">
         <v>1</v>
       </c>
-      <c r="C20" s="44" t="s">
+      <c r="C20" s="56" t="s">
         <v>41</v>
       </c>
-      <c r="D20" s="45" t="s">
+      <c r="D20" s="57" t="s">
         <v>42</v>
       </c>
-      <c r="E20" s="46">
+      <c r="E20" s="58">
         <v>-1</v>
       </c>
-      <c r="H20" s="40"/>
-      <c r="J20" s="56"/>
-      <c r="K20" s="53"/>
-    </row>
-    <row r="21" ht="15.75" spans="1:11">
-      <c r="A21" s="35">
+      <c r="H20" s="53"/>
+      <c r="J20" s="59"/>
+      <c r="K20" s="17"/>
+    </row>
+    <row r="21" ht="15.75" spans="1:12">
+      <c r="A21" s="48">
         <v>0.5</v>
       </c>
-      <c r="B21" s="36">
+      <c r="B21" s="49">
         <v>1</v>
       </c>
-      <c r="C21" s="39" t="s">
+      <c r="C21" s="52" t="s">
         <v>43</v>
       </c>
-      <c r="D21" s="47" t="s">
+      <c r="D21" s="60" t="s">
         <v>44</v>
       </c>
-      <c r="E21" s="38">
+      <c r="E21" s="51">
         <v>-2</v>
       </c>
-      <c r="H21" s="41"/>
-      <c r="K21" s="53"/>
-    </row>
-    <row r="22" ht="16.5" spans="1:11">
-      <c r="A22" s="48">
+      <c r="H21" s="18"/>
+      <c r="K21" s="17"/>
+    </row>
+    <row r="22" ht="16.5" spans="1:12">
+      <c r="A22" s="61">
         <v>1</v>
       </c>
-      <c r="B22" s="49">
+      <c r="B22" s="62">
         <v>1</v>
       </c>
-      <c r="C22" s="49" t="s">
+      <c r="C22" s="62" t="s">
         <v>45</v>
       </c>
-      <c r="D22" s="28" t="s">
+      <c r="D22" s="41" t="s">
         <v>46</v>
       </c>
-      <c r="E22" s="26">
+      <c r="E22" s="39">
         <v>-3</v>
       </c>
-      <c r="H22" s="41"/>
-      <c r="K22" s="53"/>
-    </row>
-    <row r="23" ht="15.75" spans="1:11">
-      <c r="A23" s="50">
+      <c r="H22" s="18"/>
+      <c r="K22" s="17"/>
+    </row>
+    <row r="23" ht="15.75" spans="1:12">
+      <c r="A23" s="63">
         <v>1</v>
       </c>
-      <c r="B23" s="51" t="s">
+      <c r="B23" s="64" t="s">
         <v>47</v>
       </c>
-      <c r="C23" s="52">
+      <c r="C23" s="65">
         <v>6</v>
       </c>
-      <c r="D23" s="51">
+      <c r="D23" s="64">
         <v>2</v>
       </c>
-      <c r="E23" s="33">
+      <c r="E23" s="46">
         <v>3</v>
       </c>
-      <c r="G23" s="23"/>
-      <c r="H23" s="53"/>
-      <c r="I23" s="53"/>
-      <c r="J23" s="53"/>
-      <c r="K23" s="53"/>
-    </row>
-    <row r="24" ht="16.5" spans="1:11">
-      <c r="A24" s="48">
+      <c r="G23" s="36"/>
+      <c r="H23" s="17"/>
+      <c r="I23" s="17"/>
+      <c r="J23" s="17"/>
+      <c r="K23" s="17"/>
+    </row>
+    <row r="24" ht="16.5" spans="1:12">
+      <c r="A24" s="61">
         <v>1</v>
       </c>
-      <c r="B24" s="49" t="s">
+      <c r="B24" s="62" t="s">
         <v>48</v>
       </c>
-      <c r="C24" s="54">
+      <c r="C24" s="66">
         <v>8</v>
       </c>
-      <c r="D24" s="49">
+      <c r="D24" s="62">
         <v>4</v>
       </c>
-      <c r="E24" s="26">
+      <c r="E24" s="39">
         <v>5.5</v>
       </c>
-      <c r="G24" s="23"/>
-      <c r="H24" s="53"/>
-      <c r="I24" s="53"/>
-      <c r="J24" s="53"/>
-      <c r="K24" s="53"/>
-    </row>
-    <row r="25" ht="16.5" spans="1:11">
-      <c r="A25" s="55"/>
-      <c r="B25" s="41"/>
-      <c r="C25" s="41"/>
-      <c r="D25" s="41"/>
-      <c r="E25" s="23"/>
-      <c r="F25" s="23"/>
-      <c r="G25" s="56"/>
-      <c r="H25" s="23"/>
-      <c r="I25" s="53"/>
-      <c r="J25" s="53"/>
-      <c r="K25" s="82"/>
-    </row>
-    <row r="26" ht="15.75" spans="1:11">
-      <c r="A26" s="57"/>
-      <c r="B26" s="34"/>
-      <c r="C26" s="58" t="s">
+      <c r="G24" s="36"/>
+      <c r="H24" s="17"/>
+      <c r="I24" s="17"/>
+      <c r="J24" s="17"/>
+      <c r="K24" s="17"/>
+    </row>
+    <row r="25" ht="16.5" spans="1:12">
+      <c r="A25" s="67"/>
+      <c r="B25" s="18"/>
+      <c r="C25" s="18"/>
+      <c r="D25" s="18"/>
+      <c r="E25" s="36"/>
+      <c r="F25" s="36"/>
+      <c r="G25" s="59"/>
+      <c r="H25" s="36"/>
+      <c r="I25" s="17"/>
+      <c r="J25" s="17"/>
+      <c r="K25" s="68"/>
+    </row>
+    <row r="26" ht="15.75" spans="1:12">
+      <c r="A26" s="69"/>
+      <c r="B26" s="47"/>
+      <c r="C26" s="70" t="s">
         <v>49</v>
       </c>
-      <c r="D26" s="59"/>
-      <c r="E26" s="59"/>
-      <c r="F26" s="60"/>
-      <c r="K26" s="23"/>
+      <c r="D26" s="71"/>
+      <c r="E26" s="71"/>
+      <c r="F26" s="72"/>
+      <c r="K26" s="36"/>
     </row>
     <row r="27" ht="16.5" spans="1:12">
-      <c r="A27" s="61" t="s">
+      <c r="A27" s="73" t="s">
         <v>34</v>
       </c>
-      <c r="B27" s="62" t="s">
+      <c r="B27" s="74" t="s">
         <v>35</v>
       </c>
-      <c r="C27" s="63" t="s">
+      <c r="C27" s="75" t="s">
         <v>50</v>
       </c>
-      <c r="D27" s="64"/>
-      <c r="E27" s="64"/>
-      <c r="F27" s="65"/>
-      <c r="K27" s="83"/>
-      <c r="L27" s="83"/>
-    </row>
-    <row r="28" spans="1:11">
-      <c r="A28" s="22">
+      <c r="D27" s="76"/>
+      <c r="E27" s="76"/>
+      <c r="F27" s="77"/>
+      <c r="K27" s="78"/>
+      <c r="L27" s="78"/>
+    </row>
+    <row r="28" spans="1:12">
+      <c r="A28" s="35">
         <v>0</v>
       </c>
-      <c r="B28" s="23">
+      <c r="B28" s="36">
         <v>0</v>
       </c>
-      <c r="C28" s="22" t="s">
+      <c r="C28" s="35" t="s">
         <v>51</v>
       </c>
-      <c r="D28" s="23" t="s">
+      <c r="D28" s="36" t="s">
         <v>52</v>
       </c>
-      <c r="E28" s="34"/>
-      <c r="F28" s="66"/>
-      <c r="K28" s="23"/>
-    </row>
-    <row r="29" spans="1:11">
-      <c r="A29" s="22">
+      <c r="E28" s="47"/>
+      <c r="F28" s="79"/>
+      <c r="K28" s="36"/>
+    </row>
+    <row r="29" spans="1:12">
+      <c r="A29" s="35">
         <v>0.5</v>
       </c>
-      <c r="B29" s="23">
+      <c r="B29" s="36">
         <v>0</v>
       </c>
-      <c r="C29" s="67" t="s">
+      <c r="C29" s="80" t="s">
         <v>53</v>
       </c>
-      <c r="D29" s="68" t="s">
+      <c r="D29" s="81" t="s">
         <v>54</v>
       </c>
-      <c r="E29" s="23"/>
-      <c r="F29" s="24"/>
-      <c r="K29" s="23"/>
-    </row>
-    <row r="30" spans="1:11">
-      <c r="A30" s="22">
+      <c r="E29" s="36"/>
+      <c r="F29" s="37"/>
+      <c r="K29" s="36"/>
+    </row>
+    <row r="30" spans="1:12">
+      <c r="A30" s="35">
         <v>1</v>
       </c>
-      <c r="B30" s="23">
+      <c r="B30" s="36">
         <v>0</v>
       </c>
-      <c r="C30" s="69"/>
-      <c r="D30" s="70"/>
-      <c r="E30" s="70"/>
-      <c r="F30" s="71"/>
-      <c r="K30" s="23"/>
-    </row>
-    <row r="31" spans="1:6">
-      <c r="A31" s="22">
+      <c r="C30" s="82"/>
+      <c r="D30" s="83"/>
+      <c r="E30" s="83"/>
+      <c r="F30" s="84"/>
+      <c r="K30" s="36"/>
+    </row>
+    <row r="31" spans="1:12">
+      <c r="A31" s="35">
         <v>0</v>
       </c>
-      <c r="B31" s="23">
+      <c r="B31" s="36">
         <v>1</v>
       </c>
-      <c r="C31" s="22" t="s">
+      <c r="C31" s="35" t="s">
         <v>55</v>
       </c>
-      <c r="D31" s="23" t="s">
+      <c r="D31" s="36" t="s">
         <v>56</v>
       </c>
-      <c r="E31" s="23" t="s">
+      <c r="E31" s="36" t="s">
         <v>57</v>
       </c>
-      <c r="F31" s="24" t="s">
+      <c r="F31" s="37" t="s">
         <v>58</v>
       </c>
     </row>
-    <row r="32" spans="1:6">
-      <c r="A32" s="22">
+    <row r="32" spans="1:12">
+      <c r="A32" s="35">
         <v>0.5</v>
       </c>
-      <c r="B32" s="23">
+      <c r="B32" s="36">
         <v>1</v>
       </c>
-      <c r="C32" s="22" t="s">
+      <c r="C32" s="35" t="s">
         <v>59</v>
       </c>
-      <c r="D32" s="23" t="s">
+      <c r="D32" s="36" t="s">
         <v>60</v>
       </c>
-      <c r="E32" s="23"/>
-      <c r="F32" s="24"/>
-    </row>
-    <row r="33" ht="15.75" spans="1:6">
-      <c r="A33" s="27">
+      <c r="E32" s="36"/>
+      <c r="F32" s="37"/>
+    </row>
+    <row r="33" ht="15.75" spans="1:11">
+      <c r="A33" s="40">
         <v>1</v>
       </c>
-      <c r="B33" s="28">
+      <c r="B33" s="41">
         <v>1</v>
       </c>
-      <c r="C33" s="27"/>
-      <c r="D33" s="28"/>
-      <c r="E33" s="28"/>
-      <c r="F33" s="29"/>
+      <c r="C33" s="40"/>
+      <c r="D33" s="41"/>
+      <c r="E33" s="41"/>
+      <c r="F33" s="42"/>
     </row>
     <row r="34" ht="15.75" spans="1:11">
-      <c r="A34" s="50">
+      <c r="A34" s="63">
         <v>1</v>
       </c>
-      <c r="B34" s="72" t="s">
+      <c r="B34" s="85" t="s">
         <v>47</v>
       </c>
-      <c r="C34" s="57" t="s">
+      <c r="C34" s="69" t="s">
         <v>61</v>
       </c>
-      <c r="D34" s="73"/>
-      <c r="E34" s="73"/>
-      <c r="F34" s="72"/>
-      <c r="K34" s="41"/>
+      <c r="D34" s="86"/>
+      <c r="E34" s="86"/>
+      <c r="F34" s="85"/>
+      <c r="K34" s="18"/>
     </row>
     <row r="35" ht="16.5" spans="1:11">
-      <c r="A35" s="48">
+      <c r="A35" s="61">
         <v>1</v>
       </c>
-      <c r="B35" s="74" t="s">
+      <c r="B35" s="87" t="s">
         <v>48</v>
       </c>
-      <c r="C35" s="48" t="s">
+      <c r="C35" s="61" t="s">
         <v>62</v>
       </c>
-      <c r="D35" s="75" t="s">
+      <c r="D35" s="88" t="s">
         <v>63</v>
       </c>
-      <c r="E35" s="75"/>
-      <c r="F35" s="74"/>
-      <c r="K35" s="41"/>
+      <c r="E35" s="88"/>
+      <c r="F35" s="87"/>
+      <c r="K35" s="18"/>
     </row>
     <row r="36" ht="15.75" spans="1:11">
-      <c r="A36" s="41"/>
-      <c r="B36" s="41"/>
-      <c r="C36" s="41"/>
-      <c r="D36" s="41"/>
-      <c r="E36" s="41"/>
-      <c r="F36" s="41"/>
-      <c r="G36" s="41"/>
-      <c r="H36" s="41"/>
-      <c r="I36" s="23"/>
-      <c r="J36" s="23"/>
-      <c r="K36" s="41"/>
+      <c r="A36" s="18"/>
+      <c r="B36" s="18"/>
+      <c r="C36" s="18"/>
+      <c r="D36" s="18"/>
+      <c r="E36" s="18"/>
+      <c r="F36" s="18"/>
+      <c r="G36" s="18"/>
+      <c r="H36" s="18"/>
+      <c r="I36" s="36"/>
+      <c r="J36" s="36"/>
+      <c r="K36" s="18"/>
     </row>
     <row r="37" ht="16.5" spans="1:11">
-      <c r="A37" s="41"/>
-      <c r="B37" s="41"/>
-      <c r="C37" s="41"/>
-      <c r="D37" s="41"/>
-      <c r="E37" s="41"/>
-      <c r="F37" s="41"/>
-      <c r="G37" s="41"/>
-      <c r="H37" s="41"/>
-      <c r="I37" s="23"/>
-      <c r="J37" s="23"/>
-      <c r="K37" s="41"/>
+      <c r="A37" s="18"/>
+      <c r="B37" s="18"/>
+      <c r="C37" s="18"/>
+      <c r="D37" s="18"/>
+      <c r="E37" s="18"/>
+      <c r="F37" s="18"/>
+      <c r="G37" s="18"/>
+      <c r="H37" s="18"/>
+      <c r="I37" s="36"/>
+      <c r="J37" s="36"/>
+      <c r="K37" s="18"/>
     </row>
     <row r="38" ht="16.5" spans="1:11">
-      <c r="A38" s="41"/>
-      <c r="C38" s="50" t="s">
+      <c r="A38" s="18"/>
+      <c r="C38" s="63" t="s">
         <v>64</v>
       </c>
-      <c r="D38" s="72"/>
-      <c r="F38" s="41"/>
-      <c r="G38" s="41"/>
-      <c r="H38" s="55"/>
-      <c r="I38" s="41"/>
-      <c r="J38" s="23"/>
-      <c r="K38" s="41"/>
+      <c r="D38" s="85"/>
+      <c r="F38" s="18"/>
+      <c r="G38" s="18"/>
+      <c r="H38" s="67"/>
+      <c r="I38" s="18"/>
+      <c r="J38" s="36"/>
+      <c r="K38" s="18"/>
     </row>
     <row r="39" ht="16.5" spans="1:11">
-      <c r="A39" s="55"/>
-      <c r="B39" s="57" t="s">
+      <c r="A39" s="67"/>
+      <c r="B39" s="69" t="s">
         <v>65</v>
       </c>
-      <c r="C39" s="34" t="s">
+      <c r="C39" s="47" t="s">
         <v>66</v>
       </c>
-      <c r="D39" s="34" t="s">
+      <c r="D39" s="47" t="s">
         <v>67</v>
       </c>
-      <c r="E39" s="72" t="s">
+      <c r="E39" s="85" t="s">
         <v>68</v>
       </c>
-      <c r="G39" s="23"/>
-      <c r="H39" s="23" t="s">
+      <c r="G39" s="36"/>
+      <c r="H39" s="36" t="s">
         <v>69</v>
       </c>
-      <c r="I39" s="23"/>
-      <c r="J39" s="23"/>
-      <c r="K39" s="84"/>
+      <c r="I39" s="36"/>
+      <c r="J39" s="36"/>
+      <c r="K39" s="89"/>
     </row>
     <row r="40" ht="15.75" spans="1:11">
-      <c r="A40" s="55"/>
-      <c r="B40" s="22">
+      <c r="A40" s="67"/>
+      <c r="B40" s="35">
         <v>25</v>
       </c>
-      <c r="C40" s="23">
+      <c r="C40" s="36">
         <v>7</v>
       </c>
-      <c r="D40" s="23">
+      <c r="D40" s="36">
         <v>1.5</v>
       </c>
-      <c r="E40" s="76">
+      <c r="E40" s="90">
         <v>10</v>
       </c>
-      <c r="G40" s="57" t="s">
+      <c r="G40" s="69" t="s">
         <v>70</v>
       </c>
-      <c r="H40" s="33" t="s">
+      <c r="H40" s="46" t="s">
         <v>71</v>
       </c>
-      <c r="I40" s="33" t="s">
+      <c r="I40" s="46" t="s">
         <v>72</v>
       </c>
-      <c r="K40" s="41"/>
+      <c r="K40" s="18"/>
     </row>
     <row r="41" ht="15.75" spans="1:11">
-      <c r="A41" s="55"/>
-      <c r="B41" s="22">
+      <c r="A41" s="67"/>
+      <c r="B41" s="35">
         <v>50</v>
       </c>
-      <c r="C41" s="23">
+      <c r="C41" s="36">
         <v>14</v>
       </c>
-      <c r="D41" s="23">
+      <c r="D41" s="36">
         <v>2.5</v>
       </c>
-      <c r="E41" s="76">
+      <c r="E41" s="90">
         <v>10</v>
       </c>
-      <c r="G41" s="22">
+      <c r="G41" s="35">
         <v>1</v>
       </c>
-      <c r="H41" s="38">
+      <c r="H41" s="51">
         <v>21.5</v>
       </c>
-      <c r="I41" s="38">
+      <c r="I41" s="51">
         <v>7</v>
       </c>
-      <c r="K41" s="41"/>
+      <c r="K41" s="18"/>
     </row>
     <row r="42" ht="15.75" spans="1:11">
-      <c r="A42" s="55"/>
-      <c r="B42" s="22">
+      <c r="A42" s="67"/>
+      <c r="B42" s="35">
         <v>75</v>
       </c>
-      <c r="C42" s="23">
+      <c r="C42" s="36">
         <v>20</v>
       </c>
-      <c r="D42" s="23">
+      <c r="D42" s="36">
         <v>3.5</v>
       </c>
-      <c r="E42" s="76">
+      <c r="E42" s="90">
         <v>10</v>
       </c>
-      <c r="G42" s="22">
+      <c r="G42" s="35">
         <v>2</v>
       </c>
-      <c r="H42" s="38">
+      <c r="H42" s="51">
         <v>25.5</v>
       </c>
-      <c r="I42" s="38">
+      <c r="I42" s="51">
         <v>9</v>
       </c>
-      <c r="K42" s="41"/>
+      <c r="K42" s="18"/>
     </row>
     <row r="43" ht="15.75" spans="1:11">
-      <c r="A43" s="55" t="s">
+      <c r="A43" s="67" t="s">
         <v>73</v>
       </c>
-      <c r="B43" s="35">
+      <c r="B43" s="48">
         <v>100</v>
       </c>
-      <c r="C43" s="23">
+      <c r="C43" s="36">
         <v>25</v>
       </c>
-      <c r="D43" s="41">
+      <c r="D43" s="18">
         <v>5</v>
       </c>
-      <c r="E43" s="76">
+      <c r="E43" s="90">
         <v>10</v>
       </c>
-      <c r="G43" s="22">
+      <c r="G43" s="35">
         <v>3</v>
       </c>
-      <c r="H43" s="38">
+      <c r="H43" s="51">
         <v>29.5</v>
       </c>
-      <c r="I43" s="38">
+      <c r="I43" s="51">
         <v>11</v>
       </c>
-      <c r="K43" s="41"/>
+      <c r="K43" s="18"/>
     </row>
     <row r="44" ht="15.75" spans="1:11">
-      <c r="A44" s="55" t="s">
+      <c r="A44" s="67" t="s">
         <v>74</v>
       </c>
-      <c r="B44" s="22">
+      <c r="B44" s="35">
         <v>125</v>
       </c>
-      <c r="C44" s="23">
+      <c r="C44" s="36">
         <v>30</v>
       </c>
-      <c r="D44" s="41">
+      <c r="D44" s="18">
         <v>6.5</v>
       </c>
-      <c r="E44" s="76">
+      <c r="E44" s="90">
         <v>10</v>
       </c>
-      <c r="G44" s="22">
+      <c r="G44" s="35">
         <v>4</v>
       </c>
-      <c r="H44" s="38">
+      <c r="H44" s="51">
         <v>33.5</v>
       </c>
-      <c r="I44" s="38">
+      <c r="I44" s="51">
         <v>13</v>
       </c>
-      <c r="K44" s="41"/>
+      <c r="K44" s="18"/>
     </row>
     <row r="45" ht="15.75" spans="1:11">
-      <c r="A45" s="55"/>
-      <c r="B45" s="22">
+      <c r="A45" s="67"/>
+      <c r="B45" s="35">
         <v>150</v>
       </c>
-      <c r="C45" s="23">
+      <c r="C45" s="36">
         <v>35</v>
       </c>
-      <c r="D45" s="41">
+      <c r="D45" s="18">
         <v>7.5</v>
       </c>
-      <c r="E45" s="76">
+      <c r="E45" s="90">
         <v>10</v>
       </c>
-      <c r="G45" s="22">
+      <c r="G45" s="35">
         <v>5</v>
       </c>
-      <c r="H45" s="38">
+      <c r="H45" s="51">
         <v>37.5</v>
       </c>
-      <c r="I45" s="38">
+      <c r="I45" s="51">
         <v>15</v>
       </c>
-      <c r="K45" s="41"/>
+      <c r="K45" s="18"/>
     </row>
     <row r="46" ht="15.75" spans="1:11">
-      <c r="A46" s="55" t="s">
+      <c r="A46" s="67" t="s">
         <v>75</v>
       </c>
-      <c r="B46" s="22">
+      <c r="B46" s="35">
         <v>175</v>
       </c>
-      <c r="C46" s="23">
+      <c r="C46" s="36">
         <v>40</v>
       </c>
-      <c r="D46" s="41">
+      <c r="D46" s="18">
         <v>8.5</v>
       </c>
-      <c r="E46" s="76">
+      <c r="E46" s="90">
         <v>10</v>
       </c>
       <c r="F46" t="s">
         <v>76</v>
       </c>
-      <c r="G46" s="22">
+      <c r="G46" s="35">
         <v>6</v>
       </c>
-      <c r="H46" s="38">
+      <c r="H46" s="51">
         <v>41.5</v>
       </c>
-      <c r="I46" s="38">
+      <c r="I46" s="51">
         <v>17</v>
       </c>
-      <c r="K46" s="41"/>
+      <c r="K46" s="18"/>
     </row>
     <row r="47" ht="15.75" spans="1:11">
-      <c r="A47" s="55" t="s">
+      <c r="A47" s="67" t="s">
         <v>77</v>
       </c>
-      <c r="B47" s="22">
+      <c r="B47" s="35">
         <v>200</v>
       </c>
-      <c r="C47" s="23">
+      <c r="C47" s="36">
         <v>45</v>
       </c>
-      <c r="D47" s="41">
+      <c r="D47" s="18">
         <v>9.5</v>
       </c>
-      <c r="E47" s="76">
+      <c r="E47" s="90">
         <v>11</v>
       </c>
       <c r="F47" t="s">
         <v>78</v>
       </c>
-      <c r="G47" s="22">
+      <c r="G47" s="35">
         <v>7</v>
       </c>
-      <c r="H47" s="38">
+      <c r="H47" s="51">
         <v>45.5</v>
       </c>
-      <c r="I47" s="38">
+      <c r="I47" s="51">
         <v>19</v>
       </c>
-      <c r="K47" s="41"/>
+      <c r="K47" s="18"/>
     </row>
     <row r="48" ht="15.75" spans="1:11">
-      <c r="A48" s="55"/>
-      <c r="B48" s="35">
+      <c r="A48" s="67"/>
+      <c r="B48" s="48">
         <v>225</v>
       </c>
-      <c r="C48" s="23">
+      <c r="C48" s="36">
         <v>50</v>
       </c>
-      <c r="D48" s="41">
+      <c r="D48" s="18">
         <v>10.5</v>
       </c>
-      <c r="E48" s="76">
+      <c r="E48" s="90">
         <v>11</v>
       </c>
       <c r="F48" t="s">
         <v>79</v>
       </c>
-      <c r="G48" s="22">
+      <c r="G48" s="35">
         <v>8</v>
       </c>
-      <c r="H48" s="38">
+      <c r="H48" s="51">
         <v>49.5</v>
       </c>
-      <c r="I48" s="38">
+      <c r="I48" s="51">
         <v>21</v>
       </c>
-      <c r="K48" s="41"/>
-    </row>
-    <row r="49" ht="15.75" spans="1:11">
-      <c r="A49" s="55" t="s">
+      <c r="K48" s="18"/>
+    </row>
+    <row r="49" ht="15.75" spans="1:13">
+      <c r="A49" s="67" t="s">
         <v>80</v>
       </c>
-      <c r="B49" s="22">
+      <c r="B49" s="35">
         <v>250</v>
       </c>
-      <c r="C49" s="23">
+      <c r="C49" s="36">
         <v>55</v>
       </c>
-      <c r="D49" s="41">
+      <c r="D49" s="18">
         <v>11.5</v>
       </c>
-      <c r="E49" s="76">
+      <c r="E49" s="90">
         <v>11</v>
       </c>
       <c r="F49" t="s">
         <v>81</v>
       </c>
-      <c r="G49" s="22">
+      <c r="G49" s="35">
         <v>9</v>
       </c>
-      <c r="H49" s="38">
+      <c r="H49" s="51">
         <v>53.5</v>
       </c>
-      <c r="I49" s="38">
+      <c r="I49" s="51">
         <v>23</v>
       </c>
-      <c r="K49" s="41"/>
-    </row>
-    <row r="50" ht="16.5" spans="1:11">
-      <c r="A50" s="55" t="s">
+      <c r="K49" s="18"/>
+    </row>
+    <row r="50" ht="16.5" spans="1:13">
+      <c r="A50" s="67" t="s">
         <v>82</v>
       </c>
-      <c r="B50" s="22">
+      <c r="B50" s="35">
         <v>275</v>
       </c>
-      <c r="C50" s="23">
+      <c r="C50" s="36">
         <v>60</v>
       </c>
-      <c r="D50" s="41">
+      <c r="D50" s="18">
         <v>12.5</v>
       </c>
-      <c r="E50" s="76">
+      <c r="E50" s="90">
         <v>11</v>
       </c>
       <c r="F50" t="s">
         <v>83</v>
       </c>
-      <c r="G50" s="27">
+      <c r="G50" s="40">
         <v>10</v>
       </c>
-      <c r="H50" s="26">
+      <c r="H50" s="39">
         <v>57.5</v>
       </c>
-      <c r="I50" s="26">
+      <c r="I50" s="39">
         <v>25</v>
       </c>
-      <c r="K50" s="41"/>
+      <c r="K50" s="18"/>
     </row>
     <row r="51" ht="16.5" spans="1:13">
-      <c r="A51" s="55"/>
-      <c r="B51" s="77">
+      <c r="A51" s="67"/>
+      <c r="B51" s="91">
         <v>300</v>
       </c>
-      <c r="C51" s="23">
+      <c r="C51" s="36">
         <v>65</v>
       </c>
-      <c r="D51" s="41">
+      <c r="D51" s="18">
         <v>13.5</v>
       </c>
-      <c r="E51" s="24">
+      <c r="E51" s="37">
         <v>12</v>
       </c>
       <c r="F51" t="s">
         <v>84</v>
       </c>
-      <c r="G51" s="23"/>
-      <c r="H51" s="23"/>
-      <c r="I51" s="85"/>
-      <c r="J51" s="85"/>
-      <c r="K51" s="53"/>
-      <c r="M51" s="41"/>
+      <c r="G51" s="36"/>
+      <c r="H51" s="36"/>
+      <c r="I51" s="92"/>
+      <c r="J51" s="92"/>
+      <c r="K51" s="17"/>
+      <c r="M51" s="18"/>
     </row>
     <row r="52" ht="16.5" spans="1:13">
-      <c r="A52" s="78" t="s">
+      <c r="A52" s="93" t="s">
         <v>85</v>
       </c>
-      <c r="B52" s="77">
+      <c r="B52" s="91">
         <v>325</v>
       </c>
-      <c r="C52" s="23">
+      <c r="C52" s="36">
         <v>70</v>
       </c>
-      <c r="D52" s="41">
+      <c r="D52" s="18">
         <v>14.5</v>
       </c>
-      <c r="E52" s="24">
+      <c r="E52" s="37">
         <v>12</v>
       </c>
-      <c r="G52" s="79" t="s">
+      <c r="G52" s="94" t="s">
         <v>86</v>
       </c>
-      <c r="H52" s="79" t="s">
+      <c r="H52" s="94" t="s">
         <v>87</v>
       </c>
-      <c r="I52" s="86" t="s">
+      <c r="I52" s="95" t="s">
         <v>88</v>
       </c>
-      <c r="J52" s="87" t="s">
+      <c r="J52" s="96" t="s">
         <v>89</v>
       </c>
-      <c r="M52" s="41"/>
+      <c r="M52" s="18"/>
     </row>
     <row r="53" ht="15.75" spans="1:13">
-      <c r="A53" s="78" t="s">
+      <c r="A53" s="93" t="s">
         <v>90</v>
       </c>
-      <c r="B53" s="22">
+      <c r="B53" s="35">
         <v>350</v>
       </c>
-      <c r="C53" s="23">
+      <c r="C53" s="36">
         <v>75</v>
       </c>
-      <c r="D53" s="41">
+      <c r="D53" s="18">
         <v>15.5</v>
       </c>
-      <c r="E53" s="24">
+      <c r="E53" s="37">
         <v>12</v>
       </c>
-      <c r="G53" s="80" t="s">
+      <c r="G53" s="97" t="s">
         <v>91</v>
       </c>
-      <c r="H53" s="80">
+      <c r="H53" s="97">
         <v>16</v>
       </c>
-      <c r="I53" s="33">
+      <c r="I53" s="46">
         <v>8</v>
       </c>
-      <c r="J53" s="66">
+      <c r="J53" s="79">
         <f>H53+2*I53</f>
         <v>32</v>
       </c>
-      <c r="M53" s="41"/>
-    </row>
-    <row r="54" ht="16.5" spans="1:10">
-      <c r="A54" s="78"/>
-      <c r="B54" s="48">
+      <c r="M53" s="18"/>
+    </row>
+    <row r="54" ht="16.5" spans="1:13">
+      <c r="A54" s="93"/>
+      <c r="B54" s="61">
         <v>375</v>
       </c>
-      <c r="C54" s="28">
+      <c r="C54" s="41">
         <v>80</v>
       </c>
-      <c r="D54" s="28">
+      <c r="D54" s="41">
         <v>10.5</v>
       </c>
-      <c r="E54" s="29">
+      <c r="E54" s="42">
         <v>12</v>
       </c>
-      <c r="G54" s="22" t="s">
+      <c r="G54" s="35" t="s">
         <v>92</v>
       </c>
-      <c r="H54" s="22">
+      <c r="H54" s="35">
         <v>18</v>
       </c>
-      <c r="I54" s="38">
+      <c r="I54" s="51">
         <v>7</v>
       </c>
-      <c r="J54" s="24">
+      <c r="J54" s="37">
         <f>H54+2*I54</f>
         <v>32</v>
       </c>
     </row>
-    <row r="55" ht="15.75" spans="1:10">
-      <c r="A55" s="55" t="s">
+    <row r="55" ht="15.75" spans="1:13">
+      <c r="A55" s="67" t="s">
         <v>93</v>
       </c>
-      <c r="B55" s="22">
+      <c r="B55" s="35">
         <v>400</v>
       </c>
-      <c r="C55" s="23">
+      <c r="C55" s="36">
         <v>85</v>
       </c>
-      <c r="D55" s="23">
+      <c r="D55" s="36">
         <v>11</v>
       </c>
-      <c r="E55" s="24">
+      <c r="E55" s="37">
         <v>12</v>
       </c>
-      <c r="G55" s="22" t="s">
+      <c r="G55" s="35" t="s">
         <v>94</v>
       </c>
-      <c r="H55" s="22">
+      <c r="H55" s="35">
         <v>21</v>
       </c>
-      <c r="I55" s="38">
+      <c r="I55" s="51">
         <v>5</v>
       </c>
-      <c r="J55" s="24">
+      <c r="J55" s="37">
         <f t="shared" ref="J55:J61" si="0">H55+2*I55</f>
         <v>31</v>
       </c>
     </row>
-    <row r="56" ht="15.75" spans="1:10">
-      <c r="A56" s="55"/>
-      <c r="B56" s="22">
+    <row r="56" ht="15.75" spans="1:13">
+      <c r="A56" s="67"/>
+      <c r="B56" s="35">
         <v>425</v>
       </c>
-      <c r="C56" s="23">
+      <c r="C56" s="36">
         <v>90</v>
       </c>
-      <c r="D56" s="23" t="s">
+      <c r="D56" s="36" t="s">
         <v>95</v>
       </c>
-      <c r="E56" s="24">
+      <c r="E56" s="37">
         <v>12</v>
       </c>
-      <c r="G56" s="22" t="s">
+      <c r="G56" s="35" t="s">
         <v>96</v>
       </c>
-      <c r="H56" s="22">
+      <c r="H56" s="35">
         <v>22</v>
       </c>
-      <c r="I56" s="38">
+      <c r="I56" s="51">
         <v>5</v>
       </c>
-      <c r="J56" s="24">
+      <c r="J56" s="37">
         <f t="shared" si="0"/>
         <v>32</v>
       </c>
     </row>
-    <row r="57" ht="15.75" spans="1:10">
-      <c r="A57" s="55" t="s">
+    <row r="57" ht="15.75" spans="1:13">
+      <c r="A57" s="67" t="s">
         <v>97</v>
       </c>
-      <c r="B57" s="22">
+      <c r="B57" s="35">
         <v>450</v>
       </c>
-      <c r="C57" s="23">
+      <c r="C57" s="36">
         <v>95</v>
       </c>
-      <c r="D57" s="23" t="s">
+      <c r="D57" s="36" t="s">
         <v>98</v>
       </c>
-      <c r="E57" s="24">
+      <c r="E57" s="37">
         <v>12</v>
       </c>
-      <c r="G57" s="25" t="s">
+      <c r="G57" s="38" t="s">
         <v>99</v>
       </c>
-      <c r="H57" s="25">
+      <c r="H57" s="38">
         <v>16</v>
       </c>
-      <c r="I57" s="38">
+      <c r="I57" s="51">
         <v>8</v>
       </c>
-      <c r="J57" s="24">
+      <c r="J57" s="37">
         <f t="shared" si="0"/>
         <v>32</v>
       </c>
     </row>
-    <row r="58" ht="15.75" spans="1:10">
-      <c r="A58" s="55"/>
-      <c r="B58" s="22">
+    <row r="58" ht="15.75" spans="1:13">
+      <c r="A58" s="67"/>
+      <c r="B58" s="35">
         <v>475</v>
       </c>
-      <c r="C58" s="23">
+      <c r="C58" s="36">
         <v>100</v>
       </c>
-      <c r="D58" s="23" t="s">
+      <c r="D58" s="36" t="s">
         <v>100</v>
       </c>
-      <c r="E58" s="24">
+      <c r="E58" s="37">
         <v>12</v>
       </c>
-      <c r="G58" s="22" t="s">
+      <c r="G58" s="35" t="s">
         <v>101</v>
       </c>
-      <c r="H58" s="22">
+      <c r="H58" s="35">
         <v>14</v>
       </c>
-      <c r="I58" s="38">
+      <c r="I58" s="51">
         <v>9</v>
       </c>
-      <c r="J58" s="24">
+      <c r="J58" s="37">
         <f t="shared" si="0"/>
         <v>32</v>
       </c>
     </row>
-    <row r="59" ht="15.75" spans="2:10">
-      <c r="B59" s="35">
+    <row r="59" ht="15.75" spans="1:13">
+      <c r="B59" s="48">
         <v>500</v>
       </c>
-      <c r="C59" s="23">
+      <c r="C59" s="36">
         <v>105</v>
       </c>
-      <c r="D59" s="77" t="s">
+      <c r="D59" s="91" t="s">
         <v>102</v>
       </c>
-      <c r="E59" s="24">
+      <c r="E59" s="37">
         <v>12</v>
       </c>
-      <c r="G59" s="22" t="s">
+      <c r="G59" s="35" t="s">
         <v>103</v>
       </c>
-      <c r="H59" s="22">
+      <c r="H59" s="35">
         <v>20</v>
       </c>
-      <c r="I59" s="38">
+      <c r="I59" s="51">
         <v>6</v>
       </c>
-      <c r="J59" s="24">
+      <c r="J59" s="37">
         <f t="shared" si="0"/>
         <v>32</v>
       </c>
     </row>
-    <row r="60" ht="15.75" spans="1:10">
-      <c r="A60" s="55"/>
-      <c r="B60" s="35">
+    <row r="60" ht="15.75" spans="1:13">
+      <c r="A60" s="67"/>
+      <c r="B60" s="48">
         <v>600</v>
       </c>
-      <c r="C60" s="77"/>
-      <c r="D60" s="77">
+      <c r="C60" s="91"/>
+      <c r="D60" s="91">
         <v>14.5</v>
       </c>
-      <c r="E60" s="24">
+      <c r="E60" s="37">
         <v>13</v>
       </c>
-      <c r="G60" s="22" t="s">
+      <c r="G60" s="35" t="s">
         <v>104</v>
       </c>
-      <c r="H60" s="22">
+      <c r="H60" s="35">
         <v>17</v>
       </c>
-      <c r="I60" s="38">
+      <c r="I60" s="51">
         <v>4</v>
       </c>
-      <c r="J60" s="24">
+      <c r="J60" s="37">
         <f t="shared" si="0"/>
         <v>25</v>
       </c>
     </row>
-    <row r="61" ht="16.5" spans="2:10">
-      <c r="B61" s="35">
+    <row r="61" ht="16.5" spans="1:13">
+      <c r="B61" s="48">
         <v>750</v>
       </c>
-      <c r="C61" s="77"/>
-      <c r="D61" s="77">
+      <c r="C61" s="91"/>
+      <c r="D61" s="91">
         <v>15</v>
       </c>
-      <c r="E61" s="24">
+      <c r="E61" s="37">
         <v>13</v>
       </c>
-      <c r="G61" s="27" t="s">
+      <c r="G61" s="40" t="s">
         <v>105</v>
       </c>
-      <c r="H61" s="27">
+      <c r="H61" s="40">
         <v>26</v>
       </c>
-      <c r="I61" s="26">
+      <c r="I61" s="39">
         <v>3</v>
       </c>
-      <c r="J61" s="29">
+      <c r="J61" s="42">
         <f t="shared" si="0"/>
         <v>32</v>
       </c>
     </row>
-    <row r="62" ht="16.5" spans="2:9">
-      <c r="B62" s="48">
+    <row r="62" ht="16.5" spans="1:13">
+      <c r="B62" s="61">
         <v>1000</v>
       </c>
-      <c r="C62" s="28"/>
-      <c r="D62" s="28">
+      <c r="C62" s="41"/>
+      <c r="D62" s="41">
         <v>15.5</v>
       </c>
-      <c r="E62" s="29">
+      <c r="E62" s="42">
         <v>13</v>
       </c>
-      <c r="H62" s="23"/>
-      <c r="I62" s="23"/>
-    </row>
-    <row r="63" spans="7:9">
-      <c r="G63" s="23"/>
-      <c r="H63" s="23"/>
-      <c r="I63" s="23"/>
-    </row>
-    <row r="64" ht="15.75" spans="7:9">
-      <c r="G64" s="23"/>
-      <c r="H64" s="23"/>
-      <c r="I64" s="23"/>
-    </row>
-    <row r="65" ht="75.75" spans="1:10">
+      <c r="H62" s="36"/>
+      <c r="I62" s="36"/>
+    </row>
+    <row r="63" spans="1:13">
+      <c r="G63" s="36"/>
+      <c r="H63" s="36"/>
+      <c r="I63" s="36"/>
+    </row>
+    <row r="64" ht="15.75" spans="1:13">
+      <c r="G64" s="36"/>
+      <c r="H64" s="36"/>
+      <c r="I64" s="36"/>
+    </row>
+    <row r="65" ht="75.75" spans="1:14">
       <c r="A65">
         <f>147*2*0.8</f>
         <v>235.2</v>
       </c>
-      <c r="C65" s="88" t="s">
+      <c r="C65" s="98" t="s">
         <v>106</v>
       </c>
-      <c r="D65" s="88" t="s">
+      <c r="D65" s="98" t="s">
         <v>107</v>
       </c>
-      <c r="E65" s="88" t="s">
+      <c r="E65" s="98" t="s">
         <v>108</v>
       </c>
-      <c r="G65" s="23"/>
-      <c r="H65" s="89" t="s">
+      <c r="G65" s="36"/>
+      <c r="H65" s="99" t="s">
         <v>109</v>
       </c>
       <c r="I65" t="s">
         <v>110</v>
       </c>
-      <c r="J65" s="41"/>
-    </row>
-    <row r="66" ht="90.75" spans="3:10">
-      <c r="C66" s="88" t="s">
+      <c r="J65" s="18"/>
+    </row>
+    <row r="66" ht="90.75" spans="1:14">
+      <c r="C66" s="98" t="s">
         <v>111</v>
       </c>
-      <c r="E66" s="23"/>
-      <c r="F66" s="23"/>
-      <c r="G66" s="23"/>
-      <c r="H66" s="23" t="s">
+      <c r="E66" s="36"/>
+      <c r="F66" s="36"/>
+      <c r="G66" s="36"/>
+      <c r="H66" s="36" t="s">
         <v>112</v>
       </c>
       <c r="I66" t="s">
         <v>113</v>
       </c>
-      <c r="J66" s="23" t="s">
+      <c r="J66" s="36" t="s">
         <v>114</v>
       </c>
     </row>
-    <row r="67" spans="5:10">
-      <c r="E67" s="90"/>
-      <c r="F67" s="23"/>
-      <c r="G67" s="23"/>
-      <c r="H67" s="23" t="s">
+    <row r="67" spans="1:14">
+      <c r="E67" s="100"/>
+      <c r="F67" s="36"/>
+      <c r="G67" s="36"/>
+      <c r="H67" s="36" t="s">
         <v>112</v>
       </c>
       <c r="I67" t="s">
         <v>115</v>
       </c>
-      <c r="J67" s="23" t="s">
+      <c r="J67" s="36" t="s">
         <v>114</v>
       </c>
     </row>
-    <row r="68" spans="3:10">
-      <c r="C68" s="23"/>
-      <c r="E68" s="23"/>
-      <c r="F68" s="23"/>
-      <c r="G68" s="23"/>
-      <c r="H68" s="23" t="s">
+    <row r="68" spans="1:14">
+      <c r="C68" s="36"/>
+      <c r="E68" s="36"/>
+      <c r="F68" s="36"/>
+      <c r="G68" s="36"/>
+      <c r="H68" s="36" t="s">
         <v>112</v>
       </c>
       <c r="I68" t="s">
         <v>116</v>
       </c>
-      <c r="J68" s="23" t="s">
+      <c r="J68" s="36" t="s">
         <v>117</v>
       </c>
     </row>
-    <row r="69" ht="13" customHeight="1" spans="5:10">
-      <c r="E69" s="23"/>
-      <c r="F69" s="23"/>
-      <c r="G69" s="23"/>
-      <c r="H69" s="23" t="s">
+    <row r="69" ht="13" customHeight="1" spans="1:14">
+      <c r="E69" s="36"/>
+      <c r="F69" s="36"/>
+      <c r="G69" s="36"/>
+      <c r="H69" s="36" t="s">
         <v>118</v>
       </c>
-      <c r="I69" s="89" t="s">
+      <c r="I69" s="99" t="s">
         <v>119</v>
       </c>
-      <c r="J69" s="23" t="s">
+      <c r="J69" s="36" t="s">
         <v>117</v>
       </c>
     </row>
-    <row r="70" spans="5:10">
-      <c r="E70" s="23"/>
-      <c r="F70" s="23"/>
-      <c r="G70" s="23"/>
-      <c r="H70" s="23" t="s">
+    <row r="70" spans="1:14">
+      <c r="E70" s="36"/>
+      <c r="F70" s="36"/>
+      <c r="G70" s="36"/>
+      <c r="H70" s="36" t="s">
         <v>120</v>
       </c>
-      <c r="I70" s="89" t="s">
+      <c r="I70" s="99" t="s">
         <v>121</v>
       </c>
-      <c r="J70" s="23" t="s">
+      <c r="J70" s="36" t="s">
         <v>122</v>
       </c>
     </row>
     <row r="71" ht="15.75" spans="1:14">
-      <c r="A71" s="91"/>
-      <c r="B71" s="92"/>
-      <c r="C71" s="93"/>
-      <c r="D71" s="93"/>
-      <c r="E71" s="41"/>
-      <c r="F71" s="41"/>
-      <c r="G71" s="41"/>
-      <c r="H71" s="41"/>
-      <c r="I71" s="41"/>
-      <c r="J71" s="41"/>
-      <c r="K71" s="41"/>
-      <c r="M71" s="23"/>
-      <c r="N71" s="23"/>
+      <c r="A71" s="101"/>
+      <c r="B71" s="102"/>
+      <c r="C71" s="103"/>
+      <c r="D71" s="103"/>
+      <c r="E71" s="18"/>
+      <c r="F71" s="18"/>
+      <c r="G71" s="18"/>
+      <c r="H71" s="18"/>
+      <c r="I71" s="18"/>
+      <c r="J71" s="18"/>
+      <c r="K71" s="18"/>
+      <c r="M71" s="36"/>
+      <c r="N71" s="36"/>
     </row>
     <row r="72" spans="1:14">
-      <c r="A72" s="23"/>
-      <c r="F72" s="23"/>
-      <c r="G72" s="23"/>
-      <c r="H72" s="23"/>
-      <c r="I72" s="23"/>
-      <c r="J72" s="23"/>
-      <c r="K72" s="23"/>
-      <c r="M72" s="23"/>
-      <c r="N72" s="23"/>
+      <c r="A72" s="36"/>
+      <c r="F72" s="36"/>
+      <c r="G72" s="36"/>
+      <c r="H72" s="36"/>
+      <c r="I72" s="36"/>
+      <c r="J72" s="36"/>
+      <c r="K72" s="36"/>
+      <c r="M72" s="36"/>
+      <c r="N72" s="36"/>
     </row>
     <row r="73" spans="1:14">
-      <c r="A73" s="23"/>
-      <c r="F73" s="23"/>
-      <c r="G73" s="94" t="s">
+      <c r="A73" s="36"/>
+      <c r="F73" s="36"/>
+      <c r="G73" s="104" t="s">
         <v>91</v>
       </c>
-      <c r="H73" s="94"/>
-      <c r="I73" s="94"/>
-      <c r="J73" s="23"/>
-      <c r="K73" s="23"/>
-      <c r="M73" s="23"/>
-      <c r="N73" s="23"/>
+      <c r="H73" s="104"/>
+      <c r="I73" s="104"/>
+      <c r="J73" s="36"/>
+      <c r="K73" s="36"/>
+      <c r="M73" s="36"/>
+      <c r="N73" s="36"/>
     </row>
     <row r="74" spans="1:14">
-      <c r="A74" s="23"/>
-      <c r="F74" s="23"/>
-      <c r="G74" s="23" t="s">
+      <c r="A74" s="36"/>
+      <c r="F74" s="36"/>
+      <c r="G74" s="36" t="s">
         <v>92</v>
       </c>
-      <c r="H74" s="23"/>
-      <c r="I74" s="23"/>
-      <c r="J74" s="23"/>
-      <c r="K74" s="23"/>
-      <c r="L74" s="23"/>
-      <c r="M74" s="23"/>
-      <c r="N74" s="23"/>
+      <c r="H74" s="36"/>
+      <c r="I74" s="36"/>
+      <c r="J74" s="36"/>
+      <c r="K74" s="36"/>
+      <c r="L74" s="36"/>
+      <c r="M74" s="36"/>
+      <c r="N74" s="36"/>
     </row>
     <row r="75" spans="1:14">
-      <c r="A75" s="23"/>
-      <c r="F75" s="23"/>
-      <c r="G75" s="23" t="s">
+      <c r="A75" s="36"/>
+      <c r="F75" s="36"/>
+      <c r="G75" s="36" t="s">
         <v>94</v>
       </c>
-      <c r="H75" s="23"/>
-      <c r="I75" s="23"/>
-      <c r="J75" s="23"/>
-      <c r="K75" s="23"/>
-      <c r="L75" s="23"/>
-      <c r="M75" s="23"/>
-      <c r="N75" s="23"/>
+      <c r="H75" s="36"/>
+      <c r="I75" s="36"/>
+      <c r="J75" s="36"/>
+      <c r="K75" s="36"/>
+      <c r="L75" s="36"/>
+      <c r="M75" s="36"/>
+      <c r="N75" s="36"/>
     </row>
     <row r="76" spans="1:14">
-      <c r="A76" s="23"/>
-      <c r="F76" s="23"/>
-      <c r="G76" s="23" t="s">
+      <c r="A76" s="36"/>
+      <c r="F76" s="36"/>
+      <c r="G76" s="36" t="s">
         <v>96</v>
       </c>
-      <c r="H76" s="23"/>
-      <c r="I76" s="23"/>
-      <c r="J76" s="23"/>
-      <c r="K76" s="23"/>
-      <c r="M76" s="23"/>
-      <c r="N76" s="23"/>
+      <c r="H76" s="36"/>
+      <c r="I76" s="36"/>
+      <c r="J76" s="36"/>
+      <c r="K76" s="36"/>
+      <c r="M76" s="36"/>
+      <c r="N76" s="36"/>
     </row>
     <row r="77" ht="15.75" spans="1:14">
-      <c r="A77" s="91"/>
-      <c r="F77" s="23"/>
-      <c r="G77" s="95" t="s">
+      <c r="A77" s="101"/>
+      <c r="F77" s="36"/>
+      <c r="G77" s="105" t="s">
         <v>99</v>
       </c>
-      <c r="H77" s="95"/>
-      <c r="I77" s="95"/>
-      <c r="J77" s="97"/>
-      <c r="K77" s="97"/>
-      <c r="L77" s="97"/>
-      <c r="M77" s="23"/>
-      <c r="N77" s="23"/>
+      <c r="H77" s="105"/>
+      <c r="I77" s="105"/>
+      <c r="J77" s="106"/>
+      <c r="K77" s="106"/>
+      <c r="L77" s="106"/>
+      <c r="M77" s="36"/>
+      <c r="N77" s="36"/>
     </row>
     <row r="78" spans="1:14">
-      <c r="A78" s="23"/>
-      <c r="F78" s="23"/>
-      <c r="G78" s="23" t="s">
+      <c r="A78" s="36"/>
+      <c r="F78" s="36"/>
+      <c r="G78" s="36" t="s">
         <v>101</v>
       </c>
-      <c r="H78" s="23"/>
-      <c r="I78" s="23"/>
-      <c r="J78" s="23"/>
-      <c r="K78" s="23"/>
-      <c r="M78" s="23"/>
-      <c r="N78" s="23"/>
+      <c r="H78" s="36"/>
+      <c r="I78" s="36"/>
+      <c r="J78" s="36"/>
+      <c r="K78" s="36"/>
+      <c r="M78" s="36"/>
+      <c r="N78" s="36"/>
     </row>
     <row r="79" spans="1:14">
-      <c r="A79" s="23"/>
-      <c r="F79" s="23"/>
-      <c r="G79" s="23" t="s">
+      <c r="A79" s="36"/>
+      <c r="F79" s="36"/>
+      <c r="G79" s="36" t="s">
         <v>104</v>
       </c>
-      <c r="H79" s="23"/>
-      <c r="I79" s="23"/>
-      <c r="J79" s="23"/>
-      <c r="K79" s="23"/>
-      <c r="L79" s="23"/>
-      <c r="M79" s="23"/>
-      <c r="N79" s="23"/>
+      <c r="H79" s="36"/>
+      <c r="I79" s="36"/>
+      <c r="J79" s="36"/>
+      <c r="K79" s="36"/>
+      <c r="L79" s="36"/>
+      <c r="M79" s="36"/>
+      <c r="N79" s="36"/>
     </row>
     <row r="80" spans="1:14">
-      <c r="A80" s="23"/>
-      <c r="F80" s="23"/>
-      <c r="G80" s="23" t="s">
+      <c r="A80" s="36"/>
+      <c r="F80" s="36"/>
+      <c r="G80" s="36" t="s">
         <v>103</v>
       </c>
-      <c r="H80" s="23"/>
-      <c r="I80" s="23"/>
-      <c r="J80" s="23"/>
-      <c r="K80" s="23"/>
-      <c r="L80" s="23"/>
-      <c r="M80" s="23"/>
-      <c r="N80" s="23"/>
+      <c r="H80" s="36"/>
+      <c r="I80" s="36"/>
+      <c r="J80" s="36"/>
+      <c r="K80" s="36"/>
+      <c r="L80" s="36"/>
+      <c r="M80" s="36"/>
+      <c r="N80" s="36"/>
     </row>
     <row r="81" spans="1:11">
-      <c r="A81" s="23"/>
-      <c r="F81" s="23"/>
-      <c r="G81" s="23" t="s">
+      <c r="A81" s="36"/>
+      <c r="F81" s="36"/>
+      <c r="G81" s="36" t="s">
         <v>105</v>
       </c>
-      <c r="H81" s="23"/>
-      <c r="I81" s="23"/>
-      <c r="J81" s="23"/>
-      <c r="K81" s="23"/>
+      <c r="H81" s="36"/>
+      <c r="I81" s="36"/>
+      <c r="J81" s="36"/>
+      <c r="K81" s="36"/>
     </row>
     <row r="82" spans="1:11">
-      <c r="A82" s="23"/>
-      <c r="F82" s="23"/>
-      <c r="G82" s="23"/>
-      <c r="H82" s="23"/>
-      <c r="I82" s="23"/>
-      <c r="J82" s="23"/>
-      <c r="K82" s="23"/>
+      <c r="A82" s="36"/>
+      <c r="F82" s="36"/>
+      <c r="G82" s="36"/>
+      <c r="H82" s="36"/>
+      <c r="I82" s="36"/>
+      <c r="J82" s="36"/>
+      <c r="K82" s="36"/>
     </row>
     <row r="83" spans="1:11">
-      <c r="A83" s="23"/>
-      <c r="F83" s="23"/>
-      <c r="G83" s="23"/>
-      <c r="H83" s="23"/>
-      <c r="I83" s="23"/>
-      <c r="J83" s="23"/>
-      <c r="K83" s="23"/>
+      <c r="A83" s="36"/>
+      <c r="F83" s="36"/>
+      <c r="G83" s="36"/>
+      <c r="H83" s="36"/>
+      <c r="I83" s="36"/>
+      <c r="J83" s="36"/>
+      <c r="K83" s="36"/>
     </row>
     <row r="84" spans="1:11">
-      <c r="A84" s="23"/>
-      <c r="F84" s="85"/>
-      <c r="G84" s="85"/>
-      <c r="H84" s="23">
+      <c r="A84" s="36"/>
+      <c r="F84" s="92"/>
+      <c r="G84" s="92"/>
+      <c r="H84" s="36">
         <v>5</v>
       </c>
-      <c r="I84" s="23">
+      <c r="I84" s="36">
         <v>3</v>
       </c>
-      <c r="J84" s="23"/>
-      <c r="K84" s="23"/>
-    </row>
-    <row r="85" spans="6:11">
-      <c r="F85" s="23"/>
-      <c r="G85" s="23"/>
-      <c r="H85" s="90"/>
-      <c r="I85" s="23"/>
-      <c r="J85" s="23"/>
-      <c r="K85" s="23"/>
-    </row>
-    <row r="86" spans="6:11">
-      <c r="F86" s="23"/>
-      <c r="G86" s="23"/>
-      <c r="H86" s="23"/>
-      <c r="I86" s="23"/>
-      <c r="J86" s="23"/>
-      <c r="K86" s="23"/>
-    </row>
-    <row r="87" spans="6:11">
-      <c r="F87" s="23"/>
-      <c r="G87" s="23"/>
-      <c r="H87" s="23"/>
-      <c r="I87" s="23"/>
-      <c r="J87" s="23"/>
-      <c r="K87" s="23"/>
-    </row>
-    <row r="88" spans="6:11">
-      <c r="F88" s="23"/>
-      <c r="H88" s="23"/>
-      <c r="I88" s="23"/>
-      <c r="J88" s="23"/>
-      <c r="K88" s="23"/>
-    </row>
-    <row r="89" spans="6:11">
-      <c r="F89" s="23"/>
-      <c r="H89" s="23"/>
-      <c r="I89" s="23"/>
-      <c r="J89" s="23"/>
-      <c r="K89" s="23"/>
-    </row>
-    <row r="90" spans="6:11">
-      <c r="F90" s="23"/>
-      <c r="G90" s="23"/>
-      <c r="H90" s="23"/>
-      <c r="I90" s="23"/>
-      <c r="J90" s="23"/>
-      <c r="K90" s="23"/>
-    </row>
-    <row r="91" spans="6:11">
-      <c r="F91" s="23"/>
-      <c r="G91" s="23"/>
-      <c r="H91" s="23"/>
-      <c r="I91" s="23"/>
-      <c r="J91" s="23"/>
-      <c r="K91" s="23"/>
-    </row>
-    <row r="92" spans="6:11">
-      <c r="F92" s="23"/>
-      <c r="G92" s="23"/>
-      <c r="H92" s="23"/>
-      <c r="I92" s="23"/>
-      <c r="J92" s="23"/>
-      <c r="K92" s="23"/>
-    </row>
-    <row r="93" spans="6:11">
-      <c r="F93" s="23"/>
-      <c r="G93" s="23"/>
-      <c r="H93" s="23"/>
-      <c r="I93" s="23"/>
-      <c r="J93" s="23"/>
-      <c r="K93" s="23"/>
-    </row>
-    <row r="94" spans="6:11">
-      <c r="F94" s="96"/>
-      <c r="G94" s="23"/>
-      <c r="H94" s="23"/>
-      <c r="I94" s="23"/>
-      <c r="J94" s="23"/>
-      <c r="K94" s="23"/>
-    </row>
-    <row r="95" spans="2:11">
-      <c r="B95" s="23"/>
-      <c r="C95" s="23">
+      <c r="J84" s="36"/>
+      <c r="K84" s="36"/>
+    </row>
+    <row r="85" spans="1:11">
+      <c r="F85" s="36"/>
+      <c r="G85" s="36"/>
+      <c r="H85" s="100"/>
+      <c r="I85" s="36"/>
+      <c r="J85" s="36"/>
+      <c r="K85" s="36"/>
+    </row>
+    <row r="86" spans="1:11">
+      <c r="F86" s="36"/>
+      <c r="G86" s="36"/>
+      <c r="H86" s="36"/>
+      <c r="I86" s="36"/>
+      <c r="J86" s="36"/>
+      <c r="K86" s="36"/>
+    </row>
+    <row r="87" spans="1:11">
+      <c r="F87" s="36"/>
+      <c r="G87" s="36"/>
+      <c r="H87" s="36"/>
+      <c r="I87" s="36"/>
+      <c r="J87" s="36"/>
+      <c r="K87" s="36"/>
+    </row>
+    <row r="88" spans="1:11">
+      <c r="F88" s="36"/>
+      <c r="H88" s="36"/>
+      <c r="I88" s="36"/>
+      <c r="J88" s="36"/>
+      <c r="K88" s="36"/>
+    </row>
+    <row r="89" spans="1:11">
+      <c r="F89" s="36"/>
+      <c r="H89" s="36"/>
+      <c r="I89" s="36"/>
+      <c r="J89" s="36"/>
+      <c r="K89" s="36"/>
+    </row>
+    <row r="90" spans="1:11">
+      <c r="F90" s="36"/>
+      <c r="G90" s="36"/>
+      <c r="H90" s="36"/>
+      <c r="I90" s="36"/>
+      <c r="J90" s="36"/>
+      <c r="K90" s="36"/>
+    </row>
+    <row r="91" spans="1:11">
+      <c r="F91" s="36"/>
+      <c r="G91" s="36"/>
+      <c r="H91" s="36"/>
+      <c r="I91" s="36"/>
+      <c r="J91" s="36"/>
+      <c r="K91" s="36"/>
+    </row>
+    <row r="92" spans="1:11">
+      <c r="F92" s="36"/>
+      <c r="G92" s="36"/>
+      <c r="H92" s="36"/>
+      <c r="I92" s="36"/>
+      <c r="J92" s="36"/>
+      <c r="K92" s="36"/>
+    </row>
+    <row r="93" spans="1:11">
+      <c r="F93" s="36"/>
+      <c r="G93" s="36"/>
+      <c r="H93" s="36"/>
+      <c r="I93" s="36"/>
+      <c r="J93" s="36"/>
+      <c r="K93" s="36"/>
+    </row>
+    <row r="94" spans="1:11">
+      <c r="F94" s="107"/>
+      <c r="G94" s="36"/>
+      <c r="H94" s="36"/>
+      <c r="I94" s="36"/>
+      <c r="J94" s="36"/>
+      <c r="K94" s="36"/>
+    </row>
+    <row r="95" spans="1:11">
+      <c r="B95" s="36"/>
+      <c r="C95" s="36">
         <f>AVERAGE(H53:H61)</f>
         <v>18.8888888888889</v>
       </c>
-      <c r="D95" s="23">
+      <c r="D95" s="36">
         <f>AVERAGE(I53:I61)</f>
         <v>6.11111111111111</v>
       </c>
-      <c r="E95" s="23"/>
-      <c r="F95" s="23"/>
-      <c r="G95" s="23"/>
-      <c r="H95" s="23"/>
-      <c r="I95" s="23"/>
-      <c r="J95" s="23"/>
-      <c r="K95" s="23"/>
-    </row>
-    <row r="96" spans="5:11">
-      <c r="E96" s="23"/>
-      <c r="I96" s="23"/>
-      <c r="J96" s="23"/>
-      <c r="K96" s="23"/>
+      <c r="E95" s="36"/>
+      <c r="F95" s="36"/>
+      <c r="G95" s="36"/>
+      <c r="H95" s="36"/>
+      <c r="I95" s="36"/>
+      <c r="J95" s="36"/>
+      <c r="K95" s="36"/>
+    </row>
+    <row r="96" spans="1:11">
+      <c r="E96" s="36"/>
+      <c r="I96" s="36"/>
+      <c r="J96" s="36"/>
+      <c r="K96" s="36"/>
     </row>
     <row r="97" spans="1:11">
-      <c r="A97" s="23"/>
-      <c r="B97" s="23"/>
-      <c r="C97" s="23"/>
-      <c r="D97" s="23"/>
-      <c r="E97" s="23"/>
-      <c r="F97" s="96"/>
-      <c r="G97" s="23"/>
-      <c r="H97" s="23"/>
-      <c r="I97" s="23"/>
-      <c r="J97" s="23"/>
-      <c r="K97" s="23"/>
+      <c r="A97" s="36"/>
+      <c r="B97" s="36"/>
+      <c r="C97" s="36"/>
+      <c r="D97" s="36"/>
+      <c r="E97" s="36"/>
+      <c r="F97" s="107"/>
+      <c r="G97" s="36"/>
+      <c r="H97" s="36"/>
+      <c r="I97" s="36"/>
+      <c r="J97" s="36"/>
+      <c r="K97" s="36"/>
     </row>
     <row r="98" spans="1:11">
-      <c r="A98" s="23"/>
-      <c r="B98" s="23"/>
-      <c r="C98" s="23"/>
-      <c r="D98" s="23"/>
-      <c r="E98" s="23"/>
-      <c r="F98" s="23"/>
-      <c r="G98" s="23"/>
-      <c r="H98" s="23"/>
-      <c r="I98" s="23"/>
-      <c r="J98" s="23"/>
-      <c r="K98" s="23"/>
-    </row>
-    <row r="99" spans="2:6">
-      <c r="B99" s="23"/>
-      <c r="C99" s="23"/>
-      <c r="D99" s="23"/>
-      <c r="E99" s="23"/>
-      <c r="F99" s="23"/>
-    </row>
-    <row r="100" spans="1:6">
-      <c r="A100" s="23"/>
-      <c r="B100" s="23"/>
-      <c r="C100" s="23"/>
-      <c r="D100" s="23"/>
-      <c r="E100" s="23"/>
-      <c r="F100" s="23"/>
-    </row>
-    <row r="101" spans="3:6">
-      <c r="C101" s="23"/>
-      <c r="D101" s="23"/>
-      <c r="E101" s="23"/>
-      <c r="F101" s="23"/>
-    </row>
-    <row r="102" spans="3:6">
-      <c r="C102" s="23"/>
-      <c r="D102" s="23"/>
-      <c r="E102" s="23"/>
-      <c r="F102" s="89"/>
-    </row>
-    <row r="103" spans="3:6">
-      <c r="C103" s="23"/>
-      <c r="D103" s="23"/>
-      <c r="E103" s="23"/>
-      <c r="F103" s="23"/>
-    </row>
-    <row r="104" spans="3:6">
-      <c r="C104" s="23"/>
-      <c r="D104" s="23"/>
-      <c r="E104" s="23"/>
-      <c r="F104" s="23"/>
-    </row>
-    <row r="105" spans="3:6">
-      <c r="C105" s="23"/>
-      <c r="D105" s="23"/>
-      <c r="E105" s="23"/>
-      <c r="F105" s="23"/>
-    </row>
-    <row r="106" spans="3:6">
-      <c r="C106" s="23"/>
-      <c r="D106" s="23"/>
-      <c r="E106" s="23"/>
-      <c r="F106" s="23"/>
-    </row>
-    <row r="107" spans="3:6">
-      <c r="C107" s="23"/>
-      <c r="D107" s="23"/>
-      <c r="E107" s="23"/>
-      <c r="F107" s="23"/>
-    </row>
-    <row r="108" spans="3:6">
-      <c r="C108" s="23"/>
-      <c r="D108" s="23"/>
-      <c r="E108" s="23"/>
-      <c r="F108" s="23"/>
-    </row>
-    <row r="109" spans="3:6">
-      <c r="C109" s="23"/>
-      <c r="D109" s="23"/>
-      <c r="E109" s="23"/>
-      <c r="F109" s="23"/>
-    </row>
-    <row r="110" spans="3:6">
-      <c r="C110" s="23"/>
-      <c r="D110" s="23"/>
-      <c r="E110" s="23"/>
-      <c r="F110" s="23"/>
-    </row>
-    <row r="111" spans="3:6">
-      <c r="C111" s="23"/>
-      <c r="D111" s="23"/>
-      <c r="E111" s="23"/>
-      <c r="F111" s="23"/>
+      <c r="A98" s="36"/>
+      <c r="B98" s="36"/>
+      <c r="C98" s="36"/>
+      <c r="D98" s="36"/>
+      <c r="E98" s="36"/>
+      <c r="F98" s="36"/>
+      <c r="G98" s="36"/>
+      <c r="H98" s="36"/>
+      <c r="I98" s="36"/>
+      <c r="J98" s="36"/>
+      <c r="K98" s="36"/>
+    </row>
+    <row r="99" spans="1:11">
+      <c r="B99" s="36"/>
+      <c r="C99" s="36"/>
+      <c r="D99" s="36"/>
+      <c r="E99" s="36"/>
+      <c r="F99" s="36"/>
+    </row>
+    <row r="100" spans="1:11">
+      <c r="A100" s="36"/>
+      <c r="B100" s="36"/>
+      <c r="C100" s="36"/>
+      <c r="D100" s="36"/>
+      <c r="E100" s="36"/>
+      <c r="F100" s="36"/>
+    </row>
+    <row r="101" spans="1:11">
+      <c r="C101" s="36"/>
+      <c r="D101" s="36"/>
+      <c r="E101" s="36"/>
+      <c r="F101" s="36"/>
+    </row>
+    <row r="102" spans="1:11">
+      <c r="C102" s="36"/>
+      <c r="D102" s="36"/>
+      <c r="E102" s="36"/>
+      <c r="F102" s="99"/>
+    </row>
+    <row r="103" spans="1:11">
+      <c r="C103" s="36"/>
+      <c r="D103" s="36"/>
+      <c r="E103" s="36"/>
+      <c r="F103" s="36"/>
+    </row>
+    <row r="104" spans="1:11">
+      <c r="C104" s="36"/>
+      <c r="D104" s="36"/>
+      <c r="E104" s="36"/>
+      <c r="F104" s="36"/>
+    </row>
+    <row r="105" spans="1:11">
+      <c r="C105" s="36"/>
+      <c r="D105" s="36"/>
+      <c r="E105" s="36"/>
+      <c r="F105" s="36"/>
+    </row>
+    <row r="106" spans="1:11">
+      <c r="C106" s="36"/>
+      <c r="D106" s="36"/>
+      <c r="E106" s="36"/>
+      <c r="F106" s="36"/>
+    </row>
+    <row r="107" spans="1:11">
+      <c r="C107" s="36"/>
+      <c r="D107" s="36"/>
+      <c r="E107" s="36"/>
+      <c r="F107" s="36"/>
+    </row>
+    <row r="108" spans="1:11">
+      <c r="C108" s="36"/>
+      <c r="D108" s="36"/>
+      <c r="E108" s="36"/>
+      <c r="F108" s="36"/>
+    </row>
+    <row r="109" spans="1:11">
+      <c r="C109" s="36"/>
+      <c r="D109" s="36"/>
+      <c r="E109" s="36"/>
+      <c r="F109" s="36"/>
+    </row>
+    <row r="110" spans="1:11">
+      <c r="C110" s="36"/>
+      <c r="D110" s="36"/>
+      <c r="E110" s="36"/>
+      <c r="F110" s="36"/>
+    </row>
+    <row r="111" spans="1:11">
+      <c r="C111" s="36"/>
+      <c r="D111" s="36"/>
+      <c r="E111" s="36"/>
+      <c r="F111" s="36"/>
     </row>
   </sheetData>
   <mergeCells count="14">
@@ -3898,4 +4030,401 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511805555555556" footer="0.511805555555556"/>
   <headerFooter/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
+  <dimension ref="A1:O11"/>
+  <sheetFormatPr defaultColWidth="9.14285714285714" defaultRowHeight="18.75"/>
+  <cols>
+    <col min="1" max="1" width="9.14285714285714" style="2"/>
+    <col min="2" max="2" width="12.5714285714286" style="3" customWidth="1"/>
+    <col min="3" max="3" width="11.1428571428571" style="3" customWidth="1"/>
+    <col min="4" max="4" width="14.8571428571429" style="3" customWidth="1"/>
+    <col min="5" max="5" width="18.1428571428571" style="3" customWidth="1"/>
+    <col min="6" max="6" width="11.2857142857143" style="3" customWidth="1"/>
+    <col min="7" max="7" width="12" style="3" customWidth="1"/>
+    <col min="8" max="8" width="12.1428571428571" style="3" customWidth="1"/>
+    <col min="9" max="9" width="14.1428571428571" style="3" customWidth="1"/>
+    <col min="10" max="10" width="13.7142857142857" style="3" customWidth="1"/>
+    <col min="11" max="11" width="11.7142857142857" style="3" customWidth="1"/>
+    <col min="12" max="12" width="17.2857142857143" style="3" customWidth="1"/>
+    <col min="13" max="13" width="12.1428571428571" style="3" customWidth="1"/>
+    <col min="14" max="14" width="11" style="3" customWidth="1"/>
+    <col min="15" max="16384" width="9.14285714285714" style="3"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="19.5"/>
+    <row r="2" s="1" customFormat="1" ht="19.5" spans="1:15">
+      <c r="A2" s="4"/>
+      <c r="B2" s="5" t="s">
+        <v>123</v>
+      </c>
+      <c r="C2" s="6" t="s">
+        <v>124</v>
+      </c>
+      <c r="D2" s="6" t="s">
+        <v>125</v>
+      </c>
+      <c r="E2" s="6" t="s">
+        <v>126</v>
+      </c>
+      <c r="F2" s="6" t="s">
+        <v>127</v>
+      </c>
+      <c r="G2" s="6" t="s">
+        <v>128</v>
+      </c>
+      <c r="H2" s="6" t="s">
+        <v>129</v>
+      </c>
+      <c r="I2" s="6" t="s">
+        <v>130</v>
+      </c>
+      <c r="J2" s="6" t="s">
+        <v>131</v>
+      </c>
+      <c r="K2" s="6" t="s">
+        <v>132</v>
+      </c>
+      <c r="L2" s="6" t="s">
+        <v>133</v>
+      </c>
+      <c r="M2" s="6"/>
+      <c r="N2" s="6"/>
+      <c r="O2" s="6"/>
+    </row>
+    <row r="3" spans="1:15">
+      <c r="A3" s="7">
+        <v>2</v>
+      </c>
+      <c r="B3" s="8" t="s">
+        <v>134</v>
+      </c>
+      <c r="C3" s="9" t="s">
+        <v>134</v>
+      </c>
+      <c r="D3" s="9" t="s">
+        <v>135</v>
+      </c>
+      <c r="E3" s="9" t="s">
+        <v>136</v>
+      </c>
+      <c r="F3" s="9" t="s">
+        <v>134</v>
+      </c>
+      <c r="G3" s="9" t="s">
+        <v>134</v>
+      </c>
+      <c r="H3" s="9" t="s">
+        <v>137</v>
+      </c>
+      <c r="I3" s="9" t="s">
+        <v>138</v>
+      </c>
+      <c r="J3" s="9" t="s">
+        <v>134</v>
+      </c>
+      <c r="K3" s="9" t="s">
+        <v>137</v>
+      </c>
+      <c r="L3" s="9" t="s">
+        <v>137</v>
+      </c>
+      <c r="M3" s="9"/>
+      <c r="N3" s="9"/>
+      <c r="O3" s="9"/>
+    </row>
+    <row r="4" spans="1:15">
+      <c r="A4" s="7">
+        <v>3</v>
+      </c>
+      <c r="B4" s="8" t="s">
+        <v>137</v>
+      </c>
+      <c r="C4" s="9" t="s">
+        <v>134</v>
+      </c>
+      <c r="D4" s="9" t="s">
+        <v>137</v>
+      </c>
+      <c r="E4" s="9" t="s">
+        <v>138</v>
+      </c>
+      <c r="F4" s="9" t="s">
+        <v>137</v>
+      </c>
+      <c r="G4" s="9" t="s">
+        <v>137</v>
+      </c>
+      <c r="H4" s="9" t="s">
+        <v>134</v>
+      </c>
+      <c r="I4" s="9" t="s">
+        <v>138</v>
+      </c>
+      <c r="J4" s="9" t="s">
+        <v>134</v>
+      </c>
+      <c r="K4" s="9" t="s">
+        <v>137</v>
+      </c>
+      <c r="L4" s="9" t="s">
+        <v>137</v>
+      </c>
+      <c r="M4" s="9"/>
+      <c r="N4" s="9"/>
+      <c r="O4" s="9"/>
+    </row>
+    <row r="5" spans="1:15">
+      <c r="A5" s="7">
+        <v>4</v>
+      </c>
+      <c r="B5" s="9" t="s">
+        <v>134</v>
+      </c>
+      <c r="C5" s="9" t="s">
+        <v>137</v>
+      </c>
+      <c r="D5" s="9"/>
+      <c r="E5" s="9" t="s">
+        <v>138</v>
+      </c>
+      <c r="F5" s="9" t="s">
+        <v>134</v>
+      </c>
+      <c r="G5" s="9" t="s">
+        <v>137</v>
+      </c>
+      <c r="H5" s="9" t="s">
+        <v>137</v>
+      </c>
+      <c r="I5" s="9" t="s">
+        <v>138</v>
+      </c>
+      <c r="J5" s="9" t="s">
+        <v>137</v>
+      </c>
+      <c r="K5" s="10" t="s">
+        <v>139</v>
+      </c>
+      <c r="L5" s="9" t="s">
+        <v>134</v>
+      </c>
+      <c r="M5" s="9"/>
+      <c r="N5" s="9"/>
+      <c r="O5" s="9"/>
+    </row>
+    <row r="6" spans="1:15">
+      <c r="A6" s="7">
+        <v>5</v>
+      </c>
+      <c r="B6" s="9" t="s">
+        <v>137</v>
+      </c>
+      <c r="C6" s="9" t="s">
+        <v>134</v>
+      </c>
+      <c r="D6" s="9" t="s">
+        <v>137</v>
+      </c>
+      <c r="E6" s="9" t="s">
+        <v>138</v>
+      </c>
+      <c r="F6" s="9" t="s">
+        <v>137</v>
+      </c>
+      <c r="G6" s="9" t="s">
+        <v>134</v>
+      </c>
+      <c r="H6" s="9" t="s">
+        <v>134</v>
+      </c>
+      <c r="I6" s="9"/>
+      <c r="J6" s="9" t="s">
+        <v>137</v>
+      </c>
+      <c r="K6" s="9"/>
+      <c r="L6" s="9" t="s">
+        <v>137</v>
+      </c>
+      <c r="M6" s="9"/>
+      <c r="N6" s="9"/>
+      <c r="O6" s="9"/>
+    </row>
+    <row r="7" spans="1:15">
+      <c r="A7" s="7">
+        <v>6</v>
+      </c>
+      <c r="B7" s="8" t="s">
+        <v>140</v>
+      </c>
+      <c r="C7" s="8" t="s">
+        <v>140</v>
+      </c>
+      <c r="D7" s="8" t="s">
+        <v>140</v>
+      </c>
+      <c r="E7" s="8" t="s">
+        <v>140</v>
+      </c>
+      <c r="F7" s="8" t="s">
+        <v>140</v>
+      </c>
+      <c r="G7" s="8" t="s">
+        <v>140</v>
+      </c>
+      <c r="H7" s="8" t="s">
+        <v>140</v>
+      </c>
+      <c r="I7" s="8" t="s">
+        <v>140</v>
+      </c>
+      <c r="J7" s="8" t="s">
+        <v>140</v>
+      </c>
+      <c r="K7" s="8" t="s">
+        <v>140</v>
+      </c>
+      <c r="L7" s="8" t="s">
+        <v>140</v>
+      </c>
+      <c r="M7" s="8"/>
+      <c r="N7" s="8"/>
+      <c r="O7" s="8"/>
+    </row>
+    <row r="8" spans="1:15">
+      <c r="A8" s="7">
+        <v>7</v>
+      </c>
+      <c r="B8" s="9"/>
+      <c r="C8" s="9" t="s">
+        <v>137</v>
+      </c>
+      <c r="D8" s="9"/>
+      <c r="E8" s="9" t="s">
+        <v>138</v>
+      </c>
+      <c r="F8" s="9"/>
+      <c r="G8" s="9" t="s">
+        <v>137</v>
+      </c>
+      <c r="H8" s="9" t="s">
+        <v>137</v>
+      </c>
+      <c r="I8" s="9" t="s">
+        <v>138</v>
+      </c>
+      <c r="J8" s="9" t="s">
+        <v>137</v>
+      </c>
+      <c r="K8" s="9" t="s">
+        <v>137</v>
+      </c>
+      <c r="L8" s="9" t="s">
+        <v>137</v>
+      </c>
+      <c r="M8" s="9"/>
+      <c r="N8" s="9"/>
+      <c r="O8" s="9"/>
+    </row>
+    <row r="9" spans="1:15">
+      <c r="A9" s="7">
+        <v>8</v>
+      </c>
+      <c r="B9" s="9"/>
+      <c r="C9" s="9"/>
+      <c r="D9" s="9"/>
+      <c r="E9" s="9" t="s">
+        <v>141</v>
+      </c>
+      <c r="F9" s="9"/>
+      <c r="G9" s="9"/>
+      <c r="H9" s="9"/>
+      <c r="I9" s="9"/>
+      <c r="J9" s="9"/>
+      <c r="K9" s="9"/>
+      <c r="L9" s="9"/>
+      <c r="M9" s="9"/>
+      <c r="N9" s="9"/>
+      <c r="O9" s="9"/>
+    </row>
+    <row r="10" spans="1:15">
+      <c r="A10" s="7">
+        <v>9</v>
+      </c>
+      <c r="B10" s="9" t="s">
+        <v>137</v>
+      </c>
+      <c r="C10" s="9"/>
+      <c r="D10" s="9" t="s">
+        <v>137</v>
+      </c>
+      <c r="E10" s="9" t="s">
+        <v>142</v>
+      </c>
+      <c r="F10" s="9"/>
+      <c r="G10" s="9"/>
+      <c r="H10" s="9"/>
+      <c r="I10" s="9" t="s">
+        <v>138</v>
+      </c>
+      <c r="J10" s="9"/>
+      <c r="K10" s="9" t="s">
+        <v>137</v>
+      </c>
+      <c r="L10" s="9"/>
+      <c r="M10" s="9"/>
+      <c r="N10" s="9"/>
+      <c r="O10" s="9"/>
+    </row>
+    <row r="11" spans="1:15">
+      <c r="A11" s="7">
+        <v>10</v>
+      </c>
+      <c r="B11" s="8" t="s">
+        <v>143</v>
+      </c>
+      <c r="C11" s="8" t="s">
+        <v>143</v>
+      </c>
+      <c r="D11" s="8" t="s">
+        <v>143</v>
+      </c>
+      <c r="E11" s="8" t="s">
+        <v>143</v>
+      </c>
+      <c r="F11" s="8" t="s">
+        <v>143</v>
+      </c>
+      <c r="G11" s="8" t="s">
+        <v>143</v>
+      </c>
+      <c r="H11" s="8" t="s">
+        <v>143</v>
+      </c>
+      <c r="I11" s="8" t="s">
+        <v>143</v>
+      </c>
+      <c r="J11" s="8"/>
+      <c r="K11" s="8" t="s">
+        <v>143</v>
+      </c>
+      <c r="L11" s="8" t="s">
+        <v>143</v>
+      </c>
+      <c r="M11" s="8"/>
+      <c r="N11" s="8"/>
+      <c r="O11" s="8"/>
+    </row>
+  </sheetData>
+  <mergeCells count="3">
+    <mergeCell ref="G8:G9"/>
+    <mergeCell ref="J8:J9"/>
+    <mergeCell ref="L8:L10"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <headerFooter/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Design: Worked on the Warlock.
</commit_message>
<xml_diff>
--- a/Design/Tables.xlsx
+++ b/Design/Tables.xlsx
@@ -1,10 +1,10 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:dbsheet="http://web.wps.cn/et/2021/dbsheet">
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="27945" windowHeight="12180"/>
+    <workbookView windowWidth="27630" windowHeight="12300"/>
   </bookViews>
   <sheets>
     <sheet name="Standard" sheetId="3" r:id="rId1"/>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="195" uniqueCount="114">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="196" uniqueCount="115">
   <si>
     <t>Action Points</t>
   </si>
@@ -46,6 +46,12 @@
   </si>
   <si>
     <r>
+      <rPr>
+        <sz val="12"/>
+        <rFont val="Calibri"/>
+        <charset val="134"/>
+        <scheme val="minor"/>
+      </rPr>
       <t xml:space="preserve">   6.5 | </t>
     </r>
     <r>
@@ -68,6 +74,21 @@
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve">   14 | </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="4"/>
+        <rFont val="Calibri"/>
+        <charset val="134"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>AoE 10</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">   21.5 | </t>
     </r>
     <r>
       <rPr>
@@ -212,6 +233,13 @@
   </si>
   <si>
     <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <charset val="134"/>
+        <scheme val="minor"/>
+      </rPr>
       <t xml:space="preserve">27 | </t>
     </r>
     <r>
@@ -227,6 +255,13 @@
   </si>
   <si>
     <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <charset val="134"/>
+        <scheme val="minor"/>
+      </rPr>
       <t xml:space="preserve">12 | </t>
     </r>
     <r>
@@ -530,6 +565,13 @@
   </si>
   <si>
     <r>
+      <rPr>
+        <sz val="13"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <charset val="134"/>
+        <scheme val="minor"/>
+      </rPr>
       <t xml:space="preserve">Minor
 </t>
     </r>
@@ -692,7 +734,7 @@
     <font>
       <b/>
       <sz val="12"/>
-      <color rgb="FFF68E08"/>
+      <color rgb="FFCB5D13"/>
       <name val="Calibri"/>
       <charset val="134"/>
       <scheme val="minor"/>
@@ -700,7 +742,7 @@
     <font>
       <b/>
       <sz val="12"/>
-      <color rgb="FFCB5D13"/>
+      <color rgb="FFF68E08"/>
       <name val="Calibri"/>
       <charset val="134"/>
       <scheme val="minor"/>
@@ -1490,7 +1532,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="87">
+  <cellXfs count="86">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -1545,15 +1587,15 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1572,6 +1614,9 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1586,9 +1631,6 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1">
-      <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1608,7 +1650,7 @@
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
@@ -1641,6 +1683,9 @@
     <xf numFmtId="0" fontId="13" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1683,6 +1728,9 @@
     <xf numFmtId="0" fontId="8" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1691,6 +1739,9 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
@@ -1698,6 +1749,12 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1719,37 +1776,19 @@
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -1760,12 +1799,12 @@
     <cellStyle name="Percent" xfId="3" builtinId="5"/>
     <cellStyle name="Comma [0]" xfId="4" builtinId="6"/>
     <cellStyle name="Currency [0]" xfId="5" builtinId="7"/>
-    <cellStyle name="Hyperlink" xfId="6" builtinId="8"/>
+    <cellStyle name="Link" xfId="6" builtinId="8"/>
     <cellStyle name="Followed Hyperlink" xfId="7" builtinId="9"/>
     <cellStyle name="Note" xfId="8" builtinId="10"/>
     <cellStyle name="Warning Text" xfId="9" builtinId="11"/>
     <cellStyle name="Title" xfId="10" builtinId="15"/>
-    <cellStyle name="CExplanatory Text" xfId="11" builtinId="53"/>
+    <cellStyle name="Explanatory Text" xfId="11" builtinId="53"/>
     <cellStyle name="Heading 1" xfId="12" builtinId="16"/>
     <cellStyle name="Heading 2" xfId="13" builtinId="17"/>
     <cellStyle name="Heading 3" xfId="14" builtinId="18"/>
@@ -2081,7 +2120,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A3:N100"/>
+  <dimension ref="A3:N101"/>
   <sheetFormatPr defaultColWidth="9.15238095238095" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="17.2571428571429" customWidth="1"/>
@@ -2100,13 +2139,13 @@
     <col min="14" max="14" width="11" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="3" spans="2:6">
+    <row r="3" ht="15.75" spans="1:11">
       <c r="B3" s="10"/>
       <c r="D3" s="10"/>
       <c r="E3" s="10"/>
       <c r="F3" s="10"/>
     </row>
-    <row r="4" ht="15.75" spans="1:8">
+    <row r="4" ht="15.75" spans="1:11">
       <c r="A4" s="11" t="s">
         <v>0</v>
       </c>
@@ -2124,7 +2163,7 @@
       </c>
       <c r="H4" s="10"/>
     </row>
-    <row r="5" ht="15.75" spans="1:8">
+    <row r="5" ht="15.75" spans="1:11">
       <c r="A5" s="14">
         <v>0</v>
       </c>
@@ -2137,7 +2176,7 @@
       <c r="D5" s="17">
         <v>0</v>
       </c>
-      <c r="E5" s="18">
+      <c r="E5" s="17">
         <v>0</v>
       </c>
       <c r="H5" s="10"/>
@@ -2149,342 +2188,355 @@
       <c r="B6" s="15">
         <v>0</v>
       </c>
-      <c r="C6" s="19" t="s">
+      <c r="C6" s="18" t="s">
         <v>5</v>
       </c>
       <c r="D6" s="17">
         <v>0</v>
       </c>
-      <c r="E6" s="18">
+      <c r="E6" s="17">
         <v>-1</v>
       </c>
-      <c r="H6" s="20"/>
-      <c r="K6" s="32"/>
-    </row>
-    <row r="7" ht="15.75" spans="1:11">
+      <c r="H6" s="19"/>
+      <c r="K6" s="20"/>
+    </row>
+    <row r="7" customFormat="1" ht="15.75" spans="1:11">
       <c r="A7" s="14">
         <v>2</v>
       </c>
       <c r="B7" s="15">
         <v>0</v>
       </c>
-      <c r="C7" s="19" t="s">
+      <c r="C7" s="18" t="s">
         <v>6</v>
       </c>
       <c r="D7" s="17">
         <v>0</v>
       </c>
-      <c r="E7" s="18">
+      <c r="E7" s="17">
         <v>-2</v>
       </c>
       <c r="H7" s="21"/>
-      <c r="K7" s="32"/>
+      <c r="K7" s="20"/>
     </row>
     <row r="8" ht="15.75" spans="1:11">
-      <c r="A8" s="22">
+      <c r="A8" s="14">
+        <v>3</v>
+      </c>
+      <c r="B8" s="15">
         <v>0</v>
       </c>
-      <c r="B8" s="23">
+      <c r="C8" s="18" t="s">
+        <v>7</v>
+      </c>
+      <c r="D8" s="17">
+        <v>0</v>
+      </c>
+      <c r="E8" s="17">
+        <v>-3</v>
+      </c>
+      <c r="F8"/>
+      <c r="H8" s="21"/>
+      <c r="K8" s="20"/>
+    </row>
+    <row r="9" ht="15.75" spans="1:11">
+      <c r="A9" s="22">
+        <v>0</v>
+      </c>
+      <c r="B9" s="23">
         <v>1</v>
       </c>
-      <c r="C8" s="24" t="s">
-        <v>7</v>
-      </c>
-      <c r="D8" s="25" t="s">
+      <c r="C9" s="24" t="s">
         <v>8</v>
       </c>
-      <c r="E8" s="26">
+      <c r="D9" s="25" t="s">
+        <v>9</v>
+      </c>
+      <c r="E9" s="26">
         <v>0</v>
       </c>
-      <c r="H8" s="20"/>
-      <c r="J8" s="39"/>
-      <c r="K8" s="32"/>
-    </row>
-    <row r="9" ht="15.75" spans="1:11">
-      <c r="A9" s="14">
-        <v>1</v>
-      </c>
-      <c r="B9" s="15">
-        <v>1</v>
-      </c>
-      <c r="C9" s="19" t="s">
-        <v>9</v>
-      </c>
-      <c r="D9" s="27" t="s">
-        <v>10</v>
-      </c>
-      <c r="E9" s="18">
-        <v>-1</v>
-      </c>
-      <c r="H9" s="21"/>
-      <c r="K9" s="32"/>
+      <c r="F9"/>
+      <c r="G9"/>
+      <c r="H9" s="19"/>
+      <c r="J9" s="27"/>
+      <c r="K9" s="20"/>
     </row>
     <row r="10" ht="15.75" spans="1:11">
       <c r="A10" s="14">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B10" s="15">
         <v>1</v>
       </c>
-      <c r="C10" s="14" t="s">
+      <c r="C10" s="18" t="s">
+        <v>10</v>
+      </c>
+      <c r="D10" s="28" t="s">
         <v>11</v>
       </c>
-      <c r="D10" s="18" t="s">
+      <c r="E10" s="17">
+        <v>-1</v>
+      </c>
+      <c r="H10" s="21"/>
+      <c r="K10" s="20"/>
+    </row>
+    <row r="11" ht="15.75" spans="1:11">
+      <c r="A11" s="14">
+        <v>2</v>
+      </c>
+      <c r="B11" s="15">
+        <v>1</v>
+      </c>
+      <c r="C11" s="14" t="s">
         <v>12</v>
       </c>
-      <c r="E10" s="18">
+      <c r="D11" s="17" t="s">
+        <v>13</v>
+      </c>
+      <c r="E11" s="17">
         <v>-2</v>
       </c>
-      <c r="H10" s="21"/>
-      <c r="K10" s="32"/>
-    </row>
-    <row r="11" ht="16.5" spans="1:11">
-      <c r="A11" s="28">
+      <c r="F11">
+        <f>5*2.5</f>
+        <v>12.5</v>
+      </c>
+      <c r="H11" s="21"/>
+      <c r="K11" s="20"/>
+    </row>
+    <row r="12" ht="16.5" spans="1:11">
+      <c r="A12" s="29">
         <v>3</v>
       </c>
-      <c r="B11" s="29">
+      <c r="B12" s="30">
         <v>1</v>
       </c>
-      <c r="C11" s="28" t="s">
-        <v>13</v>
-      </c>
-      <c r="D11" s="30" t="s">
+      <c r="C12" s="29" t="s">
         <v>14</v>
       </c>
-      <c r="E11" s="31">
+      <c r="D12" s="31" t="s">
+        <v>15</v>
+      </c>
+      <c r="E12" s="32">
         <v>-3</v>
       </c>
-      <c r="G11" s="10"/>
-      <c r="H11" s="32"/>
-      <c r="I11" s="32"/>
-      <c r="J11" s="32"/>
-      <c r="K11" s="32"/>
-    </row>
-    <row r="12" ht="15.75" spans="1:11">
-      <c r="A12" s="33">
+      <c r="G12" s="10"/>
+      <c r="H12" s="20"/>
+      <c r="I12" s="20"/>
+      <c r="J12" s="20"/>
+      <c r="K12" s="20"/>
+    </row>
+    <row r="13" ht="15.75" spans="1:11">
+      <c r="A13" s="33">
         <v>1</v>
       </c>
-      <c r="B12" s="34" t="s">
-        <v>15</v>
-      </c>
-      <c r="C12" s="35">
+      <c r="B13" s="34" t="s">
+        <v>16</v>
+      </c>
+      <c r="C13" s="35">
         <v>6</v>
       </c>
-      <c r="D12" s="34">
+      <c r="D13" s="34">
         <v>2</v>
       </c>
-      <c r="E12" s="13">
+      <c r="E13" s="13">
         <v>3</v>
       </c>
-      <c r="G12" s="10"/>
-      <c r="H12" s="32"/>
-      <c r="I12" s="32"/>
-      <c r="J12" s="32"/>
-      <c r="K12" s="32"/>
-    </row>
-    <row r="13" ht="16.5" spans="1:11">
-      <c r="A13" s="36">
+      <c r="G13" s="10"/>
+      <c r="H13" s="20"/>
+      <c r="I13" s="20"/>
+      <c r="J13" s="20"/>
+      <c r="K13" s="20"/>
+    </row>
+    <row r="14" ht="16.5" spans="1:11">
+      <c r="A14" s="36">
         <v>1</v>
       </c>
-      <c r="B13" s="28" t="s">
-        <v>16</v>
-      </c>
-      <c r="C13" s="37">
+      <c r="B14" s="29" t="s">
+        <v>17</v>
+      </c>
+      <c r="C14" s="37">
         <v>8</v>
       </c>
-      <c r="D13" s="28">
+      <c r="D14" s="29">
         <v>4</v>
       </c>
-      <c r="E13" s="31">
+      <c r="E14" s="32">
         <v>5.5</v>
       </c>
-      <c r="G13" s="10"/>
-      <c r="H13" s="32"/>
-      <c r="I13" s="32"/>
-      <c r="J13" s="32"/>
-      <c r="K13" s="32"/>
-    </row>
-    <row r="14" ht="16.5" spans="1:11">
-      <c r="A14" s="38"/>
-      <c r="B14" s="21"/>
-      <c r="C14" s="21"/>
-      <c r="D14" s="21"/>
-      <c r="E14" s="10"/>
-      <c r="F14" s="10"/>
-      <c r="G14" s="39"/>
-      <c r="H14" s="10"/>
-      <c r="I14" s="32"/>
-      <c r="J14" s="32"/>
-      <c r="K14" s="78"/>
-    </row>
-    <row r="15" ht="15.75" spans="1:11">
-      <c r="A15" s="40"/>
-      <c r="B15" s="41"/>
-      <c r="C15" s="42" t="s">
-        <v>17</v>
-      </c>
-      <c r="D15" s="43"/>
-      <c r="E15" s="43"/>
-      <c r="F15" s="44"/>
-      <c r="K15" s="10"/>
-    </row>
-    <row r="16" ht="16.5" spans="1:12">
-      <c r="A16" s="45" t="s">
+      <c r="G14" s="10"/>
+      <c r="H14" s="20"/>
+      <c r="I14" s="20"/>
+      <c r="J14" s="20"/>
+      <c r="K14" s="20"/>
+    </row>
+    <row r="15" ht="16.5" spans="1:11">
+      <c r="A15" s="38"/>
+      <c r="B15" s="21"/>
+      <c r="C15" s="21"/>
+      <c r="D15" s="21"/>
+      <c r="E15" s="10"/>
+      <c r="F15" s="10"/>
+      <c r="G15" s="27"/>
+      <c r="H15" s="10"/>
+      <c r="I15" s="20"/>
+      <c r="J15" s="20"/>
+      <c r="K15" s="39"/>
+    </row>
+    <row r="16" ht="15.75" spans="1:11">
+      <c r="A16" s="40"/>
+      <c r="B16" s="41"/>
+      <c r="C16" s="42" t="s">
         <v>18</v>
       </c>
-      <c r="B16" s="46" t="s">
+      <c r="D16" s="43"/>
+      <c r="E16" s="43"/>
+      <c r="F16" s="44"/>
+      <c r="K16" s="10"/>
+    </row>
+    <row r="17" ht="16.5" spans="1:12">
+      <c r="A17" s="45" t="s">
+        <v>19</v>
+      </c>
+      <c r="B17" s="46" t="s">
         <v>1</v>
       </c>
-      <c r="C16" s="47" t="s">
-        <v>19</v>
-      </c>
-      <c r="D16" s="48"/>
-      <c r="E16" s="48"/>
-      <c r="F16" s="49"/>
-      <c r="K16" s="79"/>
-      <c r="L16" s="79"/>
-    </row>
-    <row r="17" spans="1:11">
-      <c r="A17" s="50">
+      <c r="C17" s="47" t="s">
+        <v>20</v>
+      </c>
+      <c r="D17" s="48"/>
+      <c r="E17" s="48"/>
+      <c r="F17" s="49"/>
+      <c r="K17" s="50"/>
+      <c r="L17" s="50"/>
+    </row>
+    <row r="18" spans="1:12">
+      <c r="A18" s="51">
         <v>0</v>
-      </c>
-      <c r="B17" s="10">
-        <v>0</v>
-      </c>
-      <c r="C17" s="50" t="s">
-        <v>20</v>
-      </c>
-      <c r="D17" s="10" t="s">
-        <v>21</v>
-      </c>
-      <c r="E17" s="41"/>
-      <c r="F17" s="51"/>
-      <c r="K17" s="10"/>
-    </row>
-    <row r="18" spans="1:11">
-      <c r="A18" s="50">
-        <v>0.5</v>
       </c>
       <c r="B18" s="10">
         <v>0</v>
       </c>
-      <c r="C18" s="52" t="s">
+      <c r="C18" s="51" t="s">
+        <v>21</v>
+      </c>
+      <c r="D18" s="10" t="s">
         <v>22</v>
       </c>
-      <c r="D18" s="53" t="s">
-        <v>23</v>
-      </c>
-      <c r="E18" s="10"/>
-      <c r="F18" s="54"/>
+      <c r="E18" s="41"/>
+      <c r="F18" s="52"/>
       <c r="K18" s="10"/>
     </row>
-    <row r="19" spans="1:11">
-      <c r="A19" s="50">
-        <v>1</v>
+    <row r="19" spans="1:12">
+      <c r="A19" s="51">
+        <v>0.5</v>
       </c>
       <c r="B19" s="10">
         <v>0</v>
       </c>
-      <c r="C19" s="55"/>
-      <c r="D19" s="56"/>
-      <c r="E19" s="56"/>
-      <c r="F19" s="57"/>
+      <c r="C19" s="53" t="s">
+        <v>23</v>
+      </c>
+      <c r="D19" s="54" t="s">
+        <v>24</v>
+      </c>
+      <c r="E19" s="10"/>
+      <c r="F19" s="55"/>
       <c r="K19" s="10"/>
     </row>
-    <row r="20" spans="1:6">
-      <c r="A20" s="50">
+    <row r="20" spans="1:12">
+      <c r="A20" s="51">
+        <v>1</v>
+      </c>
+      <c r="B20" s="10">
         <v>0</v>
       </c>
-      <c r="B20" s="10">
-        <v>1</v>
-      </c>
-      <c r="C20" s="50" t="s">
-        <v>24</v>
-      </c>
-      <c r="D20" s="10" t="s">
-        <v>25</v>
-      </c>
-      <c r="E20" s="10" t="s">
-        <v>26</v>
-      </c>
-      <c r="F20" s="54" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="21" spans="1:6">
-      <c r="A21" s="50">
-        <v>0.5</v>
+      <c r="C20" s="56"/>
+      <c r="D20" s="57"/>
+      <c r="E20" s="57"/>
+      <c r="F20" s="58"/>
+      <c r="K20" s="10"/>
+    </row>
+    <row r="21" spans="1:12">
+      <c r="A21" s="51">
+        <v>0</v>
       </c>
       <c r="B21" s="10">
         <v>1</v>
       </c>
-      <c r="C21" s="50" t="s">
+      <c r="C21" s="51" t="s">
+        <v>25</v>
+      </c>
+      <c r="D21" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="E21" s="10" t="s">
+        <v>27</v>
+      </c>
+      <c r="F21" s="55" t="s">
         <v>28</v>
       </c>
-      <c r="D21" s="10" t="s">
+    </row>
+    <row r="22" spans="1:12">
+      <c r="A22" s="51">
+        <v>0.5</v>
+      </c>
+      <c r="B22" s="10">
+        <v>1</v>
+      </c>
+      <c r="C22" s="51" t="s">
         <v>29</v>
       </c>
-      <c r="E21" s="10"/>
-      <c r="F21" s="54"/>
-    </row>
-    <row r="22" ht="15.75" spans="1:6">
-      <c r="A22" s="58">
+      <c r="D22" s="10" t="s">
+        <v>30</v>
+      </c>
+      <c r="E22" s="10"/>
+      <c r="F22" s="55"/>
+    </row>
+    <row r="23" ht="15.75" spans="1:12">
+      <c r="A23" s="59">
         <v>1</v>
       </c>
-      <c r="B22" s="59">
+      <c r="B23" s="60">
         <v>1</v>
       </c>
-      <c r="C22" s="58"/>
-      <c r="D22" s="59"/>
-      <c r="E22" s="59"/>
-      <c r="F22" s="60"/>
-    </row>
-    <row r="23" ht="15.75" spans="1:11">
-      <c r="A23" s="33">
+      <c r="C23" s="59"/>
+      <c r="D23" s="60"/>
+      <c r="E23" s="60"/>
+      <c r="F23" s="61"/>
+    </row>
+    <row r="24" ht="15.75" spans="1:12">
+      <c r="A24" s="33">
         <v>1</v>
       </c>
-      <c r="B23" s="61" t="s">
-        <v>15</v>
-      </c>
-      <c r="C23" s="40" t="s">
-        <v>30</v>
-      </c>
-      <c r="D23" s="62"/>
-      <c r="E23" s="62"/>
-      <c r="F23" s="61"/>
-      <c r="K23" s="21"/>
-    </row>
-    <row r="24" ht="16.5" spans="1:11">
-      <c r="A24" s="36">
+      <c r="B24" s="62" t="s">
+        <v>16</v>
+      </c>
+      <c r="C24" s="40" t="s">
+        <v>31</v>
+      </c>
+      <c r="D24" s="63"/>
+      <c r="E24" s="63"/>
+      <c r="F24" s="62"/>
+      <c r="K24" s="21"/>
+    </row>
+    <row r="25" ht="16.5" spans="1:12">
+      <c r="A25" s="36">
         <v>1</v>
       </c>
-      <c r="B24" s="63" t="s">
-        <v>16</v>
-      </c>
-      <c r="C24" s="36" t="s">
-        <v>31</v>
-      </c>
-      <c r="D24" s="29" t="s">
+      <c r="B25" s="64" t="s">
+        <v>17</v>
+      </c>
+      <c r="C25" s="36" t="s">
         <v>32</v>
       </c>
-      <c r="E24" s="29"/>
-      <c r="F24" s="63"/>
-      <c r="K24" s="21"/>
-    </row>
-    <row r="25" ht="15.75" spans="1:11">
-      <c r="A25" s="21"/>
-      <c r="B25" s="21"/>
-      <c r="C25" s="21"/>
-      <c r="D25" s="21"/>
-      <c r="E25" s="21"/>
-      <c r="F25" s="21"/>
-      <c r="G25" s="21"/>
-      <c r="H25" s="21"/>
-      <c r="I25" s="10"/>
-      <c r="J25" s="10"/>
+      <c r="D25" s="30" t="s">
+        <v>33</v>
+      </c>
+      <c r="E25" s="30"/>
+      <c r="F25" s="64"/>
       <c r="K25" s="21"/>
     </row>
-    <row r="26" ht="16.5" spans="1:11">
+    <row r="26" ht="15.75" spans="1:12">
       <c r="A26" s="21"/>
       <c r="B26" s="21"/>
       <c r="C26" s="21"/>
@@ -2497,805 +2549,805 @@
       <c r="J26" s="10"/>
       <c r="K26" s="21"/>
     </row>
-    <row r="27" ht="16.5" spans="1:11">
+    <row r="27" ht="16.5" spans="1:12">
       <c r="A27" s="21"/>
-      <c r="C27" s="33" t="s">
-        <v>33</v>
-      </c>
-      <c r="D27" s="61"/>
+      <c r="B27" s="21"/>
+      <c r="C27" s="21"/>
+      <c r="D27" s="21"/>
+      <c r="E27" s="21"/>
       <c r="F27" s="21"/>
       <c r="G27" s="21"/>
-      <c r="H27" s="38"/>
-      <c r="I27" s="21"/>
+      <c r="H27" s="21"/>
+      <c r="I27" s="10"/>
       <c r="J27" s="10"/>
       <c r="K27" s="21"/>
     </row>
-    <row r="28" ht="16.5" spans="1:11">
-      <c r="A28" s="38"/>
-      <c r="B28" s="40" t="s">
+    <row r="28" ht="16.5" spans="1:12">
+      <c r="A28" s="21"/>
+      <c r="C28" s="33" t="s">
         <v>34</v>
       </c>
-      <c r="C28" s="41" t="s">
+      <c r="D28" s="62"/>
+      <c r="F28" s="21"/>
+      <c r="G28" s="21"/>
+      <c r="H28" s="38"/>
+      <c r="I28" s="21"/>
+      <c r="J28" s="10"/>
+      <c r="K28" s="21"/>
+    </row>
+    <row r="29" ht="16.5" spans="1:12">
+      <c r="A29" s="38"/>
+      <c r="B29" s="40" t="s">
         <v>35</v>
       </c>
-      <c r="D28" s="41" t="s">
+      <c r="C29" s="41" t="s">
         <v>36</v>
       </c>
-      <c r="E28" s="61" t="s">
+      <c r="D29" s="41" t="s">
         <v>37</v>
       </c>
-      <c r="G28" s="10"/>
-      <c r="H28" s="10" t="s">
+      <c r="E29" s="62" t="s">
         <v>38</v>
       </c>
-      <c r="I28" s="10"/>
-      <c r="J28" s="10"/>
-      <c r="K28" s="80"/>
-    </row>
-    <row r="29" ht="15.75" spans="1:11">
-      <c r="A29" s="38"/>
-      <c r="B29" s="50">
+      <c r="G29" s="10"/>
+      <c r="H29" s="10" t="s">
+        <v>39</v>
+      </c>
+      <c r="I29" s="10"/>
+      <c r="J29" s="10"/>
+      <c r="K29" s="65"/>
+    </row>
+    <row r="30" ht="15.75" spans="1:12">
+      <c r="A30" s="38"/>
+      <c r="B30" s="51">
         <v>25</v>
       </c>
-      <c r="C29" s="10">
+      <c r="C30" s="10">
         <v>7</v>
       </c>
-      <c r="D29" s="10">
+      <c r="D30" s="10">
         <v>1.5</v>
       </c>
-      <c r="E29" s="64">
+      <c r="E30" s="66">
         <v>10</v>
       </c>
-      <c r="G29" s="40" t="s">
-        <v>39</v>
-      </c>
-      <c r="H29" s="13" t="s">
+      <c r="G30" s="40" t="s">
         <v>40</v>
       </c>
-      <c r="I29" s="13" t="s">
+      <c r="H30" s="13" t="s">
         <v>41</v>
       </c>
-      <c r="K29" s="21"/>
-    </row>
-    <row r="30" ht="15.75" spans="1:11">
-      <c r="A30" s="38"/>
-      <c r="B30" s="50">
+      <c r="I30" s="13" t="s">
+        <v>42</v>
+      </c>
+      <c r="K30" s="21"/>
+    </row>
+    <row r="31" ht="15.75" spans="1:12">
+      <c r="A31" s="38"/>
+      <c r="B31" s="51">
         <v>50</v>
       </c>
-      <c r="C30" s="10">
+      <c r="C31" s="10">
         <v>14</v>
       </c>
-      <c r="D30" s="10">
+      <c r="D31" s="10">
         <v>2.5</v>
       </c>
-      <c r="E30" s="64">
+      <c r="E31" s="66">
         <v>10</v>
       </c>
-      <c r="G30" s="50">
+      <c r="G31" s="51">
         <v>1</v>
       </c>
-      <c r="H30" s="18">
+      <c r="H31" s="17">
         <v>21.5</v>
       </c>
-      <c r="I30" s="18">
+      <c r="I31" s="17">
         <v>7</v>
       </c>
-      <c r="K30" s="21"/>
-    </row>
-    <row r="31" ht="15.75" spans="1:11">
-      <c r="A31" s="38"/>
-      <c r="B31" s="50">
+      <c r="K31" s="21"/>
+    </row>
+    <row r="32" ht="15.75" spans="1:12">
+      <c r="A32" s="38"/>
+      <c r="B32" s="51">
         <v>75</v>
       </c>
-      <c r="C31" s="10">
+      <c r="C32" s="10">
         <v>20</v>
       </c>
-      <c r="D31" s="10">
+      <c r="D32" s="10">
         <v>3.5</v>
       </c>
-      <c r="E31" s="64">
+      <c r="E32" s="66">
         <v>10</v>
       </c>
-      <c r="G31" s="50">
+      <c r="G32" s="51">
         <v>2</v>
       </c>
-      <c r="H31" s="18">
+      <c r="H32" s="17">
         <v>25.5</v>
       </c>
-      <c r="I31" s="18">
+      <c r="I32" s="17">
         <v>9</v>
       </c>
-      <c r="K31" s="21"/>
-    </row>
-    <row r="32" ht="15.75" spans="1:11">
-      <c r="A32" s="38" t="s">
-        <v>42</v>
-      </c>
-      <c r="B32" s="65">
-        <v>100</v>
-      </c>
-      <c r="C32" s="10">
-        <v>25</v>
-      </c>
-      <c r="D32" s="21">
-        <v>5</v>
-      </c>
-      <c r="E32" s="64">
-        <v>10</v>
-      </c>
-      <c r="G32" s="50">
-        <v>3</v>
-      </c>
-      <c r="H32" s="18">
-        <v>29.5</v>
-      </c>
-      <c r="I32" s="18">
-        <v>11</v>
-      </c>
       <c r="K32" s="21"/>
     </row>
-    <row r="33" ht="15.75" spans="1:11">
+    <row r="33" ht="15.75" spans="1:13">
       <c r="A33" s="38" t="s">
         <v>43</v>
       </c>
-      <c r="B33" s="50">
+      <c r="B33" s="67">
+        <v>100</v>
+      </c>
+      <c r="C33" s="10">
+        <v>25</v>
+      </c>
+      <c r="D33" s="21">
+        <v>5</v>
+      </c>
+      <c r="E33" s="66">
+        <v>10</v>
+      </c>
+      <c r="G33" s="51">
+        <v>3</v>
+      </c>
+      <c r="H33" s="17">
+        <v>29.5</v>
+      </c>
+      <c r="I33" s="17">
+        <v>11</v>
+      </c>
+      <c r="K33" s="21"/>
+    </row>
+    <row r="34" ht="15.75" spans="1:13">
+      <c r="A34" s="38" t="s">
+        <v>44</v>
+      </c>
+      <c r="B34" s="51">
         <v>125</v>
       </c>
-      <c r="C33" s="10">
+      <c r="C34" s="10">
         <v>30</v>
       </c>
-      <c r="D33" s="21">
+      <c r="D34" s="21">
         <v>6.5</v>
       </c>
-      <c r="E33" s="64">
+      <c r="E34" s="66">
         <v>10</v>
       </c>
-      <c r="G33" s="50">
+      <c r="G34" s="51">
         <v>4</v>
       </c>
-      <c r="H33" s="18">
+      <c r="H34" s="17">
         <v>33.5</v>
       </c>
-      <c r="I33" s="18">
+      <c r="I34" s="17">
         <v>13</v>
       </c>
-      <c r="K33" s="21"/>
-    </row>
-    <row r="34" ht="15.75" spans="1:11">
-      <c r="A34" s="38"/>
-      <c r="B34" s="50">
+      <c r="K34" s="21"/>
+    </row>
+    <row r="35" ht="15.75" spans="1:13">
+      <c r="A35" s="38"/>
+      <c r="B35" s="51">
         <v>150</v>
       </c>
-      <c r="C34" s="10">
+      <c r="C35" s="10">
         <v>35</v>
       </c>
-      <c r="D34" s="21">
+      <c r="D35" s="21">
         <v>7.5</v>
       </c>
-      <c r="E34" s="64">
+      <c r="E35" s="66">
         <v>10</v>
       </c>
-      <c r="G34" s="50">
+      <c r="G35" s="51">
         <v>5</v>
       </c>
-      <c r="H34" s="18">
+      <c r="H35" s="17">
         <v>37.5</v>
       </c>
-      <c r="I34" s="18">
+      <c r="I35" s="17">
         <v>15</v>
       </c>
-      <c r="K34" s="21"/>
-    </row>
-    <row r="35" ht="15.75" spans="1:11">
-      <c r="A35" s="38" t="s">
-        <v>44</v>
-      </c>
-      <c r="B35" s="50">
+      <c r="K35" s="21"/>
+    </row>
+    <row r="36" ht="15.75" spans="1:13">
+      <c r="A36" s="38" t="s">
+        <v>45</v>
+      </c>
+      <c r="B36" s="51">
         <v>175</v>
       </c>
-      <c r="C35" s="10">
+      <c r="C36" s="10">
         <v>40</v>
       </c>
-      <c r="D35" s="21">
+      <c r="D36" s="21">
         <v>8.5</v>
       </c>
-      <c r="E35" s="64">
+      <c r="E36" s="66">
         <v>10</v>
       </c>
-      <c r="F35" t="s">
+      <c r="F36" t="s">
+        <v>46</v>
+      </c>
+      <c r="G36" s="51">
+        <v>6</v>
+      </c>
+      <c r="H36" s="17">
+        <v>41.5</v>
+      </c>
+      <c r="I36" s="17">
+        <v>17</v>
+      </c>
+      <c r="K36" s="21"/>
+    </row>
+    <row r="37" ht="15.75" spans="1:13">
+      <c r="A37" s="38" t="s">
+        <v>47</v>
+      </c>
+      <c r="B37" s="51">
+        <v>200</v>
+      </c>
+      <c r="C37" s="10">
         <v>45</v>
       </c>
-      <c r="G35" s="50">
-        <v>6</v>
-      </c>
-      <c r="H35" s="18">
-        <v>41.5</v>
-      </c>
-      <c r="I35" s="18">
-        <v>17</v>
-      </c>
-      <c r="K35" s="21"/>
-    </row>
-    <row r="36" ht="15.75" spans="1:11">
-      <c r="A36" s="38" t="s">
-        <v>46</v>
-      </c>
-      <c r="B36" s="50">
-        <v>200</v>
-      </c>
-      <c r="C36" s="10">
-        <v>45</v>
-      </c>
-      <c r="D36" s="21">
+      <c r="D37" s="21">
         <v>9.5</v>
       </c>
-      <c r="E36" s="64">
-        <v>11</v>
-      </c>
-      <c r="F36" t="s">
-        <v>47</v>
-      </c>
-      <c r="G36" s="50">
-        <v>7</v>
-      </c>
-      <c r="H36" s="18">
-        <v>45.5</v>
-      </c>
-      <c r="I36" s="18">
-        <v>19</v>
-      </c>
-      <c r="K36" s="21"/>
-    </row>
-    <row r="37" ht="15.75" spans="1:11">
-      <c r="A37" s="38"/>
-      <c r="B37" s="65">
-        <v>225</v>
-      </c>
-      <c r="C37" s="10">
-        <v>50</v>
-      </c>
-      <c r="D37" s="21">
-        <v>10.5</v>
-      </c>
-      <c r="E37" s="64">
+      <c r="E37" s="66">
         <v>11</v>
       </c>
       <c r="F37" t="s">
         <v>48</v>
       </c>
-      <c r="G37" s="50">
+      <c r="G37" s="51">
+        <v>7</v>
+      </c>
+      <c r="H37" s="17">
+        <v>45.5</v>
+      </c>
+      <c r="I37" s="17">
+        <v>19</v>
+      </c>
+      <c r="K37" s="21"/>
+    </row>
+    <row r="38" ht="15.75" spans="1:13">
+      <c r="A38" s="38"/>
+      <c r="B38" s="67">
+        <v>225</v>
+      </c>
+      <c r="C38" s="10">
+        <v>50</v>
+      </c>
+      <c r="D38" s="21">
+        <v>10.5</v>
+      </c>
+      <c r="E38" s="66">
+        <v>11</v>
+      </c>
+      <c r="F38" t="s">
+        <v>49</v>
+      </c>
+      <c r="G38" s="51">
         <v>8</v>
       </c>
-      <c r="H37" s="18">
+      <c r="H38" s="17">
         <v>49.5</v>
       </c>
-      <c r="I37" s="18">
+      <c r="I38" s="17">
         <v>21</v>
       </c>
-      <c r="K37" s="21"/>
-    </row>
-    <row r="38" ht="15.75" spans="1:11">
-      <c r="A38" s="38" t="s">
-        <v>49</v>
-      </c>
-      <c r="B38" s="50">
+      <c r="K38" s="21"/>
+    </row>
+    <row r="39" ht="15.75" spans="1:13">
+      <c r="A39" s="38" t="s">
+        <v>50</v>
+      </c>
+      <c r="B39" s="51">
         <v>250</v>
       </c>
-      <c r="C38" s="10">
+      <c r="C39" s="10">
         <v>55</v>
       </c>
-      <c r="D38" s="21">
+      <c r="D39" s="21">
         <v>11.5</v>
       </c>
-      <c r="E38" s="64">
+      <c r="E39" s="66">
         <v>11</v>
       </c>
-      <c r="F38" t="s">
-        <v>50</v>
-      </c>
-      <c r="G38" s="50">
+      <c r="F39" t="s">
+        <v>51</v>
+      </c>
+      <c r="G39" s="51">
         <v>9</v>
       </c>
-      <c r="H38" s="18">
+      <c r="H39" s="17">
         <v>53.5</v>
       </c>
-      <c r="I38" s="18">
+      <c r="I39" s="17">
         <v>23</v>
       </c>
-      <c r="K38" s="21"/>
-    </row>
-    <row r="39" ht="16.5" spans="1:11">
-      <c r="A39" s="38" t="s">
-        <v>51</v>
-      </c>
-      <c r="B39" s="50">
+      <c r="K39" s="21"/>
+    </row>
+    <row r="40" ht="16.5" spans="1:13">
+      <c r="A40" s="38" t="s">
+        <v>52</v>
+      </c>
+      <c r="B40" s="51">
         <v>275</v>
       </c>
-      <c r="C39" s="10">
+      <c r="C40" s="10">
         <v>60</v>
       </c>
-      <c r="D39" s="21">
+      <c r="D40" s="21">
         <v>12.5</v>
       </c>
-      <c r="E39" s="64">
+      <c r="E40" s="66">
         <v>11</v>
-      </c>
-      <c r="F39" t="s">
-        <v>52</v>
-      </c>
-      <c r="G39" s="58">
-        <v>10</v>
-      </c>
-      <c r="H39" s="31">
-        <v>57.5</v>
-      </c>
-      <c r="I39" s="31">
-        <v>25</v>
-      </c>
-      <c r="K39" s="21"/>
-    </row>
-    <row r="40" ht="16.5" spans="1:13">
-      <c r="A40" s="38"/>
-      <c r="B40" s="66">
-        <v>300</v>
-      </c>
-      <c r="C40" s="10">
-        <v>65</v>
-      </c>
-      <c r="D40" s="21">
-        <v>13.5</v>
-      </c>
-      <c r="E40" s="54">
-        <v>12</v>
       </c>
       <c r="F40" t="s">
         <v>53</v>
       </c>
-      <c r="G40" s="10"/>
-      <c r="H40" s="10"/>
-      <c r="I40" s="81"/>
-      <c r="J40" s="81"/>
-      <c r="K40" s="32"/>
-      <c r="M40" s="21"/>
+      <c r="G40" s="59">
+        <v>10</v>
+      </c>
+      <c r="H40" s="32">
+        <v>57.5</v>
+      </c>
+      <c r="I40" s="32">
+        <v>25</v>
+      </c>
+      <c r="K40" s="21"/>
     </row>
     <row r="41" ht="16.5" spans="1:13">
-      <c r="A41" s="67" t="s">
+      <c r="A41" s="38"/>
+      <c r="B41" s="68">
+        <v>300</v>
+      </c>
+      <c r="C41" s="10">
+        <v>65</v>
+      </c>
+      <c r="D41" s="21">
+        <v>13.5</v>
+      </c>
+      <c r="E41" s="55">
+        <v>12</v>
+      </c>
+      <c r="F41" t="s">
         <v>54</v>
       </c>
-      <c r="B41" s="66">
+      <c r="G41" s="10"/>
+      <c r="H41" s="10"/>
+      <c r="I41" s="69"/>
+      <c r="J41" s="69"/>
+      <c r="K41" s="20"/>
+      <c r="M41" s="21"/>
+    </row>
+    <row r="42" ht="16.5" spans="1:13">
+      <c r="A42" s="70" t="s">
+        <v>55</v>
+      </c>
+      <c r="B42" s="68">
         <v>325</v>
       </c>
-      <c r="C41" s="10">
+      <c r="C42" s="10">
         <v>70</v>
       </c>
-      <c r="D41" s="21">
+      <c r="D42" s="21">
         <v>14.5</v>
       </c>
-      <c r="E41" s="54">
+      <c r="E42" s="55">
         <v>12</v>
       </c>
-      <c r="G41" s="68" t="s">
-        <v>55</v>
-      </c>
-      <c r="H41" s="68" t="s">
+      <c r="G42" s="71" t="s">
         <v>56</v>
       </c>
-      <c r="I41" s="82" t="s">
+      <c r="H42" s="71" t="s">
         <v>57</v>
       </c>
-      <c r="J41" s="83" t="s">
+      <c r="I42" s="72" t="s">
         <v>58</v>
       </c>
-      <c r="M41" s="21"/>
-    </row>
-    <row r="42" ht="15.75" spans="1:13">
-      <c r="A42" s="67" t="s">
+      <c r="J42" s="73" t="s">
         <v>59</v>
       </c>
-      <c r="B42" s="50">
+      <c r="M42" s="21"/>
+    </row>
+    <row r="43" ht="15.75" spans="1:13">
+      <c r="A43" s="70" t="s">
+        <v>60</v>
+      </c>
+      <c r="B43" s="51">
         <v>350</v>
       </c>
-      <c r="C42" s="10">
+      <c r="C43" s="10">
         <v>75</v>
       </c>
-      <c r="D42" s="21">
+      <c r="D43" s="21">
         <v>15.5</v>
       </c>
-      <c r="E42" s="54">
+      <c r="E43" s="55">
         <v>12</v>
       </c>
-      <c r="G42" s="69" t="s">
-        <v>60</v>
-      </c>
-      <c r="H42" s="69">
+      <c r="G43" s="74" t="s">
+        <v>61</v>
+      </c>
+      <c r="H43" s="74">
         <v>16</v>
       </c>
-      <c r="I42" s="13">
+      <c r="I43" s="13">
         <v>8</v>
       </c>
-      <c r="J42" s="51">
-        <f>H42+2*I42</f>
-        <v>32</v>
-      </c>
-      <c r="M42" s="21"/>
-    </row>
-    <row r="43" ht="16.5" spans="1:10">
-      <c r="A43" s="67"/>
-      <c r="B43" s="36">
-        <v>375</v>
-      </c>
-      <c r="C43" s="59">
-        <v>80</v>
-      </c>
-      <c r="D43" s="59">
-        <v>10.5</v>
-      </c>
-      <c r="E43" s="60">
-        <v>12</v>
-      </c>
-      <c r="G43" s="50" t="s">
-        <v>61</v>
-      </c>
-      <c r="H43" s="50">
-        <v>18</v>
-      </c>
-      <c r="I43" s="18">
-        <v>7</v>
-      </c>
-      <c r="J43" s="54">
+      <c r="J43" s="52">
         <f>H43+2*I43</f>
         <v>32</v>
       </c>
-    </row>
-    <row r="44" ht="15.75" spans="1:10">
-      <c r="A44" s="38" t="s">
+      <c r="M43" s="21"/>
+    </row>
+    <row r="44" ht="16.5" spans="1:13">
+      <c r="A44" s="70"/>
+      <c r="B44" s="36">
+        <v>375</v>
+      </c>
+      <c r="C44" s="60">
+        <v>80</v>
+      </c>
+      <c r="D44" s="60">
+        <v>10.5</v>
+      </c>
+      <c r="E44" s="61">
+        <v>12</v>
+      </c>
+      <c r="G44" s="51" t="s">
         <v>62</v>
       </c>
-      <c r="B44" s="50">
+      <c r="H44" s="51">
+        <v>18</v>
+      </c>
+      <c r="I44" s="17">
+        <v>7</v>
+      </c>
+      <c r="J44" s="55">
+        <f>H44+2*I44</f>
+        <v>32</v>
+      </c>
+    </row>
+    <row r="45" ht="15.75" spans="1:13">
+      <c r="A45" s="38" t="s">
+        <v>63</v>
+      </c>
+      <c r="B45" s="51">
         <v>400</v>
       </c>
-      <c r="C44" s="10">
+      <c r="C45" s="10">
         <v>85</v>
       </c>
-      <c r="D44" s="10">
+      <c r="D45" s="10">
         <v>11</v>
       </c>
-      <c r="E44" s="54">
+      <c r="E45" s="55">
         <v>12</v>
       </c>
-      <c r="G44" s="50" t="s">
-        <v>63</v>
-      </c>
-      <c r="H44" s="50">
+      <c r="G45" s="51" t="s">
+        <v>64</v>
+      </c>
+      <c r="H45" s="51">
         <v>21</v>
       </c>
-      <c r="I44" s="18">
+      <c r="I45" s="17">
         <v>5</v>
       </c>
-      <c r="J44" s="54">
-        <f t="shared" ref="J44:J50" si="0">H44+2*I44</f>
+      <c r="J45" s="55">
+        <f t="shared" ref="J45:J51" si="0">H45+2*I45</f>
         <v>31</v>
       </c>
     </row>
-    <row r="45" ht="15.75" spans="1:10">
-      <c r="A45" s="38"/>
-      <c r="B45" s="50">
+    <row r="46" ht="15.75" spans="1:13">
+      <c r="A46" s="38"/>
+      <c r="B46" s="51">
         <v>425</v>
       </c>
-      <c r="C45" s="10">
+      <c r="C46" s="10">
         <v>90</v>
       </c>
-      <c r="D45" s="10" t="s">
-        <v>64</v>
-      </c>
-      <c r="E45" s="54">
+      <c r="D46" s="10" t="s">
+        <v>65</v>
+      </c>
+      <c r="E46" s="55">
         <v>12</v>
       </c>
-      <c r="G45" s="50" t="s">
-        <v>65</v>
-      </c>
-      <c r="H45" s="50">
+      <c r="G46" s="51" t="s">
+        <v>66</v>
+      </c>
+      <c r="H46" s="51">
         <v>22</v>
       </c>
-      <c r="I45" s="18">
+      <c r="I46" s="17">
         <v>5</v>
       </c>
-      <c r="J45" s="54">
+      <c r="J46" s="55">
         <f t="shared" si="0"/>
         <v>32</v>
       </c>
     </row>
-    <row r="46" ht="15.75" spans="1:10">
-      <c r="A46" s="38" t="s">
-        <v>66</v>
-      </c>
-      <c r="B46" s="50">
+    <row r="47" ht="15.75" spans="1:13">
+      <c r="A47" s="38" t="s">
+        <v>67</v>
+      </c>
+      <c r="B47" s="51">
         <v>450</v>
       </c>
-      <c r="C46" s="10">
+      <c r="C47" s="10">
         <v>95</v>
       </c>
-      <c r="D46" s="10" t="s">
-        <v>67</v>
-      </c>
-      <c r="E46" s="54">
+      <c r="D47" s="10" t="s">
+        <v>68</v>
+      </c>
+      <c r="E47" s="55">
         <v>12</v>
       </c>
-      <c r="G46" s="70" t="s">
-        <v>68</v>
-      </c>
-      <c r="H46" s="70">
+      <c r="G47" s="75" t="s">
+        <v>69</v>
+      </c>
+      <c r="H47" s="75">
         <v>16</v>
       </c>
-      <c r="I46" s="18">
+      <c r="I47" s="17">
         <v>8</v>
       </c>
-      <c r="J46" s="54">
+      <c r="J47" s="55">
         <f t="shared" si="0"/>
         <v>32</v>
       </c>
     </row>
-    <row r="47" ht="15.75" spans="1:10">
-      <c r="A47" s="38"/>
-      <c r="B47" s="50">
+    <row r="48" ht="15.75" spans="1:13">
+      <c r="A48" s="38"/>
+      <c r="B48" s="51">
         <v>475</v>
       </c>
-      <c r="C47" s="10">
+      <c r="C48" s="10">
         <v>100</v>
       </c>
-      <c r="D47" s="10" t="s">
-        <v>69</v>
-      </c>
-      <c r="E47" s="54">
+      <c r="D48" s="10" t="s">
+        <v>70</v>
+      </c>
+      <c r="E48" s="55">
         <v>12</v>
       </c>
-      <c r="G47" s="50" t="s">
-        <v>70</v>
-      </c>
-      <c r="H47" s="50">
+      <c r="G48" s="51" t="s">
+        <v>71</v>
+      </c>
+      <c r="H48" s="51">
         <v>14</v>
       </c>
-      <c r="I47" s="18">
+      <c r="I48" s="17">
         <v>9</v>
       </c>
-      <c r="J47" s="54">
+      <c r="J48" s="55">
         <f t="shared" si="0"/>
         <v>32</v>
       </c>
     </row>
-    <row r="48" ht="15.75" spans="2:10">
-      <c r="B48" s="65">
+    <row r="49" ht="15.75" spans="1:14">
+      <c r="B49" s="67">
         <v>500</v>
       </c>
-      <c r="C48" s="10">
+      <c r="C49" s="10">
         <v>105</v>
       </c>
-      <c r="D48" s="66" t="s">
-        <v>71</v>
-      </c>
-      <c r="E48" s="54">
+      <c r="D49" s="68" t="s">
+        <v>72</v>
+      </c>
+      <c r="E49" s="55">
         <v>12</v>
       </c>
-      <c r="G48" s="50" t="s">
-        <v>72</v>
-      </c>
-      <c r="H48" s="50">
+      <c r="G49" s="51" t="s">
+        <v>73</v>
+      </c>
+      <c r="H49" s="51">
         <v>20</v>
       </c>
-      <c r="I48" s="18">
+      <c r="I49" s="17">
         <v>6</v>
       </c>
-      <c r="J48" s="54">
+      <c r="J49" s="55">
         <f t="shared" si="0"/>
         <v>32</v>
       </c>
     </row>
-    <row r="49" ht="15.75" spans="1:10">
-      <c r="A49" s="38"/>
-      <c r="B49" s="65">
+    <row r="50" ht="15.75" spans="1:14">
+      <c r="A50" s="38"/>
+      <c r="B50" s="67">
         <v>600</v>
       </c>
-      <c r="C49" s="66"/>
-      <c r="D49" s="66">
+      <c r="C50" s="68"/>
+      <c r="D50" s="68">
         <v>14.5</v>
       </c>
-      <c r="E49" s="54">
+      <c r="E50" s="55">
         <v>13</v>
       </c>
-      <c r="G49" s="50" t="s">
-        <v>73</v>
-      </c>
-      <c r="H49" s="50">
+      <c r="G50" s="51" t="s">
+        <v>74</v>
+      </c>
+      <c r="H50" s="51">
         <v>17</v>
       </c>
-      <c r="I49" s="18">
+      <c r="I50" s="17">
         <v>4</v>
       </c>
-      <c r="J49" s="54">
+      <c r="J50" s="55">
         <f t="shared" si="0"/>
         <v>25</v>
       </c>
     </row>
-    <row r="50" ht="16.5" spans="2:10">
-      <c r="B50" s="65">
+    <row r="51" ht="16.5" spans="1:14">
+      <c r="B51" s="67">
         <v>750</v>
       </c>
-      <c r="C50" s="66"/>
-      <c r="D50" s="66">
+      <c r="C51" s="68"/>
+      <c r="D51" s="68">
         <v>15</v>
       </c>
-      <c r="E50" s="54">
+      <c r="E51" s="55">
         <v>13</v>
       </c>
-      <c r="G50" s="58" t="s">
-        <v>74</v>
-      </c>
-      <c r="H50" s="58">
+      <c r="G51" s="59" t="s">
+        <v>75</v>
+      </c>
+      <c r="H51" s="59">
         <v>26</v>
       </c>
-      <c r="I50" s="31">
+      <c r="I51" s="32">
         <v>3</v>
       </c>
-      <c r="J50" s="60">
+      <c r="J51" s="61">
         <f t="shared" si="0"/>
         <v>32</v>
       </c>
     </row>
-    <row r="51" ht="16.5" spans="2:9">
-      <c r="B51" s="36">
+    <row r="52" ht="16.5" spans="1:14">
+      <c r="B52" s="36">
         <v>1000</v>
       </c>
-      <c r="C51" s="59"/>
-      <c r="D51" s="59">
+      <c r="C52" s="60"/>
+      <c r="D52" s="60">
         <v>15.5</v>
       </c>
-      <c r="E51" s="60">
+      <c r="E52" s="61">
         <v>13</v>
       </c>
-      <c r="H51" s="10"/>
-      <c r="I51" s="10"/>
-    </row>
-    <row r="52" spans="7:9">
-      <c r="G52" s="10"/>
       <c r="H52" s="10"/>
       <c r="I52" s="10"/>
     </row>
-    <row r="53" ht="15.75" spans="7:9">
+    <row r="53" spans="1:14">
       <c r="G53" s="10"/>
       <c r="H53" s="10"/>
       <c r="I53" s="10"/>
     </row>
-    <row r="54" ht="75.75" spans="1:10">
-      <c r="A54">
+    <row r="54" ht="15.75" spans="1:14">
+      <c r="G54" s="10"/>
+      <c r="H54" s="10"/>
+      <c r="I54" s="10"/>
+    </row>
+    <row r="55" ht="75.75" spans="1:14">
+      <c r="A55">
         <f>147*2*0.8</f>
         <v>235.2</v>
       </c>
-      <c r="C54" s="71" t="s">
-        <v>75</v>
-      </c>
-      <c r="D54" s="71" t="s">
+      <c r="C55" s="76" t="s">
         <v>76</v>
       </c>
-      <c r="E54" s="71" t="s">
+      <c r="D55" s="76" t="s">
         <v>77</v>
       </c>
-      <c r="G54" s="10"/>
-      <c r="H54" s="72" t="s">
+      <c r="E55" s="76" t="s">
         <v>78</v>
       </c>
-      <c r="I54" t="s">
+      <c r="G55" s="10"/>
+      <c r="H55" s="77" t="s">
         <v>79</v>
       </c>
-      <c r="J54" s="21"/>
-    </row>
-    <row r="55" ht="90.75" spans="3:10">
-      <c r="C55" s="71" t="s">
+      <c r="I55" t="s">
         <v>80</v>
       </c>
-      <c r="E55" s="10"/>
-      <c r="F55" s="10"/>
-      <c r="G55" s="10"/>
-      <c r="H55" s="10" t="s">
+      <c r="J55" s="21"/>
+    </row>
+    <row r="56" ht="90.75" spans="1:14">
+      <c r="C56" s="76" t="s">
         <v>81</v>
       </c>
-      <c r="I55" t="s">
-        <v>82</v>
-      </c>
-      <c r="J55" s="10" t="s">
-        <v>83</v>
-      </c>
-    </row>
-    <row r="56" spans="5:10">
-      <c r="E56" s="73"/>
+      <c r="E56" s="10"/>
       <c r="F56" s="10"/>
       <c r="G56" s="10"/>
       <c r="H56" s="10" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="I56" t="s">
+        <v>83</v>
+      </c>
+      <c r="J56" s="10" t="s">
         <v>84</v>
       </c>
-      <c r="J56" s="10" t="s">
-        <v>83</v>
-      </c>
-    </row>
-    <row r="57" spans="3:10">
-      <c r="C57" s="10"/>
-      <c r="E57" s="10"/>
+    </row>
+    <row r="57" spans="1:14">
+      <c r="E57" s="78"/>
       <c r="F57" s="10"/>
       <c r="G57" s="10"/>
       <c r="H57" s="10" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="I57" t="s">
         <v>85</v>
       </c>
       <c r="J57" s="10" t="s">
-        <v>86</v>
-      </c>
-    </row>
-    <row r="58" ht="13" customHeight="1" spans="5:10">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="58" spans="1:14">
+      <c r="C58" s="10"/>
       <c r="E58" s="10"/>
       <c r="F58" s="10"/>
       <c r="G58" s="10"/>
       <c r="H58" s="10" t="s">
+        <v>82</v>
+      </c>
+      <c r="I58" t="s">
+        <v>86</v>
+      </c>
+      <c r="J58" s="10" t="s">
         <v>87</v>
       </c>
-      <c r="I58" s="72" t="s">
-        <v>88</v>
-      </c>
-      <c r="J58" s="10" t="s">
-        <v>86</v>
-      </c>
-    </row>
-    <row r="59" spans="5:10">
+    </row>
+    <row r="59" ht="13" customHeight="1" spans="1:14">
       <c r="E59" s="10"/>
       <c r="F59" s="10"/>
       <c r="G59" s="10"/>
       <c r="H59" s="10" t="s">
+        <v>88</v>
+      </c>
+      <c r="I59" s="77" t="s">
         <v>89</v>
       </c>
-      <c r="I59" s="72" t="s">
+      <c r="J59" s="10" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="60" spans="1:14">
+      <c r="E60" s="10"/>
+      <c r="F60" s="10"/>
+      <c r="G60" s="10"/>
+      <c r="H60" s="10" t="s">
         <v>90</v>
       </c>
-      <c r="J59" s="10" t="s">
+      <c r="I60" s="77" t="s">
         <v>91</v>
       </c>
-    </row>
-    <row r="60" ht="15.75" spans="1:14">
-      <c r="A60" s="74"/>
-      <c r="B60" s="75"/>
-      <c r="C60" s="76"/>
-      <c r="D60" s="76"/>
-      <c r="E60" s="21"/>
-      <c r="F60" s="21"/>
-      <c r="G60" s="21"/>
-      <c r="H60" s="21"/>
-      <c r="I60" s="21"/>
-      <c r="J60" s="21"/>
-      <c r="K60" s="21"/>
-      <c r="M60" s="10"/>
-      <c r="N60" s="10"/>
-    </row>
-    <row r="61" spans="1:14">
-      <c r="A61" s="10"/>
-      <c r="F61" s="10"/>
-      <c r="G61" s="10"/>
-      <c r="H61" s="10"/>
-      <c r="I61" s="10"/>
-      <c r="J61" s="10"/>
-      <c r="K61" s="10"/>
+      <c r="J60" s="10" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="61" ht="15.75" spans="1:14">
+      <c r="A61" s="79"/>
+      <c r="B61" s="80"/>
+      <c r="C61" s="81"/>
+      <c r="D61" s="81"/>
+      <c r="E61" s="21"/>
+      <c r="F61" s="21"/>
+      <c r="G61" s="21"/>
+      <c r="H61" s="21"/>
+      <c r="I61" s="21"/>
+      <c r="J61" s="21"/>
+      <c r="K61" s="21"/>
       <c r="M61" s="10"/>
       <c r="N61" s="10"/>
     </row>
     <row r="62" spans="1:14">
       <c r="A62" s="10"/>
       <c r="F62" s="10"/>
-      <c r="G62" s="77" t="s">
-        <v>60</v>
-      </c>
-      <c r="H62" s="77"/>
-      <c r="I62" s="77"/>
+      <c r="G62" s="10"/>
+      <c r="H62" s="10"/>
+      <c r="I62" s="10"/>
       <c r="J62" s="10"/>
       <c r="K62" s="10"/>
       <c r="M62" s="10"/>
@@ -3304,14 +3356,13 @@
     <row r="63" spans="1:14">
       <c r="A63" s="10"/>
       <c r="F63" s="10"/>
-      <c r="G63" s="10" t="s">
+      <c r="G63" s="82" t="s">
         <v>61</v>
       </c>
-      <c r="H63" s="10"/>
-      <c r="I63" s="10"/>
+      <c r="H63" s="82"/>
+      <c r="I63" s="82"/>
       <c r="J63" s="10"/>
       <c r="K63" s="10"/>
-      <c r="L63" s="10"/>
       <c r="M63" s="10"/>
       <c r="N63" s="10"/>
     </row>
@@ -3319,7 +3370,7 @@
       <c r="A64" s="10"/>
       <c r="F64" s="10"/>
       <c r="G64" s="10" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="H64" s="10"/>
       <c r="I64" s="10"/>
@@ -3333,39 +3384,40 @@
       <c r="A65" s="10"/>
       <c r="F65" s="10"/>
       <c r="G65" s="10" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="H65" s="10"/>
       <c r="I65" s="10"/>
       <c r="J65" s="10"/>
       <c r="K65" s="10"/>
+      <c r="L65" s="10"/>
       <c r="M65" s="10"/>
       <c r="N65" s="10"/>
     </row>
-    <row r="66" ht="15.75" spans="1:14">
-      <c r="A66" s="74"/>
+    <row r="66" spans="1:14">
+      <c r="A66" s="10"/>
       <c r="F66" s="10"/>
-      <c r="G66" s="84" t="s">
-        <v>68</v>
-      </c>
-      <c r="H66" s="84"/>
-      <c r="I66" s="84"/>
-      <c r="J66" s="86"/>
-      <c r="K66" s="86"/>
-      <c r="L66" s="86"/>
+      <c r="G66" s="10" t="s">
+        <v>66</v>
+      </c>
+      <c r="H66" s="10"/>
+      <c r="I66" s="10"/>
+      <c r="J66" s="10"/>
+      <c r="K66" s="10"/>
       <c r="M66" s="10"/>
       <c r="N66" s="10"/>
     </row>
-    <row r="67" spans="1:14">
-      <c r="A67" s="10"/>
+    <row r="67" ht="15.75" spans="1:14">
+      <c r="A67" s="79"/>
       <c r="F67" s="10"/>
-      <c r="G67" s="10" t="s">
-        <v>70</v>
-      </c>
-      <c r="H67" s="10"/>
-      <c r="I67" s="10"/>
-      <c r="J67" s="10"/>
-      <c r="K67" s="10"/>
+      <c r="G67" s="83" t="s">
+        <v>69</v>
+      </c>
+      <c r="H67" s="83"/>
+      <c r="I67" s="83"/>
+      <c r="J67" s="84"/>
+      <c r="K67" s="84"/>
+      <c r="L67" s="84"/>
       <c r="M67" s="10"/>
       <c r="N67" s="10"/>
     </row>
@@ -3373,13 +3425,12 @@
       <c r="A68" s="10"/>
       <c r="F68" s="10"/>
       <c r="G68" s="10" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="H68" s="10"/>
       <c r="I68" s="10"/>
       <c r="J68" s="10"/>
       <c r="K68" s="10"/>
-      <c r="L68" s="10"/>
       <c r="M68" s="10"/>
       <c r="N68" s="10"/>
     </row>
@@ -3387,7 +3438,7 @@
       <c r="A69" s="10"/>
       <c r="F69" s="10"/>
       <c r="G69" s="10" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="H69" s="10"/>
       <c r="I69" s="10"/>
@@ -3397,27 +3448,32 @@
       <c r="M69" s="10"/>
       <c r="N69" s="10"/>
     </row>
-    <row r="70" spans="1:11">
+    <row r="70" spans="1:14">
       <c r="A70" s="10"/>
       <c r="F70" s="10"/>
       <c r="G70" s="10" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="H70" s="10"/>
       <c r="I70" s="10"/>
       <c r="J70" s="10"/>
       <c r="K70" s="10"/>
-    </row>
-    <row r="71" spans="1:11">
+      <c r="L70" s="10"/>
+      <c r="M70" s="10"/>
+      <c r="N70" s="10"/>
+    </row>
+    <row r="71" spans="1:14">
       <c r="A71" s="10"/>
       <c r="F71" s="10"/>
-      <c r="G71" s="10"/>
+      <c r="G71" s="10" t="s">
+        <v>75</v>
+      </c>
       <c r="H71" s="10"/>
       <c r="I71" s="10"/>
       <c r="J71" s="10"/>
       <c r="K71" s="10"/>
     </row>
-    <row r="72" spans="1:11">
+    <row r="72" spans="1:14">
       <c r="A72" s="10"/>
       <c r="F72" s="10"/>
       <c r="G72" s="10"/>
@@ -3426,36 +3482,37 @@
       <c r="J72" s="10"/>
       <c r="K72" s="10"/>
     </row>
-    <row r="73" spans="1:11">
+    <row r="73" spans="1:14">
       <c r="A73" s="10"/>
-      <c r="F73" s="81"/>
-      <c r="G73" s="81"/>
-      <c r="H73" s="10">
-        <v>5</v>
-      </c>
-      <c r="I73" s="10">
-        <v>3</v>
-      </c>
+      <c r="F73" s="10"/>
+      <c r="G73" s="10"/>
+      <c r="H73" s="10"/>
+      <c r="I73" s="10"/>
       <c r="J73" s="10"/>
       <c r="K73" s="10"/>
     </row>
-    <row r="74" spans="6:11">
-      <c r="F74" s="10"/>
-      <c r="G74" s="10"/>
-      <c r="H74" s="73"/>
-      <c r="I74" s="10"/>
+    <row r="74" spans="1:14">
+      <c r="A74" s="10"/>
+      <c r="F74" s="69"/>
+      <c r="G74" s="69"/>
+      <c r="H74" s="10">
+        <v>5</v>
+      </c>
+      <c r="I74" s="10">
+        <v>3</v>
+      </c>
       <c r="J74" s="10"/>
       <c r="K74" s="10"/>
     </row>
-    <row r="75" spans="6:11">
+    <row r="75" spans="1:14">
       <c r="F75" s="10"/>
       <c r="G75" s="10"/>
-      <c r="H75" s="10"/>
+      <c r="H75" s="78"/>
       <c r="I75" s="10"/>
       <c r="J75" s="10"/>
       <c r="K75" s="10"/>
     </row>
-    <row r="76" spans="6:11">
+    <row r="76" spans="1:14">
       <c r="F76" s="10"/>
       <c r="G76" s="10"/>
       <c r="H76" s="10"/>
@@ -3463,29 +3520,29 @@
       <c r="J76" s="10"/>
       <c r="K76" s="10"/>
     </row>
-    <row r="77" spans="6:11">
+    <row r="77" spans="1:14">
       <c r="F77" s="10"/>
+      <c r="G77" s="10"/>
       <c r="H77" s="10"/>
       <c r="I77" s="10"/>
       <c r="J77" s="10"/>
       <c r="K77" s="10"/>
     </row>
-    <row r="78" spans="6:11">
+    <row r="78" spans="1:14">
       <c r="F78" s="10"/>
       <c r="H78" s="10"/>
       <c r="I78" s="10"/>
       <c r="J78" s="10"/>
       <c r="K78" s="10"/>
     </row>
-    <row r="79" spans="6:11">
+    <row r="79" spans="1:14">
       <c r="F79" s="10"/>
-      <c r="G79" s="10"/>
       <c r="H79" s="10"/>
       <c r="I79" s="10"/>
       <c r="J79" s="10"/>
       <c r="K79" s="10"/>
     </row>
-    <row r="80" spans="6:11">
+    <row r="80" spans="1:14">
       <c r="F80" s="10"/>
       <c r="G80" s="10"/>
       <c r="H80" s="10"/>
@@ -3493,7 +3550,7 @@
       <c r="J80" s="10"/>
       <c r="K80" s="10"/>
     </row>
-    <row r="81" spans="6:11">
+    <row r="81" spans="1:11">
       <c r="F81" s="10"/>
       <c r="G81" s="10"/>
       <c r="H81" s="10"/>
@@ -3501,7 +3558,7 @@
       <c r="J81" s="10"/>
       <c r="K81" s="10"/>
     </row>
-    <row r="82" spans="6:11">
+    <row r="82" spans="1:11">
       <c r="F82" s="10"/>
       <c r="G82" s="10"/>
       <c r="H82" s="10"/>
@@ -3509,47 +3566,42 @@
       <c r="J82" s="10"/>
       <c r="K82" s="10"/>
     </row>
-    <row r="83" spans="6:11">
-      <c r="F83" s="85"/>
+    <row r="83" spans="1:11">
+      <c r="F83" s="10"/>
       <c r="G83" s="10"/>
       <c r="H83" s="10"/>
       <c r="I83" s="10"/>
       <c r="J83" s="10"/>
       <c r="K83" s="10"/>
     </row>
-    <row r="84" spans="2:11">
-      <c r="B84" s="10"/>
-      <c r="C84" s="10">
-        <f>AVERAGE(H42:H50)</f>
-        <v>18.8888888888889</v>
-      </c>
-      <c r="D84" s="10">
-        <f>AVERAGE(I42:I50)</f>
-        <v>6.11111111111111</v>
-      </c>
-      <c r="E84" s="10"/>
-      <c r="F84" s="10"/>
+    <row r="84" spans="1:11">
+      <c r="F84" s="85"/>
       <c r="G84" s="10"/>
       <c r="H84" s="10"/>
       <c r="I84" s="10"/>
       <c r="J84" s="10"/>
       <c r="K84" s="10"/>
     </row>
-    <row r="85" spans="5:11">
+    <row r="85" spans="1:11">
+      <c r="B85" s="10"/>
+      <c r="C85" s="10">
+        <f>AVERAGE(H43:H51)</f>
+        <v>18.8888888888889</v>
+      </c>
+      <c r="D85" s="10">
+        <f>AVERAGE(I43:I51)</f>
+        <v>6.11111111111111</v>
+      </c>
       <c r="E85" s="10"/>
+      <c r="F85" s="10"/>
+      <c r="G85" s="10"/>
+      <c r="H85" s="10"/>
       <c r="I85" s="10"/>
       <c r="J85" s="10"/>
       <c r="K85" s="10"/>
     </row>
     <row r="86" spans="1:11">
-      <c r="A86" s="10"/>
-      <c r="B86" s="10"/>
-      <c r="C86" s="10"/>
-      <c r="D86" s="10"/>
       <c r="E86" s="10"/>
-      <c r="F86" s="85"/>
-      <c r="G86" s="10"/>
-      <c r="H86" s="10"/>
       <c r="I86" s="10"/>
       <c r="J86" s="10"/>
       <c r="K86" s="10"/>
@@ -3560,65 +3612,72 @@
       <c r="C87" s="10"/>
       <c r="D87" s="10"/>
       <c r="E87" s="10"/>
-      <c r="F87" s="10"/>
+      <c r="F87" s="85"/>
       <c r="G87" s="10"/>
       <c r="H87" s="10"/>
       <c r="I87" s="10"/>
       <c r="J87" s="10"/>
       <c r="K87" s="10"/>
     </row>
-    <row r="88" spans="2:6">
+    <row r="88" spans="1:11">
+      <c r="A88" s="10"/>
       <c r="B88" s="10"/>
       <c r="C88" s="10"/>
       <c r="D88" s="10"/>
       <c r="E88" s="10"/>
       <c r="F88" s="10"/>
-    </row>
-    <row r="89" spans="1:6">
-      <c r="A89" s="10"/>
+      <c r="G88" s="10"/>
+      <c r="H88" s="10"/>
+      <c r="I88" s="10"/>
+      <c r="J88" s="10"/>
+      <c r="K88" s="10"/>
+    </row>
+    <row r="89" spans="1:11">
       <c r="B89" s="10"/>
       <c r="C89" s="10"/>
       <c r="D89" s="10"/>
       <c r="E89" s="10"/>
       <c r="F89" s="10"/>
     </row>
-    <row r="90" spans="3:6">
+    <row r="90" spans="1:11">
+      <c r="A90" s="10"/>
+      <c r="B90" s="10"/>
       <c r="C90" s="10"/>
       <c r="D90" s="10"/>
       <c r="E90" s="10"/>
       <c r="F90" s="10"/>
     </row>
-    <row r="91" spans="3:6">
+    <row r="91" spans="1:11">
       <c r="C91" s="10"/>
       <c r="D91" s="10"/>
       <c r="E91" s="10"/>
-      <c r="F91" s="72"/>
-    </row>
-    <row r="92" spans="3:6">
+      <c r="F91" s="10"/>
+    </row>
+    <row r="92" spans="1:11">
       <c r="C92" s="10"/>
       <c r="D92" s="10"/>
       <c r="E92" s="10"/>
-      <c r="F92" s="10"/>
-    </row>
-    <row r="93" spans="3:6">
+      <c r="F92" s="77"/>
+    </row>
+    <row r="93" spans="1:11">
       <c r="C93" s="10"/>
       <c r="D93" s="10"/>
       <c r="E93" s="10"/>
       <c r="F93" s="10"/>
     </row>
-    <row r="94" spans="3:6">
+    <row r="94" spans="1:11">
       <c r="C94" s="10"/>
       <c r="D94" s="10"/>
       <c r="E94" s="10"/>
       <c r="F94" s="10"/>
     </row>
-    <row r="95" spans="3:6">
+    <row r="95" spans="1:11">
       <c r="C95" s="10"/>
       <c r="D95" s="10"/>
       <c r="E95" s="10"/>
       <c r="F95" s="10"/>
     </row>
-    <row r="96" spans="3:6">
+    <row r="96" spans="1:11">
       <c r="C96" s="10"/>
       <c r="D96" s="10"/>
       <c r="E96" s="10"/>
@@ -3648,14 +3707,20 @@
       <c r="E100" s="10"/>
       <c r="F100" s="10"/>
     </row>
+    <row r="101" spans="3:6">
+      <c r="C101" s="10"/>
+      <c r="D101" s="10"/>
+      <c r="E101" s="10"/>
+      <c r="F101" s="10"/>
+    </row>
   </sheetData>
   <mergeCells count="6">
-    <mergeCell ref="C15:F15"/>
     <mergeCell ref="C16:F16"/>
-    <mergeCell ref="C26:D26"/>
+    <mergeCell ref="C17:F17"/>
     <mergeCell ref="C27:D27"/>
-    <mergeCell ref="K63:L63"/>
+    <mergeCell ref="C28:D28"/>
     <mergeCell ref="K64:L64"/>
+    <mergeCell ref="K65:L65"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511805555555556" footer="0.511805555555556"/>
   <headerFooter/>
@@ -3688,37 +3753,37 @@
     <row r="2" s="1" customFormat="1" ht="19.5" spans="1:15">
       <c r="A2" s="4"/>
       <c r="B2" s="5" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="C2" s="5" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="D2" s="5" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="E2" s="5" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="F2" s="5" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="G2" s="5" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="H2" s="5" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="I2" s="5" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="J2" s="5" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="K2" s="5" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="L2" s="5" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="M2" s="5"/>
       <c r="N2" s="5"/>
@@ -3729,37 +3794,37 @@
         <v>2</v>
       </c>
       <c r="B3" s="7" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="C3" s="7" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="D3" s="7" t="s">
+        <v>105</v>
+      </c>
+      <c r="E3" s="7" t="s">
+        <v>106</v>
+      </c>
+      <c r="F3" s="7" t="s">
         <v>104</v>
       </c>
-      <c r="E3" s="7" t="s">
-        <v>105</v>
-      </c>
-      <c r="F3" s="7" t="s">
-        <v>103</v>
-      </c>
       <c r="G3" s="7" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="H3" s="7" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="I3" s="7" t="s">
+        <v>108</v>
+      </c>
+      <c r="J3" s="7" t="s">
+        <v>104</v>
+      </c>
+      <c r="K3" s="7" t="s">
         <v>107</v>
       </c>
-      <c r="J3" s="7" t="s">
-        <v>103</v>
-      </c>
-      <c r="K3" s="7" t="s">
-        <v>106</v>
-      </c>
       <c r="L3" s="7" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="M3" s="7"/>
       <c r="N3" s="7"/>
@@ -3770,37 +3835,37 @@
         <v>3</v>
       </c>
       <c r="B4" s="7" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="C4" s="7" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="D4" s="7" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="E4" s="7" t="s">
+        <v>108</v>
+      </c>
+      <c r="F4" s="7" t="s">
         <v>107</v>
       </c>
-      <c r="F4" s="7" t="s">
-        <v>106</v>
-      </c>
       <c r="G4" s="7" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="H4" s="7" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="I4" s="7" t="s">
+        <v>108</v>
+      </c>
+      <c r="J4" s="7" t="s">
+        <v>104</v>
+      </c>
+      <c r="K4" s="7" t="s">
         <v>107</v>
       </c>
-      <c r="J4" s="7" t="s">
-        <v>103</v>
-      </c>
-      <c r="K4" s="7" t="s">
-        <v>106</v>
-      </c>
       <c r="L4" s="7" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="M4" s="7"/>
       <c r="N4" s="7"/>
@@ -3811,35 +3876,35 @@
         <v>4</v>
       </c>
       <c r="B5" s="8" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="C5" s="7" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="D5" s="7"/>
       <c r="E5" s="7" t="s">
+        <v>108</v>
+      </c>
+      <c r="F5" s="8" t="s">
+        <v>109</v>
+      </c>
+      <c r="G5" s="7" t="s">
         <v>107</v>
       </c>
-      <c r="F5" s="8" t="s">
+      <c r="H5" s="7" t="s">
+        <v>107</v>
+      </c>
+      <c r="I5" s="7" t="s">
         <v>108</v>
       </c>
-      <c r="G5" s="7" t="s">
-        <v>106</v>
-      </c>
-      <c r="H5" s="7" t="s">
-        <v>106</v>
-      </c>
-      <c r="I5" s="7" t="s">
+      <c r="J5" s="7" t="s">
         <v>107</v>
       </c>
-      <c r="J5" s="7" t="s">
-        <v>106</v>
-      </c>
       <c r="K5" s="9" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="L5" s="7" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="M5" s="7"/>
       <c r="N5" s="7"/>
@@ -3850,33 +3915,33 @@
         <v>5</v>
       </c>
       <c r="B6" s="7" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="C6" s="8" t="s">
+        <v>109</v>
+      </c>
+      <c r="D6" s="7" t="s">
+        <v>107</v>
+      </c>
+      <c r="E6" s="7" t="s">
         <v>108</v>
       </c>
-      <c r="D6" s="7" t="s">
-        <v>106</v>
-      </c>
-      <c r="E6" s="7" t="s">
+      <c r="F6" s="7" t="s">
         <v>107</v>
       </c>
-      <c r="F6" s="7" t="s">
-        <v>106</v>
-      </c>
       <c r="G6" s="8" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="H6" s="7" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="I6" s="7"/>
       <c r="J6" s="7" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="K6" s="7"/>
       <c r="L6" s="7" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="M6" s="7"/>
       <c r="N6" s="7"/>
@@ -3887,37 +3952,37 @@
         <v>6</v>
       </c>
       <c r="B7" s="7" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="C7" s="7" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="D7" s="7" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="E7" s="7" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="F7" s="7" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="G7" s="7" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="H7" s="7" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="I7" s="7" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="J7" s="7" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="K7" s="7" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="L7" s="7" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="M7" s="7"/>
       <c r="N7" s="7"/>
@@ -3929,30 +3994,30 @@
       </c>
       <c r="B8" s="7"/>
       <c r="C8" s="7" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="D8" s="7"/>
       <c r="E8" s="7" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="F8" s="7"/>
       <c r="G8" s="7" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="H8" s="7" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="I8" s="7" t="s">
+        <v>108</v>
+      </c>
+      <c r="J8" s="7" t="s">
         <v>107</v>
       </c>
-      <c r="J8" s="7" t="s">
-        <v>106</v>
-      </c>
       <c r="K8" s="7" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="L8" s="7" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="M8" s="7"/>
       <c r="N8" s="7"/>
@@ -3966,7 +4031,7 @@
       <c r="C9" s="7"/>
       <c r="D9" s="7"/>
       <c r="E9" s="7" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="F9" s="7"/>
       <c r="G9" s="7"/>
@@ -3984,24 +4049,24 @@
         <v>9</v>
       </c>
       <c r="B10" s="7" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="C10" s="7"/>
       <c r="D10" s="7" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="E10" s="7" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="F10" s="7"/>
       <c r="G10" s="7"/>
       <c r="H10" s="7"/>
       <c r="I10" s="7" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="J10" s="7"/>
       <c r="K10" s="7" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="L10" s="7"/>
       <c r="M10" s="7"/>
@@ -4013,35 +4078,35 @@
         <v>10</v>
       </c>
       <c r="B11" s="7" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="C11" s="7" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="D11" s="7" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="E11" s="7" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="F11" s="7" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="G11" s="7" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="H11" s="7" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="I11" s="7" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="J11" s="7"/>
       <c r="K11" s="7" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="L11" s="7" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="M11" s="7"/>
       <c r="N11" s="7"/>

</xml_diff>

<commit_message>
Design: Working on Warrior.
</commit_message>
<xml_diff>
--- a/Design/Tables.xlsx
+++ b/Design/Tables.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="27630" windowHeight="12300"/>
+    <workbookView windowWidth="20475" windowHeight="12300"/>
   </bookViews>
   <sheets>
     <sheet name="Standard" sheetId="3" r:id="rId1"/>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="196" uniqueCount="115">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="199" uniqueCount="118">
   <si>
     <t>Action Points</t>
   </si>
@@ -40,6 +40,9 @@
   </si>
   <si>
     <t>Heal</t>
+  </si>
+  <si>
+    <t>Shielding</t>
   </si>
   <si>
     <t>Ranged Penalty</t>
@@ -64,6 +67,10 @@
       </rPr>
       <t>AoE 5</t>
     </r>
+  </si>
+  <si>
+    <t>Katana 1d8+, Magic Ward 1d6
+Grenade Xd4, Reforge W. 1d6</t>
   </si>
   <si>
     <r>
@@ -143,6 +150,9 @@
       </rPr>
       <t>AoE 2</t>
     </r>
+  </si>
+  <si>
+    <t>Homecoming 2d6</t>
   </si>
   <si>
     <r>
@@ -1532,7 +1542,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="86">
+  <cellXfs count="87">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -1589,6 +1599,9 @@
     </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -2127,9 +2140,9 @@
     <col min="2" max="2" width="19.7333333333333" customWidth="1"/>
     <col min="3" max="3" width="24.4761904761905" customWidth="1"/>
     <col min="4" max="4" width="26.8285714285714" customWidth="1"/>
-    <col min="5" max="5" width="30.7904761904762" customWidth="1"/>
+    <col min="5" max="5" width="30.2857142857143" customWidth="1"/>
     <col min="6" max="6" width="24.5809523809524" customWidth="1"/>
-    <col min="7" max="7" width="27.9428571428571" customWidth="1"/>
+    <col min="7" max="7" width="44.2857142857143" customWidth="1"/>
     <col min="8" max="8" width="21" customWidth="1"/>
     <col min="9" max="9" width="25.952380952381" customWidth="1"/>
     <col min="10" max="10" width="23.7238095238095" customWidth="1"/>
@@ -2161,6 +2174,9 @@
       <c r="E4" s="13" t="s">
         <v>4</v>
       </c>
+      <c r="F4" s="13" t="s">
+        <v>5</v>
+      </c>
       <c r="H4" s="10"/>
     </row>
     <row r="5" ht="15.75" spans="1:11">
@@ -2179,9 +2195,13 @@
       <c r="E5" s="17">
         <v>0</v>
       </c>
+      <c r="F5" s="17">
+        <v>0</v>
+      </c>
+      <c r="G5"/>
       <c r="H5" s="10"/>
     </row>
-    <row r="6" ht="15.75" spans="1:11">
+    <row r="6" ht="30" spans="1:11">
       <c r="A6" s="14">
         <v>1</v>
       </c>
@@ -2189,16 +2209,22 @@
         <v>0</v>
       </c>
       <c r="C6" s="18" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D6" s="17">
         <v>0</v>
       </c>
       <c r="E6" s="17">
+        <v>3.5</v>
+      </c>
+      <c r="F6" s="17">
         <v>-1</v>
       </c>
-      <c r="H6" s="19"/>
-      <c r="K6" s="20"/>
+      <c r="G6" s="19" t="s">
+        <v>7</v>
+      </c>
+      <c r="H6" s="20"/>
+      <c r="K6" s="21"/>
     </row>
     <row r="7" customFormat="1" ht="15.75" spans="1:11">
       <c r="A7" s="14">
@@ -2208,16 +2234,19 @@
         <v>0</v>
       </c>
       <c r="C7" s="18" t="s">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="D7" s="17">
         <v>0</v>
       </c>
       <c r="E7" s="17">
+        <v>5.5</v>
+      </c>
+      <c r="F7" s="17">
         <v>-2</v>
       </c>
-      <c r="H7" s="21"/>
-      <c r="K7" s="20"/>
+      <c r="H7" s="22"/>
+      <c r="K7" s="21"/>
     </row>
     <row r="8" ht="15.75" spans="1:11">
       <c r="A8" s="14">
@@ -2227,39 +2256,46 @@
         <v>0</v>
       </c>
       <c r="C8" s="18" t="s">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="D8" s="17">
         <v>0</v>
       </c>
       <c r="E8" s="17">
+        <v>9.5</v>
+      </c>
+      <c r="F8" s="17">
         <v>-3</v>
       </c>
-      <c r="F8"/>
-      <c r="H8" s="21"/>
-      <c r="K8" s="20"/>
+      <c r="G8"/>
+      <c r="H8" s="22"/>
+      <c r="K8" s="21"/>
     </row>
     <row r="9" ht="15.75" spans="1:11">
-      <c r="A9" s="22">
+      <c r="A9" s="23">
         <v>0</v>
       </c>
-      <c r="B9" s="23">
+      <c r="B9" s="24">
         <v>1</v>
       </c>
-      <c r="C9" s="24" t="s">
-        <v>8</v>
-      </c>
-      <c r="D9" s="25" t="s">
-        <v>9</v>
+      <c r="C9" s="25" t="s">
+        <v>10</v>
+      </c>
+      <c r="D9" s="26" t="s">
+        <v>11</v>
       </c>
       <c r="E9" s="26">
+        <v>5</v>
+      </c>
+      <c r="F9" s="27">
         <v>0</v>
       </c>
-      <c r="F9"/>
-      <c r="G9"/>
-      <c r="H9" s="19"/>
-      <c r="J9" s="27"/>
-      <c r="K9" s="20"/>
+      <c r="G9" t="s">
+        <v>12</v>
+      </c>
+      <c r="H9" s="20"/>
+      <c r="J9" s="28"/>
+      <c r="K9" s="21"/>
     </row>
     <row r="10" ht="15.75" spans="1:11">
       <c r="A10" s="14">
@@ -2269,16 +2305,19 @@
         <v>1</v>
       </c>
       <c r="C10" s="18" t="s">
-        <v>10</v>
-      </c>
-      <c r="D10" s="28" t="s">
-        <v>11</v>
-      </c>
-      <c r="E10" s="17">
+        <v>13</v>
+      </c>
+      <c r="D10" s="29" t="s">
+        <v>14</v>
+      </c>
+      <c r="E10" s="29">
+        <v>8.5</v>
+      </c>
+      <c r="F10" s="17">
         <v>-1</v>
       </c>
-      <c r="H10" s="21"/>
-      <c r="K10" s="20"/>
+      <c r="H10" s="22"/>
+      <c r="K10" s="21"/>
     </row>
     <row r="11" ht="15.75" spans="1:11">
       <c r="A11" s="14">
@@ -2288,318 +2327,333 @@
         <v>1</v>
       </c>
       <c r="C11" s="14" t="s">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="D11" s="17" t="s">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="E11" s="17">
+        <v>11</v>
+      </c>
+      <c r="F11" s="17">
         <v>-2</v>
       </c>
-      <c r="F11">
-        <f>5*2.5</f>
-        <v>12.5</v>
-      </c>
-      <c r="H11" s="21"/>
-      <c r="K11" s="20"/>
+      <c r="G11">
+        <f>5*3.5</f>
+        <v>17.5</v>
+      </c>
+      <c r="H11" s="22"/>
+      <c r="K11" s="21"/>
     </row>
     <row r="12" ht="16.5" spans="1:11">
-      <c r="A12" s="29">
+      <c r="A12" s="30">
         <v>3</v>
       </c>
-      <c r="B12" s="30">
+      <c r="B12" s="31">
         <v>1</v>
       </c>
-      <c r="C12" s="29" t="s">
+      <c r="C12" s="30" t="s">
+        <v>17</v>
+      </c>
+      <c r="D12" s="32" t="s">
+        <v>18</v>
+      </c>
+      <c r="E12" s="32">
         <v>14</v>
       </c>
-      <c r="D12" s="31" t="s">
-        <v>15</v>
-      </c>
-      <c r="E12" s="32">
+      <c r="F12" s="33">
         <v>-3</v>
       </c>
-      <c r="G12" s="10"/>
-      <c r="H12" s="20"/>
-      <c r="I12" s="20"/>
-      <c r="J12" s="20"/>
-      <c r="K12" s="20"/>
+      <c r="G12" s="10">
+        <f>3*5.5</f>
+        <v>16.5</v>
+      </c>
+      <c r="H12" s="21"/>
+      <c r="I12" s="21"/>
+      <c r="J12" s="21"/>
+      <c r="K12" s="21"/>
     </row>
     <row r="13" ht="15.75" spans="1:11">
-      <c r="A13" s="33">
+      <c r="A13" s="34">
         <v>1</v>
       </c>
-      <c r="B13" s="34" t="s">
-        <v>16</v>
-      </c>
-      <c r="C13" s="35">
+      <c r="B13" s="35" t="s">
+        <v>19</v>
+      </c>
+      <c r="C13" s="36">
         <v>6</v>
       </c>
-      <c r="D13" s="34">
+      <c r="D13" s="35">
         <v>2</v>
       </c>
       <c r="E13" s="13">
         <v>3</v>
       </c>
+      <c r="F13" s="13">
+        <v>3</v>
+      </c>
       <c r="G13" s="10"/>
-      <c r="H13" s="20"/>
-      <c r="I13" s="20"/>
-      <c r="J13" s="20"/>
-      <c r="K13" s="20"/>
+      <c r="H13" s="21"/>
+      <c r="I13" s="21"/>
+      <c r="J13" s="21"/>
+      <c r="K13" s="21"/>
     </row>
     <row r="14" ht="16.5" spans="1:11">
-      <c r="A14" s="36">
+      <c r="A14" s="37">
         <v>1</v>
       </c>
-      <c r="B14" s="29" t="s">
-        <v>17</v>
-      </c>
-      <c r="C14" s="37">
+      <c r="B14" s="30" t="s">
+        <v>20</v>
+      </c>
+      <c r="C14" s="38">
         <v>8</v>
       </c>
-      <c r="D14" s="29">
+      <c r="D14" s="30">
         <v>4</v>
       </c>
-      <c r="E14" s="32">
+      <c r="E14" s="33">
         <v>5.5</v>
       </c>
+      <c r="F14" s="33">
+        <v>5.5</v>
+      </c>
       <c r="G14" s="10"/>
-      <c r="H14" s="20"/>
-      <c r="I14" s="20"/>
-      <c r="J14" s="20"/>
-      <c r="K14" s="20"/>
+      <c r="H14" s="21"/>
+      <c r="I14" s="21"/>
+      <c r="J14" s="21"/>
+      <c r="K14" s="21"/>
     </row>
     <row r="15" ht="16.5" spans="1:11">
-      <c r="A15" s="38"/>
-      <c r="B15" s="21"/>
-      <c r="C15" s="21"/>
-      <c r="D15" s="21"/>
+      <c r="A15" s="39"/>
+      <c r="B15" s="22"/>
+      <c r="C15" s="22"/>
+      <c r="D15" s="22"/>
       <c r="E15" s="10"/>
       <c r="F15" s="10"/>
-      <c r="G15" s="27"/>
+      <c r="G15" s="28"/>
       <c r="H15" s="10"/>
-      <c r="I15" s="20"/>
-      <c r="J15" s="20"/>
-      <c r="K15" s="39"/>
+      <c r="I15" s="21"/>
+      <c r="J15" s="21"/>
+      <c r="K15" s="40"/>
     </row>
     <row r="16" ht="15.75" spans="1:11">
-      <c r="A16" s="40"/>
-      <c r="B16" s="41"/>
-      <c r="C16" s="42" t="s">
-        <v>18</v>
-      </c>
-      <c r="D16" s="43"/>
-      <c r="E16" s="43"/>
-      <c r="F16" s="44"/>
+      <c r="A16" s="41"/>
+      <c r="B16" s="42"/>
+      <c r="C16" s="43" t="s">
+        <v>21</v>
+      </c>
+      <c r="D16" s="44"/>
+      <c r="E16" s="44"/>
+      <c r="F16" s="45"/>
       <c r="K16" s="10"/>
     </row>
     <row r="17" ht="16.5" spans="1:12">
-      <c r="A17" s="45" t="s">
-        <v>19</v>
-      </c>
-      <c r="B17" s="46" t="s">
+      <c r="A17" s="46" t="s">
+        <v>22</v>
+      </c>
+      <c r="B17" s="47" t="s">
         <v>1</v>
       </c>
-      <c r="C17" s="47" t="s">
-        <v>20</v>
-      </c>
-      <c r="D17" s="48"/>
-      <c r="E17" s="48"/>
-      <c r="F17" s="49"/>
-      <c r="K17" s="50"/>
-      <c r="L17" s="50"/>
+      <c r="C17" s="48" t="s">
+        <v>23</v>
+      </c>
+      <c r="D17" s="49"/>
+      <c r="E17" s="49"/>
+      <c r="F17" s="50"/>
+      <c r="K17" s="51"/>
+      <c r="L17" s="51"/>
     </row>
     <row r="18" spans="1:12">
-      <c r="A18" s="51">
+      <c r="A18" s="52">
         <v>0</v>
       </c>
       <c r="B18" s="10">
         <v>0</v>
       </c>
-      <c r="C18" s="51" t="s">
-        <v>21</v>
+      <c r="C18" s="52" t="s">
+        <v>24</v>
       </c>
       <c r="D18" s="10" t="s">
-        <v>22</v>
-      </c>
-      <c r="E18" s="41"/>
-      <c r="F18" s="52"/>
+        <v>25</v>
+      </c>
+      <c r="E18" s="42"/>
+      <c r="F18" s="53"/>
       <c r="K18" s="10"/>
     </row>
     <row r="19" spans="1:12">
-      <c r="A19" s="51">
+      <c r="A19" s="52">
         <v>0.5</v>
       </c>
       <c r="B19" s="10">
         <v>0</v>
       </c>
-      <c r="C19" s="53" t="s">
-        <v>23</v>
-      </c>
-      <c r="D19" s="54" t="s">
-        <v>24</v>
+      <c r="C19" s="54" t="s">
+        <v>26</v>
+      </c>
+      <c r="D19" s="55" t="s">
+        <v>27</v>
       </c>
       <c r="E19" s="10"/>
-      <c r="F19" s="55"/>
+      <c r="F19" s="56"/>
       <c r="K19" s="10"/>
     </row>
     <row r="20" spans="1:12">
-      <c r="A20" s="51">
+      <c r="A20" s="52">
         <v>1</v>
       </c>
       <c r="B20" s="10">
         <v>0</v>
       </c>
-      <c r="C20" s="56"/>
-      <c r="D20" s="57"/>
-      <c r="E20" s="57"/>
-      <c r="F20" s="58"/>
+      <c r="C20" s="57"/>
+      <c r="D20" s="58"/>
+      <c r="E20" s="58"/>
+      <c r="F20" s="59"/>
       <c r="K20" s="10"/>
     </row>
     <row r="21" spans="1:12">
-      <c r="A21" s="51">
+      <c r="A21" s="52">
         <v>0</v>
       </c>
       <c r="B21" s="10">
         <v>1</v>
       </c>
-      <c r="C21" s="51" t="s">
-        <v>25</v>
+      <c r="C21" s="52" t="s">
+        <v>28</v>
       </c>
       <c r="D21" s="10" t="s">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="E21" s="10" t="s">
-        <v>27</v>
-      </c>
-      <c r="F21" s="55" t="s">
-        <v>28</v>
+        <v>30</v>
+      </c>
+      <c r="F21" s="56" t="s">
+        <v>31</v>
       </c>
     </row>
     <row r="22" spans="1:12">
-      <c r="A22" s="51">
+      <c r="A22" s="52">
         <v>0.5</v>
       </c>
       <c r="B22" s="10">
         <v>1</v>
       </c>
-      <c r="C22" s="51" t="s">
-        <v>29</v>
+      <c r="C22" s="52" t="s">
+        <v>32</v>
       </c>
       <c r="D22" s="10" t="s">
-        <v>30</v>
+        <v>33</v>
       </c>
       <c r="E22" s="10"/>
-      <c r="F22" s="55"/>
+      <c r="F22" s="56"/>
     </row>
     <row r="23" ht="15.75" spans="1:12">
-      <c r="A23" s="59">
+      <c r="A23" s="60">
         <v>1</v>
       </c>
-      <c r="B23" s="60">
+      <c r="B23" s="61">
         <v>1</v>
       </c>
-      <c r="C23" s="59"/>
-      <c r="D23" s="60"/>
-      <c r="E23" s="60"/>
-      <c r="F23" s="61"/>
+      <c r="C23" s="60"/>
+      <c r="D23" s="61"/>
+      <c r="E23" s="61"/>
+      <c r="F23" s="62"/>
     </row>
     <row r="24" ht="15.75" spans="1:12">
-      <c r="A24" s="33">
+      <c r="A24" s="34">
         <v>1</v>
       </c>
-      <c r="B24" s="62" t="s">
-        <v>16</v>
-      </c>
-      <c r="C24" s="40" t="s">
-        <v>31</v>
-      </c>
-      <c r="D24" s="63"/>
-      <c r="E24" s="63"/>
-      <c r="F24" s="62"/>
-      <c r="K24" s="21"/>
+      <c r="B24" s="63" t="s">
+        <v>19</v>
+      </c>
+      <c r="C24" s="41" t="s">
+        <v>34</v>
+      </c>
+      <c r="D24" s="64"/>
+      <c r="E24" s="64"/>
+      <c r="F24" s="63"/>
+      <c r="K24" s="22"/>
     </row>
     <row r="25" ht="16.5" spans="1:12">
-      <c r="A25" s="36">
+      <c r="A25" s="37">
         <v>1</v>
       </c>
-      <c r="B25" s="64" t="s">
-        <v>17</v>
-      </c>
-      <c r="C25" s="36" t="s">
-        <v>32</v>
-      </c>
-      <c r="D25" s="30" t="s">
-        <v>33</v>
-      </c>
-      <c r="E25" s="30"/>
-      <c r="F25" s="64"/>
-      <c r="K25" s="21"/>
+      <c r="B25" s="65" t="s">
+        <v>20</v>
+      </c>
+      <c r="C25" s="37" t="s">
+        <v>35</v>
+      </c>
+      <c r="D25" s="31" t="s">
+        <v>36</v>
+      </c>
+      <c r="E25" s="31"/>
+      <c r="F25" s="65"/>
+      <c r="K25" s="22"/>
     </row>
     <row r="26" ht="15.75" spans="1:12">
-      <c r="A26" s="21"/>
-      <c r="B26" s="21"/>
-      <c r="C26" s="21"/>
-      <c r="D26" s="21"/>
-      <c r="E26" s="21"/>
-      <c r="F26" s="21"/>
-      <c r="G26" s="21"/>
-      <c r="H26" s="21"/>
+      <c r="A26" s="22"/>
+      <c r="B26" s="22"/>
+      <c r="C26" s="22"/>
+      <c r="D26" s="22"/>
+      <c r="E26" s="22"/>
+      <c r="F26" s="22"/>
+      <c r="G26" s="22"/>
+      <c r="H26" s="22"/>
       <c r="I26" s="10"/>
       <c r="J26" s="10"/>
-      <c r="K26" s="21"/>
+      <c r="K26" s="22"/>
     </row>
     <row r="27" ht="16.5" spans="1:12">
-      <c r="A27" s="21"/>
-      <c r="B27" s="21"/>
-      <c r="C27" s="21"/>
-      <c r="D27" s="21"/>
-      <c r="E27" s="21"/>
-      <c r="F27" s="21"/>
-      <c r="G27" s="21"/>
-      <c r="H27" s="21"/>
+      <c r="A27" s="22"/>
+      <c r="B27" s="22"/>
+      <c r="C27" s="22"/>
+      <c r="D27" s="22"/>
+      <c r="E27" s="22"/>
+      <c r="F27" s="22"/>
+      <c r="G27" s="22"/>
+      <c r="H27" s="22"/>
       <c r="I27" s="10"/>
       <c r="J27" s="10"/>
-      <c r="K27" s="21"/>
+      <c r="K27" s="22"/>
     </row>
     <row r="28" ht="16.5" spans="1:12">
-      <c r="A28" s="21"/>
-      <c r="C28" s="33" t="s">
-        <v>34</v>
-      </c>
-      <c r="D28" s="62"/>
-      <c r="F28" s="21"/>
-      <c r="G28" s="21"/>
-      <c r="H28" s="38"/>
-      <c r="I28" s="21"/>
+      <c r="A28" s="22"/>
+      <c r="C28" s="34" t="s">
+        <v>37</v>
+      </c>
+      <c r="D28" s="63"/>
+      <c r="F28" s="22"/>
+      <c r="G28" s="22"/>
+      <c r="H28" s="39"/>
+      <c r="I28" s="22"/>
       <c r="J28" s="10"/>
-      <c r="K28" s="21"/>
+      <c r="K28" s="22"/>
     </row>
     <row r="29" ht="16.5" spans="1:12">
-      <c r="A29" s="38"/>
-      <c r="B29" s="40" t="s">
-        <v>35</v>
-      </c>
-      <c r="C29" s="41" t="s">
-        <v>36</v>
-      </c>
-      <c r="D29" s="41" t="s">
-        <v>37</v>
-      </c>
-      <c r="E29" s="62" t="s">
+      <c r="A29" s="39"/>
+      <c r="B29" s="41" t="s">
         <v>38</v>
+      </c>
+      <c r="C29" s="42" t="s">
+        <v>39</v>
+      </c>
+      <c r="D29" s="42" t="s">
+        <v>40</v>
+      </c>
+      <c r="E29" s="63" t="s">
+        <v>41</v>
       </c>
       <c r="G29" s="10"/>
       <c r="H29" s="10" t="s">
-        <v>39</v>
+        <v>42</v>
       </c>
       <c r="I29" s="10"/>
       <c r="J29" s="10"/>
-      <c r="K29" s="65"/>
+      <c r="K29" s="66"/>
     </row>
     <row r="30" ht="15.75" spans="1:12">
-      <c r="A30" s="38"/>
-      <c r="B30" s="51">
+      <c r="A30" s="39"/>
+      <c r="B30" s="52">
         <v>25</v>
       </c>
       <c r="C30" s="10">
@@ -2608,23 +2662,23 @@
       <c r="D30" s="10">
         <v>1.5</v>
       </c>
-      <c r="E30" s="66">
+      <c r="E30" s="67">
         <v>10</v>
       </c>
-      <c r="G30" s="40" t="s">
-        <v>40</v>
+      <c r="G30" s="41" t="s">
+        <v>43</v>
       </c>
       <c r="H30" s="13" t="s">
-        <v>41</v>
+        <v>44</v>
       </c>
       <c r="I30" s="13" t="s">
-        <v>42</v>
-      </c>
-      <c r="K30" s="21"/>
+        <v>45</v>
+      </c>
+      <c r="K30" s="22"/>
     </row>
     <row r="31" ht="15.75" spans="1:12">
-      <c r="A31" s="38"/>
-      <c r="B31" s="51">
+      <c r="A31" s="39"/>
+      <c r="B31" s="52">
         <v>50</v>
       </c>
       <c r="C31" s="10">
@@ -2633,10 +2687,10 @@
       <c r="D31" s="10">
         <v>2.5</v>
       </c>
-      <c r="E31" s="66">
+      <c r="E31" s="67">
         <v>10</v>
       </c>
-      <c r="G31" s="51">
+      <c r="G31" s="52">
         <v>1</v>
       </c>
       <c r="H31" s="17">
@@ -2645,11 +2699,11 @@
       <c r="I31" s="17">
         <v>7</v>
       </c>
-      <c r="K31" s="21"/>
+      <c r="K31" s="22"/>
     </row>
     <row r="32" ht="15.75" spans="1:12">
-      <c r="A32" s="38"/>
-      <c r="B32" s="51">
+      <c r="A32" s="39"/>
+      <c r="B32" s="52">
         <v>75</v>
       </c>
       <c r="C32" s="10">
@@ -2658,10 +2712,10 @@
       <c r="D32" s="10">
         <v>3.5</v>
       </c>
-      <c r="E32" s="66">
+      <c r="E32" s="67">
         <v>10</v>
       </c>
-      <c r="G32" s="51">
+      <c r="G32" s="52">
         <v>2</v>
       </c>
       <c r="H32" s="17">
@@ -2670,25 +2724,25 @@
       <c r="I32" s="17">
         <v>9</v>
       </c>
-      <c r="K32" s="21"/>
+      <c r="K32" s="22"/>
     </row>
     <row r="33" ht="15.75" spans="1:13">
-      <c r="A33" s="38" t="s">
-        <v>43</v>
-      </c>
-      <c r="B33" s="67">
+      <c r="A33" s="39" t="s">
+        <v>46</v>
+      </c>
+      <c r="B33" s="68">
         <v>100</v>
       </c>
       <c r="C33" s="10">
         <v>25</v>
       </c>
-      <c r="D33" s="21">
+      <c r="D33" s="22">
         <v>5</v>
       </c>
-      <c r="E33" s="66">
+      <c r="E33" s="67">
         <v>10</v>
       </c>
-      <c r="G33" s="51">
+      <c r="G33" s="52">
         <v>3</v>
       </c>
       <c r="H33" s="17">
@@ -2697,25 +2751,25 @@
       <c r="I33" s="17">
         <v>11</v>
       </c>
-      <c r="K33" s="21"/>
+      <c r="K33" s="22"/>
     </row>
     <row r="34" ht="15.75" spans="1:13">
-      <c r="A34" s="38" t="s">
-        <v>44</v>
-      </c>
-      <c r="B34" s="51">
+      <c r="A34" s="39" t="s">
+        <v>47</v>
+      </c>
+      <c r="B34" s="52">
         <v>125</v>
       </c>
       <c r="C34" s="10">
         <v>30</v>
       </c>
-      <c r="D34" s="21">
+      <c r="D34" s="22">
         <v>6.5</v>
       </c>
-      <c r="E34" s="66">
+      <c r="E34" s="67">
         <v>10</v>
       </c>
-      <c r="G34" s="51">
+      <c r="G34" s="52">
         <v>4</v>
       </c>
       <c r="H34" s="17">
@@ -2724,23 +2778,23 @@
       <c r="I34" s="17">
         <v>13</v>
       </c>
-      <c r="K34" s="21"/>
+      <c r="K34" s="22"/>
     </row>
     <row r="35" ht="15.75" spans="1:13">
-      <c r="A35" s="38"/>
-      <c r="B35" s="51">
+      <c r="A35" s="39"/>
+      <c r="B35" s="52">
         <v>150</v>
       </c>
       <c r="C35" s="10">
         <v>35</v>
       </c>
-      <c r="D35" s="21">
+      <c r="D35" s="22">
         <v>7.5</v>
       </c>
-      <c r="E35" s="66">
+      <c r="E35" s="67">
         <v>10</v>
       </c>
-      <c r="G35" s="51">
+      <c r="G35" s="52">
         <v>5</v>
       </c>
       <c r="H35" s="17">
@@ -2749,28 +2803,28 @@
       <c r="I35" s="17">
         <v>15</v>
       </c>
-      <c r="K35" s="21"/>
+      <c r="K35" s="22"/>
     </row>
     <row r="36" ht="15.75" spans="1:13">
-      <c r="A36" s="38" t="s">
-        <v>45</v>
-      </c>
-      <c r="B36" s="51">
+      <c r="A36" s="39" t="s">
+        <v>48</v>
+      </c>
+      <c r="B36" s="52">
         <v>175</v>
       </c>
       <c r="C36" s="10">
         <v>40</v>
       </c>
-      <c r="D36" s="21">
+      <c r="D36" s="22">
         <v>8.5</v>
       </c>
-      <c r="E36" s="66">
+      <c r="E36" s="67">
         <v>10</v>
       </c>
       <c r="F36" t="s">
-        <v>46</v>
-      </c>
-      <c r="G36" s="51">
+        <v>49</v>
+      </c>
+      <c r="G36" s="52">
         <v>6</v>
       </c>
       <c r="H36" s="17">
@@ -2779,28 +2833,28 @@
       <c r="I36" s="17">
         <v>17</v>
       </c>
-      <c r="K36" s="21"/>
+      <c r="K36" s="22"/>
     </row>
     <row r="37" ht="15.75" spans="1:13">
-      <c r="A37" s="38" t="s">
-        <v>47</v>
-      </c>
-      <c r="B37" s="51">
+      <c r="A37" s="39" t="s">
+        <v>50</v>
+      </c>
+      <c r="B37" s="52">
         <v>200</v>
       </c>
       <c r="C37" s="10">
         <v>45</v>
       </c>
-      <c r="D37" s="21">
+      <c r="D37" s="22">
         <v>9.5</v>
       </c>
-      <c r="E37" s="66">
+      <c r="E37" s="67">
         <v>11</v>
       </c>
       <c r="F37" t="s">
-        <v>48</v>
-      </c>
-      <c r="G37" s="51">
+        <v>51</v>
+      </c>
+      <c r="G37" s="52">
         <v>7</v>
       </c>
       <c r="H37" s="17">
@@ -2809,26 +2863,26 @@
       <c r="I37" s="17">
         <v>19</v>
       </c>
-      <c r="K37" s="21"/>
+      <c r="K37" s="22"/>
     </row>
     <row r="38" ht="15.75" spans="1:13">
-      <c r="A38" s="38"/>
-      <c r="B38" s="67">
+      <c r="A38" s="39"/>
+      <c r="B38" s="68">
         <v>225</v>
       </c>
       <c r="C38" s="10">
         <v>50</v>
       </c>
-      <c r="D38" s="21">
+      <c r="D38" s="22">
         <v>10.5</v>
       </c>
-      <c r="E38" s="66">
+      <c r="E38" s="67">
         <v>11</v>
       </c>
       <c r="F38" t="s">
-        <v>49</v>
-      </c>
-      <c r="G38" s="51">
+        <v>52</v>
+      </c>
+      <c r="G38" s="52">
         <v>8</v>
       </c>
       <c r="H38" s="17">
@@ -2837,28 +2891,28 @@
       <c r="I38" s="17">
         <v>21</v>
       </c>
-      <c r="K38" s="21"/>
+      <c r="K38" s="22"/>
     </row>
     <row r="39" ht="15.75" spans="1:13">
-      <c r="A39" s="38" t="s">
-        <v>50</v>
-      </c>
-      <c r="B39" s="51">
+      <c r="A39" s="39" t="s">
+        <v>53</v>
+      </c>
+      <c r="B39" s="52">
         <v>250</v>
       </c>
       <c r="C39" s="10">
         <v>55</v>
       </c>
-      <c r="D39" s="21">
+      <c r="D39" s="22">
         <v>11.5</v>
       </c>
-      <c r="E39" s="66">
+      <c r="E39" s="67">
         <v>11</v>
       </c>
       <c r="F39" t="s">
-        <v>51</v>
-      </c>
-      <c r="G39" s="51">
+        <v>54</v>
+      </c>
+      <c r="G39" s="52">
         <v>9</v>
       </c>
       <c r="H39" s="17">
@@ -2867,156 +2921,156 @@
       <c r="I39" s="17">
         <v>23</v>
       </c>
-      <c r="K39" s="21"/>
+      <c r="K39" s="22"/>
     </row>
     <row r="40" ht="16.5" spans="1:13">
-      <c r="A40" s="38" t="s">
-        <v>52</v>
-      </c>
-      <c r="B40" s="51">
+      <c r="A40" s="39" t="s">
+        <v>55</v>
+      </c>
+      <c r="B40" s="52">
         <v>275</v>
       </c>
       <c r="C40" s="10">
         <v>60</v>
       </c>
-      <c r="D40" s="21">
+      <c r="D40" s="22">
         <v>12.5</v>
       </c>
-      <c r="E40" s="66">
+      <c r="E40" s="67">
         <v>11</v>
       </c>
       <c r="F40" t="s">
-        <v>53</v>
-      </c>
-      <c r="G40" s="59">
+        <v>56</v>
+      </c>
+      <c r="G40" s="60">
         <v>10</v>
       </c>
-      <c r="H40" s="32">
+      <c r="H40" s="33">
         <v>57.5</v>
       </c>
-      <c r="I40" s="32">
+      <c r="I40" s="33">
         <v>25</v>
       </c>
-      <c r="K40" s="21"/>
+      <c r="K40" s="22"/>
     </row>
     <row r="41" ht="16.5" spans="1:13">
-      <c r="A41" s="38"/>
-      <c r="B41" s="68">
+      <c r="A41" s="39"/>
+      <c r="B41" s="69">
         <v>300</v>
       </c>
       <c r="C41" s="10">
         <v>65</v>
       </c>
-      <c r="D41" s="21">
+      <c r="D41" s="22">
         <v>13.5</v>
       </c>
-      <c r="E41" s="55">
+      <c r="E41" s="56">
         <v>12</v>
       </c>
       <c r="F41" t="s">
-        <v>54</v>
+        <v>57</v>
       </c>
       <c r="G41" s="10"/>
       <c r="H41" s="10"/>
-      <c r="I41" s="69"/>
-      <c r="J41" s="69"/>
-      <c r="K41" s="20"/>
-      <c r="M41" s="21"/>
+      <c r="I41" s="70"/>
+      <c r="J41" s="70"/>
+      <c r="K41" s="21"/>
+      <c r="M41" s="22"/>
     </row>
     <row r="42" ht="16.5" spans="1:13">
-      <c r="A42" s="70" t="s">
-        <v>55</v>
-      </c>
-      <c r="B42" s="68">
+      <c r="A42" s="71" t="s">
+        <v>58</v>
+      </c>
+      <c r="B42" s="69">
         <v>325</v>
       </c>
       <c r="C42" s="10">
         <v>70</v>
       </c>
-      <c r="D42" s="21">
+      <c r="D42" s="22">
         <v>14.5</v>
       </c>
-      <c r="E42" s="55">
+      <c r="E42" s="56">
         <v>12</v>
       </c>
-      <c r="G42" s="71" t="s">
-        <v>56</v>
-      </c>
-      <c r="H42" s="71" t="s">
-        <v>57</v>
-      </c>
-      <c r="I42" s="72" t="s">
-        <v>58</v>
-      </c>
-      <c r="J42" s="73" t="s">
+      <c r="G42" s="72" t="s">
         <v>59</v>
       </c>
-      <c r="M42" s="21"/>
+      <c r="H42" s="72" t="s">
+        <v>60</v>
+      </c>
+      <c r="I42" s="73" t="s">
+        <v>61</v>
+      </c>
+      <c r="J42" s="74" t="s">
+        <v>62</v>
+      </c>
+      <c r="M42" s="22"/>
     </row>
     <row r="43" ht="15.75" spans="1:13">
-      <c r="A43" s="70" t="s">
-        <v>60</v>
-      </c>
-      <c r="B43" s="51">
+      <c r="A43" s="71" t="s">
+        <v>63</v>
+      </c>
+      <c r="B43" s="52">
         <v>350</v>
       </c>
       <c r="C43" s="10">
         <v>75</v>
       </c>
-      <c r="D43" s="21">
+      <c r="D43" s="22">
         <v>15.5</v>
       </c>
-      <c r="E43" s="55">
+      <c r="E43" s="56">
         <v>12</v>
       </c>
-      <c r="G43" s="74" t="s">
-        <v>61</v>
-      </c>
-      <c r="H43" s="74">
+      <c r="G43" s="75" t="s">
+        <v>64</v>
+      </c>
+      <c r="H43" s="75">
         <v>16</v>
       </c>
       <c r="I43" s="13">
         <v>8</v>
       </c>
-      <c r="J43" s="52">
+      <c r="J43" s="53">
         <f>H43+2*I43</f>
         <v>32</v>
       </c>
-      <c r="M43" s="21"/>
+      <c r="M43" s="22"/>
     </row>
     <row r="44" ht="16.5" spans="1:13">
-      <c r="A44" s="70"/>
-      <c r="B44" s="36">
+      <c r="A44" s="71"/>
+      <c r="B44" s="37">
         <v>375</v>
       </c>
-      <c r="C44" s="60">
+      <c r="C44" s="61">
         <v>80</v>
       </c>
-      <c r="D44" s="60">
+      <c r="D44" s="61">
         <v>10.5</v>
       </c>
-      <c r="E44" s="61">
+      <c r="E44" s="62">
         <v>12</v>
       </c>
-      <c r="G44" s="51" t="s">
-        <v>62</v>
-      </c>
-      <c r="H44" s="51">
+      <c r="G44" s="52" t="s">
+        <v>65</v>
+      </c>
+      <c r="H44" s="52">
         <v>18</v>
       </c>
       <c r="I44" s="17">
         <v>7</v>
       </c>
-      <c r="J44" s="55">
+      <c r="J44" s="56">
         <f>H44+2*I44</f>
         <v>32</v>
       </c>
     </row>
     <row r="45" ht="15.75" spans="1:13">
-      <c r="A45" s="38" t="s">
-        <v>63</v>
-      </c>
-      <c r="B45" s="51">
+      <c r="A45" s="39" t="s">
+        <v>66</v>
+      </c>
+      <c r="B45" s="52">
         <v>400</v>
       </c>
       <c r="C45" s="10">
@@ -3025,196 +3079,196 @@
       <c r="D45" s="10">
         <v>11</v>
       </c>
-      <c r="E45" s="55">
+      <c r="E45" s="56">
         <v>12</v>
       </c>
-      <c r="G45" s="51" t="s">
-        <v>64</v>
-      </c>
-      <c r="H45" s="51">
+      <c r="G45" s="52" t="s">
+        <v>67</v>
+      </c>
+      <c r="H45" s="52">
         <v>21</v>
       </c>
       <c r="I45" s="17">
         <v>5</v>
       </c>
-      <c r="J45" s="55">
+      <c r="J45" s="56">
         <f t="shared" ref="J45:J51" si="0">H45+2*I45</f>
         <v>31</v>
       </c>
     </row>
     <row r="46" ht="15.75" spans="1:13">
-      <c r="A46" s="38"/>
-      <c r="B46" s="51">
+      <c r="A46" s="39"/>
+      <c r="B46" s="52">
         <v>425</v>
       </c>
       <c r="C46" s="10">
         <v>90</v>
       </c>
       <c r="D46" s="10" t="s">
-        <v>65</v>
-      </c>
-      <c r="E46" s="55">
+        <v>68</v>
+      </c>
+      <c r="E46" s="56">
         <v>12</v>
       </c>
-      <c r="G46" s="51" t="s">
-        <v>66</v>
-      </c>
-      <c r="H46" s="51">
+      <c r="G46" s="52" t="s">
+        <v>69</v>
+      </c>
+      <c r="H46" s="52">
         <v>22</v>
       </c>
       <c r="I46" s="17">
         <v>5</v>
       </c>
-      <c r="J46" s="55">
+      <c r="J46" s="56">
         <f t="shared" si="0"/>
         <v>32</v>
       </c>
     </row>
     <row r="47" ht="15.75" spans="1:13">
-      <c r="A47" s="38" t="s">
-        <v>67</v>
-      </c>
-      <c r="B47" s="51">
+      <c r="A47" s="39" t="s">
+        <v>70</v>
+      </c>
+      <c r="B47" s="52">
         <v>450</v>
       </c>
       <c r="C47" s="10">
         <v>95</v>
       </c>
       <c r="D47" s="10" t="s">
-        <v>68</v>
-      </c>
-      <c r="E47" s="55">
+        <v>71</v>
+      </c>
+      <c r="E47" s="56">
         <v>12</v>
       </c>
-      <c r="G47" s="75" t="s">
-        <v>69</v>
-      </c>
-      <c r="H47" s="75">
+      <c r="G47" s="76" t="s">
+        <v>72</v>
+      </c>
+      <c r="H47" s="76">
         <v>16</v>
       </c>
       <c r="I47" s="17">
         <v>8</v>
       </c>
-      <c r="J47" s="55">
+      <c r="J47" s="56">
         <f t="shared" si="0"/>
         <v>32</v>
       </c>
     </row>
     <row r="48" ht="15.75" spans="1:13">
-      <c r="A48" s="38"/>
-      <c r="B48" s="51">
+      <c r="A48" s="39"/>
+      <c r="B48" s="52">
         <v>475</v>
       </c>
       <c r="C48" s="10">
         <v>100</v>
       </c>
       <c r="D48" s="10" t="s">
-        <v>70</v>
-      </c>
-      <c r="E48" s="55">
+        <v>73</v>
+      </c>
+      <c r="E48" s="56">
         <v>12</v>
       </c>
-      <c r="G48" s="51" t="s">
-        <v>71</v>
-      </c>
-      <c r="H48" s="51">
+      <c r="G48" s="52" t="s">
+        <v>74</v>
+      </c>
+      <c r="H48" s="52">
         <v>14</v>
       </c>
       <c r="I48" s="17">
         <v>9</v>
       </c>
-      <c r="J48" s="55">
+      <c r="J48" s="56">
         <f t="shared" si="0"/>
         <v>32</v>
       </c>
     </row>
     <row r="49" ht="15.75" spans="1:14">
-      <c r="B49" s="67">
+      <c r="B49" s="68">
         <v>500</v>
       </c>
       <c r="C49" s="10">
         <v>105</v>
       </c>
-      <c r="D49" s="68" t="s">
-        <v>72</v>
-      </c>
-      <c r="E49" s="55">
+      <c r="D49" s="69" t="s">
+        <v>75</v>
+      </c>
+      <c r="E49" s="56">
         <v>12</v>
       </c>
-      <c r="G49" s="51" t="s">
-        <v>73</v>
-      </c>
-      <c r="H49" s="51">
+      <c r="G49" s="52" t="s">
+        <v>76</v>
+      </c>
+      <c r="H49" s="52">
         <v>20</v>
       </c>
       <c r="I49" s="17">
         <v>6</v>
       </c>
-      <c r="J49" s="55">
+      <c r="J49" s="56">
         <f t="shared" si="0"/>
         <v>32</v>
       </c>
     </row>
     <row r="50" ht="15.75" spans="1:14">
-      <c r="A50" s="38"/>
-      <c r="B50" s="67">
+      <c r="A50" s="39"/>
+      <c r="B50" s="68">
         <v>600</v>
       </c>
-      <c r="C50" s="68"/>
-      <c r="D50" s="68">
+      <c r="C50" s="69"/>
+      <c r="D50" s="69">
         <v>14.5</v>
       </c>
-      <c r="E50" s="55">
+      <c r="E50" s="56">
         <v>13</v>
       </c>
-      <c r="G50" s="51" t="s">
-        <v>74</v>
-      </c>
-      <c r="H50" s="51">
+      <c r="G50" s="52" t="s">
+        <v>77</v>
+      </c>
+      <c r="H50" s="52">
         <v>17</v>
       </c>
       <c r="I50" s="17">
         <v>4</v>
       </c>
-      <c r="J50" s="55">
+      <c r="J50" s="56">
         <f t="shared" si="0"/>
         <v>25</v>
       </c>
     </row>
     <row r="51" ht="16.5" spans="1:14">
-      <c r="B51" s="67">
+      <c r="B51" s="68">
         <v>750</v>
       </c>
-      <c r="C51" s="68"/>
-      <c r="D51" s="68">
+      <c r="C51" s="69"/>
+      <c r="D51" s="69">
         <v>15</v>
       </c>
-      <c r="E51" s="55">
+      <c r="E51" s="56">
         <v>13</v>
       </c>
-      <c r="G51" s="59" t="s">
-        <v>75</v>
-      </c>
-      <c r="H51" s="59">
+      <c r="G51" s="60" t="s">
+        <v>78</v>
+      </c>
+      <c r="H51" s="60">
         <v>26</v>
       </c>
-      <c r="I51" s="32">
+      <c r="I51" s="33">
         <v>3</v>
       </c>
-      <c r="J51" s="61">
+      <c r="J51" s="62">
         <f t="shared" si="0"/>
         <v>32</v>
       </c>
     </row>
     <row r="52" ht="16.5" spans="1:14">
-      <c r="B52" s="36">
+      <c r="B52" s="37">
         <v>1000</v>
       </c>
-      <c r="C52" s="60"/>
-      <c r="D52" s="60">
+      <c r="C52" s="61"/>
+      <c r="D52" s="61">
         <v>15.5</v>
       </c>
-      <c r="E52" s="61">
+      <c r="E52" s="62">
         <v>13</v>
       </c>
       <c r="H52" s="10"/>
@@ -3235,53 +3289,53 @@
         <f>147*2*0.8</f>
         <v>235.2</v>
       </c>
-      <c r="C55" s="76" t="s">
-        <v>76</v>
-      </c>
-      <c r="D55" s="76" t="s">
-        <v>77</v>
-      </c>
-      <c r="E55" s="76" t="s">
-        <v>78</v>
+      <c r="C55" s="77" t="s">
+        <v>79</v>
+      </c>
+      <c r="D55" s="77" t="s">
+        <v>80</v>
+      </c>
+      <c r="E55" s="77" t="s">
+        <v>81</v>
       </c>
       <c r="G55" s="10"/>
-      <c r="H55" s="77" t="s">
-        <v>79</v>
+      <c r="H55" s="78" t="s">
+        <v>82</v>
       </c>
       <c r="I55" t="s">
-        <v>80</v>
-      </c>
-      <c r="J55" s="21"/>
+        <v>83</v>
+      </c>
+      <c r="J55" s="22"/>
     </row>
     <row r="56" ht="90.75" spans="1:14">
-      <c r="C56" s="76" t="s">
-        <v>81</v>
+      <c r="C56" s="77" t="s">
+        <v>84</v>
       </c>
       <c r="E56" s="10"/>
       <c r="F56" s="10"/>
       <c r="G56" s="10"/>
       <c r="H56" s="10" t="s">
-        <v>82</v>
+        <v>85</v>
       </c>
       <c r="I56" t="s">
-        <v>83</v>
+        <v>86</v>
       </c>
       <c r="J56" s="10" t="s">
-        <v>84</v>
+        <v>87</v>
       </c>
     </row>
     <row r="57" spans="1:14">
-      <c r="E57" s="78"/>
+      <c r="E57" s="79"/>
       <c r="F57" s="10"/>
       <c r="G57" s="10"/>
       <c r="H57" s="10" t="s">
-        <v>82</v>
+        <v>85</v>
       </c>
       <c r="I57" t="s">
-        <v>85</v>
+        <v>88</v>
       </c>
       <c r="J57" s="10" t="s">
-        <v>84</v>
+        <v>87</v>
       </c>
     </row>
     <row r="58" spans="1:14">
@@ -3290,13 +3344,13 @@
       <c r="F58" s="10"/>
       <c r="G58" s="10"/>
       <c r="H58" s="10" t="s">
-        <v>82</v>
+        <v>85</v>
       </c>
       <c r="I58" t="s">
-        <v>86</v>
+        <v>89</v>
       </c>
       <c r="J58" s="10" t="s">
-        <v>87</v>
+        <v>90</v>
       </c>
     </row>
     <row r="59" ht="13" customHeight="1" spans="1:14">
@@ -3304,13 +3358,13 @@
       <c r="F59" s="10"/>
       <c r="G59" s="10"/>
       <c r="H59" s="10" t="s">
-        <v>88</v>
-      </c>
-      <c r="I59" s="77" t="s">
-        <v>89</v>
+        <v>91</v>
+      </c>
+      <c r="I59" s="78" t="s">
+        <v>92</v>
       </c>
       <c r="J59" s="10" t="s">
-        <v>87</v>
+        <v>90</v>
       </c>
     </row>
     <row r="60" spans="1:14">
@@ -3318,27 +3372,27 @@
       <c r="F60" s="10"/>
       <c r="G60" s="10"/>
       <c r="H60" s="10" t="s">
-        <v>90</v>
-      </c>
-      <c r="I60" s="77" t="s">
-        <v>91</v>
+        <v>93</v>
+      </c>
+      <c r="I60" s="78" t="s">
+        <v>94</v>
       </c>
       <c r="J60" s="10" t="s">
-        <v>92</v>
+        <v>95</v>
       </c>
     </row>
     <row r="61" ht="15.75" spans="1:14">
-      <c r="A61" s="79"/>
-      <c r="B61" s="80"/>
-      <c r="C61" s="81"/>
-      <c r="D61" s="81"/>
-      <c r="E61" s="21"/>
-      <c r="F61" s="21"/>
-      <c r="G61" s="21"/>
-      <c r="H61" s="21"/>
-      <c r="I61" s="21"/>
-      <c r="J61" s="21"/>
-      <c r="K61" s="21"/>
+      <c r="A61" s="80"/>
+      <c r="B61" s="81"/>
+      <c r="C61" s="82"/>
+      <c r="D61" s="82"/>
+      <c r="E61" s="22"/>
+      <c r="F61" s="22"/>
+      <c r="G61" s="22"/>
+      <c r="H61" s="22"/>
+      <c r="I61" s="22"/>
+      <c r="J61" s="22"/>
+      <c r="K61" s="22"/>
       <c r="M61" s="10"/>
       <c r="N61" s="10"/>
     </row>
@@ -3356,11 +3410,11 @@
     <row r="63" spans="1:14">
       <c r="A63" s="10"/>
       <c r="F63" s="10"/>
-      <c r="G63" s="82" t="s">
-        <v>61</v>
-      </c>
-      <c r="H63" s="82"/>
-      <c r="I63" s="82"/>
+      <c r="G63" s="83" t="s">
+        <v>64</v>
+      </c>
+      <c r="H63" s="83"/>
+      <c r="I63" s="83"/>
       <c r="J63" s="10"/>
       <c r="K63" s="10"/>
       <c r="M63" s="10"/>
@@ -3370,7 +3424,7 @@
       <c r="A64" s="10"/>
       <c r="F64" s="10"/>
       <c r="G64" s="10" t="s">
-        <v>62</v>
+        <v>65</v>
       </c>
       <c r="H64" s="10"/>
       <c r="I64" s="10"/>
@@ -3384,7 +3438,7 @@
       <c r="A65" s="10"/>
       <c r="F65" s="10"/>
       <c r="G65" s="10" t="s">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="H65" s="10"/>
       <c r="I65" s="10"/>
@@ -3398,7 +3452,7 @@
       <c r="A66" s="10"/>
       <c r="F66" s="10"/>
       <c r="G66" s="10" t="s">
-        <v>66</v>
+        <v>69</v>
       </c>
       <c r="H66" s="10"/>
       <c r="I66" s="10"/>
@@ -3408,16 +3462,16 @@
       <c r="N66" s="10"/>
     </row>
     <row r="67" ht="15.75" spans="1:14">
-      <c r="A67" s="79"/>
+      <c r="A67" s="80"/>
       <c r="F67" s="10"/>
-      <c r="G67" s="83" t="s">
-        <v>69</v>
-      </c>
-      <c r="H67" s="83"/>
-      <c r="I67" s="83"/>
-      <c r="J67" s="84"/>
-      <c r="K67" s="84"/>
-      <c r="L67" s="84"/>
+      <c r="G67" s="84" t="s">
+        <v>72</v>
+      </c>
+      <c r="H67" s="84"/>
+      <c r="I67" s="84"/>
+      <c r="J67" s="85"/>
+      <c r="K67" s="85"/>
+      <c r="L67" s="85"/>
       <c r="M67" s="10"/>
       <c r="N67" s="10"/>
     </row>
@@ -3425,7 +3479,7 @@
       <c r="A68" s="10"/>
       <c r="F68" s="10"/>
       <c r="G68" s="10" t="s">
-        <v>71</v>
+        <v>74</v>
       </c>
       <c r="H68" s="10"/>
       <c r="I68" s="10"/>
@@ -3438,7 +3492,7 @@
       <c r="A69" s="10"/>
       <c r="F69" s="10"/>
       <c r="G69" s="10" t="s">
-        <v>74</v>
+        <v>77</v>
       </c>
       <c r="H69" s="10"/>
       <c r="I69" s="10"/>
@@ -3452,7 +3506,7 @@
       <c r="A70" s="10"/>
       <c r="F70" s="10"/>
       <c r="G70" s="10" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="H70" s="10"/>
       <c r="I70" s="10"/>
@@ -3466,7 +3520,7 @@
       <c r="A71" s="10"/>
       <c r="F71" s="10"/>
       <c r="G71" s="10" t="s">
-        <v>75</v>
+        <v>78</v>
       </c>
       <c r="H71" s="10"/>
       <c r="I71" s="10"/>
@@ -3493,8 +3547,8 @@
     </row>
     <row r="74" spans="1:14">
       <c r="A74" s="10"/>
-      <c r="F74" s="69"/>
-      <c r="G74" s="69"/>
+      <c r="F74" s="70"/>
+      <c r="G74" s="70"/>
       <c r="H74" s="10">
         <v>5</v>
       </c>
@@ -3507,7 +3561,7 @@
     <row r="75" spans="1:14">
       <c r="F75" s="10"/>
       <c r="G75" s="10"/>
-      <c r="H75" s="78"/>
+      <c r="H75" s="79"/>
       <c r="I75" s="10"/>
       <c r="J75" s="10"/>
       <c r="K75" s="10"/>
@@ -3575,7 +3629,7 @@
       <c r="K83" s="10"/>
     </row>
     <row r="84" spans="1:11">
-      <c r="F84" s="85"/>
+      <c r="F84" s="86"/>
       <c r="G84" s="10"/>
       <c r="H84" s="10"/>
       <c r="I84" s="10"/>
@@ -3612,7 +3666,7 @@
       <c r="C87" s="10"/>
       <c r="D87" s="10"/>
       <c r="E87" s="10"/>
-      <c r="F87" s="85"/>
+      <c r="F87" s="86"/>
       <c r="G87" s="10"/>
       <c r="H87" s="10"/>
       <c r="I87" s="10"/>
@@ -3657,7 +3711,7 @@
       <c r="C92" s="10"/>
       <c r="D92" s="10"/>
       <c r="E92" s="10"/>
-      <c r="F92" s="77"/>
+      <c r="F92" s="78"/>
     </row>
     <row r="93" spans="1:11">
       <c r="C93" s="10"/>
@@ -3753,37 +3807,37 @@
     <row r="2" s="1" customFormat="1" ht="19.5" spans="1:15">
       <c r="A2" s="4"/>
       <c r="B2" s="5" t="s">
-        <v>93</v>
+        <v>96</v>
       </c>
       <c r="C2" s="5" t="s">
-        <v>94</v>
+        <v>97</v>
       </c>
       <c r="D2" s="5" t="s">
-        <v>95</v>
+        <v>98</v>
       </c>
       <c r="E2" s="5" t="s">
-        <v>96</v>
+        <v>99</v>
       </c>
       <c r="F2" s="5" t="s">
-        <v>97</v>
+        <v>100</v>
       </c>
       <c r="G2" s="5" t="s">
-        <v>98</v>
+        <v>101</v>
       </c>
       <c r="H2" s="5" t="s">
-        <v>99</v>
+        <v>102</v>
       </c>
       <c r="I2" s="5" t="s">
-        <v>100</v>
+        <v>103</v>
       </c>
       <c r="J2" s="5" t="s">
-        <v>101</v>
+        <v>104</v>
       </c>
       <c r="K2" s="5" t="s">
-        <v>102</v>
+        <v>105</v>
       </c>
       <c r="L2" s="5" t="s">
-        <v>103</v>
+        <v>106</v>
       </c>
       <c r="M2" s="5"/>
       <c r="N2" s="5"/>
@@ -3794,37 +3848,37 @@
         <v>2</v>
       </c>
       <c r="B3" s="7" t="s">
-        <v>104</v>
+        <v>107</v>
       </c>
       <c r="C3" s="7" t="s">
-        <v>104</v>
+        <v>107</v>
       </c>
       <c r="D3" s="7" t="s">
-        <v>105</v>
+        <v>108</v>
       </c>
       <c r="E3" s="7" t="s">
-        <v>106</v>
+        <v>109</v>
       </c>
       <c r="F3" s="7" t="s">
-        <v>104</v>
+        <v>107</v>
       </c>
       <c r="G3" s="7" t="s">
-        <v>104</v>
+        <v>107</v>
       </c>
       <c r="H3" s="7" t="s">
+        <v>110</v>
+      </c>
+      <c r="I3" s="7" t="s">
+        <v>111</v>
+      </c>
+      <c r="J3" s="7" t="s">
         <v>107</v>
       </c>
-      <c r="I3" s="7" t="s">
-        <v>108</v>
-      </c>
-      <c r="J3" s="7" t="s">
-        <v>104</v>
-      </c>
       <c r="K3" s="7" t="s">
-        <v>107</v>
+        <v>110</v>
       </c>
       <c r="L3" s="7" t="s">
-        <v>107</v>
+        <v>110</v>
       </c>
       <c r="M3" s="7"/>
       <c r="N3" s="7"/>
@@ -3835,37 +3889,37 @@
         <v>3</v>
       </c>
       <c r="B4" s="7" t="s">
+        <v>110</v>
+      </c>
+      <c r="C4" s="7" t="s">
         <v>107</v>
       </c>
-      <c r="C4" s="7" t="s">
-        <v>104</v>
-      </c>
       <c r="D4" s="7" t="s">
+        <v>110</v>
+      </c>
+      <c r="E4" s="7" t="s">
+        <v>111</v>
+      </c>
+      <c r="F4" s="7" t="s">
+        <v>110</v>
+      </c>
+      <c r="G4" s="7" t="s">
+        <v>110</v>
+      </c>
+      <c r="H4" s="7" t="s">
         <v>107</v>
       </c>
-      <c r="E4" s="7" t="s">
-        <v>108</v>
-      </c>
-      <c r="F4" s="7" t="s">
+      <c r="I4" s="7" t="s">
+        <v>111</v>
+      </c>
+      <c r="J4" s="7" t="s">
         <v>107</v>
       </c>
-      <c r="G4" s="7" t="s">
-        <v>107</v>
-      </c>
-      <c r="H4" s="7" t="s">
-        <v>104</v>
-      </c>
-      <c r="I4" s="7" t="s">
-        <v>108</v>
-      </c>
-      <c r="J4" s="7" t="s">
-        <v>104</v>
-      </c>
       <c r="K4" s="7" t="s">
-        <v>107</v>
+        <v>110</v>
       </c>
       <c r="L4" s="7" t="s">
-        <v>107</v>
+        <v>110</v>
       </c>
       <c r="M4" s="7"/>
       <c r="N4" s="7"/>
@@ -3876,35 +3930,35 @@
         <v>4</v>
       </c>
       <c r="B5" s="8" t="s">
-        <v>109</v>
+        <v>112</v>
       </c>
       <c r="C5" s="7" t="s">
-        <v>107</v>
+        <v>110</v>
       </c>
       <c r="D5" s="7"/>
       <c r="E5" s="7" t="s">
-        <v>108</v>
+        <v>111</v>
       </c>
       <c r="F5" s="8" t="s">
-        <v>109</v>
+        <v>112</v>
       </c>
       <c r="G5" s="7" t="s">
+        <v>110</v>
+      </c>
+      <c r="H5" s="7" t="s">
+        <v>110</v>
+      </c>
+      <c r="I5" s="7" t="s">
+        <v>111</v>
+      </c>
+      <c r="J5" s="7" t="s">
+        <v>110</v>
+      </c>
+      <c r="K5" s="9" t="s">
+        <v>113</v>
+      </c>
+      <c r="L5" s="7" t="s">
         <v>107</v>
-      </c>
-      <c r="H5" s="7" t="s">
-        <v>107</v>
-      </c>
-      <c r="I5" s="7" t="s">
-        <v>108</v>
-      </c>
-      <c r="J5" s="7" t="s">
-        <v>107</v>
-      </c>
-      <c r="K5" s="9" t="s">
-        <v>110</v>
-      </c>
-      <c r="L5" s="7" t="s">
-        <v>104</v>
       </c>
       <c r="M5" s="7"/>
       <c r="N5" s="7"/>
@@ -3915,33 +3969,33 @@
         <v>5</v>
       </c>
       <c r="B6" s="7" t="s">
+        <v>110</v>
+      </c>
+      <c r="C6" s="8" t="s">
+        <v>112</v>
+      </c>
+      <c r="D6" s="7" t="s">
+        <v>110</v>
+      </c>
+      <c r="E6" s="7" t="s">
+        <v>111</v>
+      </c>
+      <c r="F6" s="7" t="s">
+        <v>110</v>
+      </c>
+      <c r="G6" s="8" t="s">
+        <v>112</v>
+      </c>
+      <c r="H6" s="7" t="s">
         <v>107</v>
-      </c>
-      <c r="C6" s="8" t="s">
-        <v>109</v>
-      </c>
-      <c r="D6" s="7" t="s">
-        <v>107</v>
-      </c>
-      <c r="E6" s="7" t="s">
-        <v>108</v>
-      </c>
-      <c r="F6" s="7" t="s">
-        <v>107</v>
-      </c>
-      <c r="G6" s="8" t="s">
-        <v>109</v>
-      </c>
-      <c r="H6" s="7" t="s">
-        <v>104</v>
       </c>
       <c r="I6" s="7"/>
       <c r="J6" s="7" t="s">
-        <v>107</v>
+        <v>110</v>
       </c>
       <c r="K6" s="7"/>
       <c r="L6" s="7" t="s">
-        <v>107</v>
+        <v>110</v>
       </c>
       <c r="M6" s="7"/>
       <c r="N6" s="7"/>
@@ -3952,37 +4006,37 @@
         <v>6</v>
       </c>
       <c r="B7" s="7" t="s">
-        <v>111</v>
+        <v>114</v>
       </c>
       <c r="C7" s="7" t="s">
-        <v>111</v>
+        <v>114</v>
       </c>
       <c r="D7" s="7" t="s">
-        <v>111</v>
+        <v>114</v>
       </c>
       <c r="E7" s="7" t="s">
-        <v>111</v>
+        <v>114</v>
       </c>
       <c r="F7" s="7" t="s">
-        <v>111</v>
+        <v>114</v>
       </c>
       <c r="G7" s="7" t="s">
-        <v>111</v>
+        <v>114</v>
       </c>
       <c r="H7" s="7" t="s">
-        <v>111</v>
+        <v>114</v>
       </c>
       <c r="I7" s="7" t="s">
-        <v>111</v>
+        <v>114</v>
       </c>
       <c r="J7" s="7" t="s">
-        <v>111</v>
+        <v>114</v>
       </c>
       <c r="K7" s="7" t="s">
-        <v>111</v>
+        <v>114</v>
       </c>
       <c r="L7" s="7" t="s">
-        <v>111</v>
+        <v>114</v>
       </c>
       <c r="M7" s="7"/>
       <c r="N7" s="7"/>
@@ -3994,30 +4048,30 @@
       </c>
       <c r="B8" s="7"/>
       <c r="C8" s="7" t="s">
-        <v>107</v>
+        <v>110</v>
       </c>
       <c r="D8" s="7"/>
       <c r="E8" s="7" t="s">
-        <v>108</v>
+        <v>111</v>
       </c>
       <c r="F8" s="7"/>
       <c r="G8" s="7" t="s">
-        <v>107</v>
+        <v>110</v>
       </c>
       <c r="H8" s="7" t="s">
-        <v>107</v>
+        <v>110</v>
       </c>
       <c r="I8" s="7" t="s">
-        <v>108</v>
+        <v>111</v>
       </c>
       <c r="J8" s="7" t="s">
-        <v>107</v>
+        <v>110</v>
       </c>
       <c r="K8" s="7" t="s">
-        <v>107</v>
+        <v>110</v>
       </c>
       <c r="L8" s="7" t="s">
-        <v>107</v>
+        <v>110</v>
       </c>
       <c r="M8" s="7"/>
       <c r="N8" s="7"/>
@@ -4031,7 +4085,7 @@
       <c r="C9" s="7"/>
       <c r="D9" s="7"/>
       <c r="E9" s="7" t="s">
-        <v>112</v>
+        <v>115</v>
       </c>
       <c r="F9" s="7"/>
       <c r="G9" s="7"/>
@@ -4049,24 +4103,24 @@
         <v>9</v>
       </c>
       <c r="B10" s="7" t="s">
-        <v>107</v>
+        <v>110</v>
       </c>
       <c r="C10" s="7"/>
       <c r="D10" s="7" t="s">
-        <v>107</v>
+        <v>110</v>
       </c>
       <c r="E10" s="7" t="s">
-        <v>113</v>
+        <v>116</v>
       </c>
       <c r="F10" s="7"/>
       <c r="G10" s="7"/>
       <c r="H10" s="7"/>
       <c r="I10" s="7" t="s">
-        <v>108</v>
+        <v>111</v>
       </c>
       <c r="J10" s="7"/>
       <c r="K10" s="7" t="s">
-        <v>107</v>
+        <v>110</v>
       </c>
       <c r="L10" s="7"/>
       <c r="M10" s="7"/>
@@ -4078,35 +4132,35 @@
         <v>10</v>
       </c>
       <c r="B11" s="7" t="s">
-        <v>114</v>
+        <v>117</v>
       </c>
       <c r="C11" s="7" t="s">
-        <v>114</v>
+        <v>117</v>
       </c>
       <c r="D11" s="7" t="s">
-        <v>114</v>
+        <v>117</v>
       </c>
       <c r="E11" s="7" t="s">
-        <v>114</v>
+        <v>117</v>
       </c>
       <c r="F11" s="7" t="s">
-        <v>114</v>
+        <v>117</v>
       </c>
       <c r="G11" s="7" t="s">
-        <v>114</v>
+        <v>117</v>
       </c>
       <c r="H11" s="7" t="s">
-        <v>114</v>
+        <v>117</v>
       </c>
       <c r="I11" s="7" t="s">
-        <v>114</v>
+        <v>117</v>
       </c>
       <c r="J11" s="7"/>
       <c r="K11" s="7" t="s">
-        <v>114</v>
+        <v>117</v>
       </c>
       <c r="L11" s="7" t="s">
-        <v>114</v>
+        <v>117</v>
       </c>
       <c r="M11" s="7"/>
       <c r="N11" s="7"/>

</xml_diff>

<commit_message>
Design: Worked on Wizard and Spell Fonts.
</commit_message>
<xml_diff>
--- a/Design/Tables.xlsx
+++ b/Design/Tables.xlsx
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="199" uniqueCount="118">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="198" uniqueCount="117">
   <si>
     <t>Action Points</t>
   </si>
@@ -150,9 +150,6 @@
       </rPr>
       <t>AoE 2</t>
     </r>
-  </si>
-  <si>
-    <t>Homecoming 2d6</t>
   </si>
   <si>
     <r>
@@ -2290,8 +2287,9 @@
       <c r="F9" s="27">
         <v>0</v>
       </c>
-      <c r="G9" t="s">
-        <v>12</v>
+      <c r="G9">
+        <f>7*3.5</f>
+        <v>24.5</v>
       </c>
       <c r="H9" s="20"/>
       <c r="J9" s="28"/>
@@ -2305,10 +2303,10 @@
         <v>1</v>
       </c>
       <c r="C10" s="18" t="s">
+        <v>12</v>
+      </c>
+      <c r="D10" s="29" t="s">
         <v>13</v>
-      </c>
-      <c r="D10" s="29" t="s">
-        <v>14</v>
       </c>
       <c r="E10" s="29">
         <v>8.5</v>
@@ -2327,10 +2325,10 @@
         <v>1</v>
       </c>
       <c r="C11" s="14" t="s">
+        <v>14</v>
+      </c>
+      <c r="D11" s="17" t="s">
         <v>15</v>
-      </c>
-      <c r="D11" s="17" t="s">
-        <v>16</v>
       </c>
       <c r="E11" s="17">
         <v>11</v>
@@ -2338,10 +2336,7 @@
       <c r="F11" s="17">
         <v>-2</v>
       </c>
-      <c r="G11">
-        <f>5*3.5</f>
-        <v>17.5</v>
-      </c>
+      <c r="G11"/>
       <c r="H11" s="22"/>
       <c r="K11" s="21"/>
     </row>
@@ -2353,10 +2348,10 @@
         <v>1</v>
       </c>
       <c r="C12" s="30" t="s">
+        <v>16</v>
+      </c>
+      <c r="D12" s="32" t="s">
         <v>17</v>
-      </c>
-      <c r="D12" s="32" t="s">
-        <v>18</v>
       </c>
       <c r="E12" s="32">
         <v>14</v>
@@ -2365,8 +2360,8 @@
         <v>-3</v>
       </c>
       <c r="G12" s="10">
-        <f>3*5.5</f>
-        <v>16.5</v>
+        <f>18+6</f>
+        <v>24</v>
       </c>
       <c r="H12" s="21"/>
       <c r="I12" s="21"/>
@@ -2378,7 +2373,7 @@
         <v>1</v>
       </c>
       <c r="B13" s="35" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C13" s="36">
         <v>6</v>
@@ -2392,7 +2387,10 @@
       <c r="F13" s="13">
         <v>3</v>
       </c>
-      <c r="G13" s="10"/>
+      <c r="G13" s="10">
+        <f>6*4.5</f>
+        <v>27</v>
+      </c>
       <c r="H13" s="21"/>
       <c r="I13" s="21"/>
       <c r="J13" s="21"/>
@@ -2403,7 +2401,7 @@
         <v>1</v>
       </c>
       <c r="B14" s="30" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="C14" s="38">
         <v>8</v>
@@ -2417,7 +2415,10 @@
       <c r="F14" s="33">
         <v>5.5</v>
       </c>
-      <c r="G14" s="10"/>
+      <c r="G14" s="10">
+        <f>6*3.5</f>
+        <v>21</v>
+      </c>
       <c r="H14" s="21"/>
       <c r="I14" s="21"/>
       <c r="J14" s="21"/>
@@ -2440,7 +2441,7 @@
       <c r="A16" s="41"/>
       <c r="B16" s="42"/>
       <c r="C16" s="43" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="D16" s="44"/>
       <c r="E16" s="44"/>
@@ -2449,13 +2450,13 @@
     </row>
     <row r="17" ht="16.5" spans="1:12">
       <c r="A17" s="46" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B17" s="47" t="s">
         <v>1</v>
       </c>
       <c r="C17" s="48" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D17" s="49"/>
       <c r="E17" s="49"/>
@@ -2471,10 +2472,10 @@
         <v>0</v>
       </c>
       <c r="C18" s="52" t="s">
+        <v>23</v>
+      </c>
+      <c r="D18" s="10" t="s">
         <v>24</v>
-      </c>
-      <c r="D18" s="10" t="s">
-        <v>25</v>
       </c>
       <c r="E18" s="42"/>
       <c r="F18" s="53"/>
@@ -2488,10 +2489,10 @@
         <v>0</v>
       </c>
       <c r="C19" s="54" t="s">
+        <v>25</v>
+      </c>
+      <c r="D19" s="55" t="s">
         <v>26</v>
-      </c>
-      <c r="D19" s="55" t="s">
-        <v>27</v>
       </c>
       <c r="E19" s="10"/>
       <c r="F19" s="56"/>
@@ -2518,16 +2519,16 @@
         <v>1</v>
       </c>
       <c r="C21" s="52" t="s">
+        <v>27</v>
+      </c>
+      <c r="D21" s="10" t="s">
         <v>28</v>
       </c>
-      <c r="D21" s="10" t="s">
+      <c r="E21" s="10" t="s">
         <v>29</v>
       </c>
-      <c r="E21" s="10" t="s">
+      <c r="F21" s="56" t="s">
         <v>30</v>
-      </c>
-      <c r="F21" s="56" t="s">
-        <v>31</v>
       </c>
     </row>
     <row r="22" spans="1:12">
@@ -2538,10 +2539,10 @@
         <v>1</v>
       </c>
       <c r="C22" s="52" t="s">
+        <v>31</v>
+      </c>
+      <c r="D22" s="10" t="s">
         <v>32</v>
-      </c>
-      <c r="D22" s="10" t="s">
-        <v>33</v>
       </c>
       <c r="E22" s="10"/>
       <c r="F22" s="56"/>
@@ -2563,10 +2564,10 @@
         <v>1</v>
       </c>
       <c r="B24" s="63" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C24" s="41" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="D24" s="64"/>
       <c r="E24" s="64"/>
@@ -2578,13 +2579,13 @@
         <v>1</v>
       </c>
       <c r="B25" s="65" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="C25" s="37" t="s">
+        <v>34</v>
+      </c>
+      <c r="D25" s="31" t="s">
         <v>35</v>
-      </c>
-      <c r="D25" s="31" t="s">
-        <v>36</v>
       </c>
       <c r="E25" s="31"/>
       <c r="F25" s="65"/>
@@ -2619,7 +2620,7 @@
     <row r="28" ht="16.5" spans="1:12">
       <c r="A28" s="22"/>
       <c r="C28" s="34" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="D28" s="63"/>
       <c r="F28" s="22"/>
@@ -2632,20 +2633,20 @@
     <row r="29" ht="16.5" spans="1:12">
       <c r="A29" s="39"/>
       <c r="B29" s="41" t="s">
+        <v>37</v>
+      </c>
+      <c r="C29" s="42" t="s">
         <v>38</v>
       </c>
-      <c r="C29" s="42" t="s">
+      <c r="D29" s="42" t="s">
         <v>39</v>
       </c>
-      <c r="D29" s="42" t="s">
+      <c r="E29" s="63" t="s">
         <v>40</v>
-      </c>
-      <c r="E29" s="63" t="s">
-        <v>41</v>
       </c>
       <c r="G29" s="10"/>
       <c r="H29" s="10" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="I29" s="10"/>
       <c r="J29" s="10"/>
@@ -2666,13 +2667,13 @@
         <v>10</v>
       </c>
       <c r="G30" s="41" t="s">
+        <v>42</v>
+      </c>
+      <c r="H30" s="13" t="s">
         <v>43</v>
       </c>
-      <c r="H30" s="13" t="s">
+      <c r="I30" s="13" t="s">
         <v>44</v>
-      </c>
-      <c r="I30" s="13" t="s">
-        <v>45</v>
       </c>
       <c r="K30" s="22"/>
     </row>
@@ -2728,7 +2729,7 @@
     </row>
     <row r="33" ht="15.75" spans="1:13">
       <c r="A33" s="39" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="B33" s="68">
         <v>100</v>
@@ -2755,7 +2756,7 @@
     </row>
     <row r="34" ht="15.75" spans="1:13">
       <c r="A34" s="39" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="B34" s="52">
         <v>125</v>
@@ -2807,7 +2808,7 @@
     </row>
     <row r="36" ht="15.75" spans="1:13">
       <c r="A36" s="39" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B36" s="52">
         <v>175</v>
@@ -2822,7 +2823,7 @@
         <v>10</v>
       </c>
       <c r="F36" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="G36" s="52">
         <v>6</v>
@@ -2837,7 +2838,7 @@
     </row>
     <row r="37" ht="15.75" spans="1:13">
       <c r="A37" s="39" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="B37" s="52">
         <v>200</v>
@@ -2852,7 +2853,7 @@
         <v>11</v>
       </c>
       <c r="F37" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="G37" s="52">
         <v>7</v>
@@ -2880,7 +2881,7 @@
         <v>11</v>
       </c>
       <c r="F38" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="G38" s="52">
         <v>8</v>
@@ -2895,7 +2896,7 @@
     </row>
     <row r="39" ht="15.75" spans="1:13">
       <c r="A39" s="39" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="B39" s="52">
         <v>250</v>
@@ -2910,7 +2911,7 @@
         <v>11</v>
       </c>
       <c r="F39" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="G39" s="52">
         <v>9</v>
@@ -2925,7 +2926,7 @@
     </row>
     <row r="40" ht="16.5" spans="1:13">
       <c r="A40" s="39" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="B40" s="52">
         <v>275</v>
@@ -2940,7 +2941,7 @@
         <v>11</v>
       </c>
       <c r="F40" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="G40" s="60">
         <v>10</v>
@@ -2968,7 +2969,7 @@
         <v>12</v>
       </c>
       <c r="F41" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="G41" s="10"/>
       <c r="H41" s="10"/>
@@ -2979,7 +2980,7 @@
     </row>
     <row r="42" ht="16.5" spans="1:13">
       <c r="A42" s="71" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B42" s="69">
         <v>325</v>
@@ -2994,22 +2995,22 @@
         <v>12</v>
       </c>
       <c r="G42" s="72" t="s">
+        <v>58</v>
+      </c>
+      <c r="H42" s="72" t="s">
         <v>59</v>
       </c>
-      <c r="H42" s="72" t="s">
+      <c r="I42" s="73" t="s">
         <v>60</v>
       </c>
-      <c r="I42" s="73" t="s">
+      <c r="J42" s="74" t="s">
         <v>61</v>
-      </c>
-      <c r="J42" s="74" t="s">
-        <v>62</v>
       </c>
       <c r="M42" s="22"/>
     </row>
     <row r="43" ht="15.75" spans="1:13">
       <c r="A43" s="71" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="B43" s="52">
         <v>350</v>
@@ -3024,7 +3025,7 @@
         <v>12</v>
       </c>
       <c r="G43" s="75" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="H43" s="75">
         <v>16</v>
@@ -3053,7 +3054,7 @@
         <v>12</v>
       </c>
       <c r="G44" s="52" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="H44" s="52">
         <v>18</v>
@@ -3068,7 +3069,7 @@
     </row>
     <row r="45" ht="15.75" spans="1:13">
       <c r="A45" s="39" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="B45" s="52">
         <v>400</v>
@@ -3083,7 +3084,7 @@
         <v>12</v>
       </c>
       <c r="G45" s="52" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="H45" s="52">
         <v>21</v>
@@ -3105,13 +3106,13 @@
         <v>90</v>
       </c>
       <c r="D46" s="10" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E46" s="56">
         <v>12</v>
       </c>
       <c r="G46" s="52" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="H46" s="52">
         <v>22</v>
@@ -3126,7 +3127,7 @@
     </row>
     <row r="47" ht="15.75" spans="1:13">
       <c r="A47" s="39" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="B47" s="52">
         <v>450</v>
@@ -3135,13 +3136,13 @@
         <v>95</v>
       </c>
       <c r="D47" s="10" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="E47" s="56">
         <v>12</v>
       </c>
       <c r="G47" s="76" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="H47" s="76">
         <v>16</v>
@@ -3163,13 +3164,13 @@
         <v>100</v>
       </c>
       <c r="D48" s="10" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="E48" s="56">
         <v>12</v>
       </c>
       <c r="G48" s="52" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="H48" s="52">
         <v>14</v>
@@ -3190,13 +3191,13 @@
         <v>105</v>
       </c>
       <c r="D49" s="69" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="E49" s="56">
         <v>12</v>
       </c>
       <c r="G49" s="52" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="H49" s="52">
         <v>20</v>
@@ -3222,7 +3223,7 @@
         <v>13</v>
       </c>
       <c r="G50" s="52" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="H50" s="52">
         <v>17</v>
@@ -3247,7 +3248,7 @@
         <v>13</v>
       </c>
       <c r="G51" s="60" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="H51" s="60">
         <v>26</v>
@@ -3290,38 +3291,38 @@
         <v>235.2</v>
       </c>
       <c r="C55" s="77" t="s">
+        <v>78</v>
+      </c>
+      <c r="D55" s="77" t="s">
         <v>79</v>
       </c>
-      <c r="D55" s="77" t="s">
+      <c r="E55" s="77" t="s">
         <v>80</v>
-      </c>
-      <c r="E55" s="77" t="s">
-        <v>81</v>
       </c>
       <c r="G55" s="10"/>
       <c r="H55" s="78" t="s">
+        <v>81</v>
+      </c>
+      <c r="I55" t="s">
         <v>82</v>
-      </c>
-      <c r="I55" t="s">
-        <v>83</v>
       </c>
       <c r="J55" s="22"/>
     </row>
     <row r="56" ht="90.75" spans="1:14">
       <c r="C56" s="77" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="E56" s="10"/>
       <c r="F56" s="10"/>
       <c r="G56" s="10"/>
       <c r="H56" s="10" t="s">
+        <v>84</v>
+      </c>
+      <c r="I56" t="s">
         <v>85</v>
       </c>
-      <c r="I56" t="s">
+      <c r="J56" s="10" t="s">
         <v>86</v>
-      </c>
-      <c r="J56" s="10" t="s">
-        <v>87</v>
       </c>
     </row>
     <row r="57" spans="1:14">
@@ -3329,13 +3330,13 @@
       <c r="F57" s="10"/>
       <c r="G57" s="10"/>
       <c r="H57" s="10" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="I57" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="J57" s="10" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
     </row>
     <row r="58" spans="1:14">
@@ -3344,13 +3345,13 @@
       <c r="F58" s="10"/>
       <c r="G58" s="10"/>
       <c r="H58" s="10" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="I58" t="s">
+        <v>88</v>
+      </c>
+      <c r="J58" s="10" t="s">
         <v>89</v>
-      </c>
-      <c r="J58" s="10" t="s">
-        <v>90</v>
       </c>
     </row>
     <row r="59" ht="13" customHeight="1" spans="1:14">
@@ -3358,13 +3359,13 @@
       <c r="F59" s="10"/>
       <c r="G59" s="10"/>
       <c r="H59" s="10" t="s">
+        <v>90</v>
+      </c>
+      <c r="I59" s="78" t="s">
         <v>91</v>
       </c>
-      <c r="I59" s="78" t="s">
-        <v>92</v>
-      </c>
       <c r="J59" s="10" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
     </row>
     <row r="60" spans="1:14">
@@ -3372,13 +3373,13 @@
       <c r="F60" s="10"/>
       <c r="G60" s="10"/>
       <c r="H60" s="10" t="s">
+        <v>92</v>
+      </c>
+      <c r="I60" s="78" t="s">
         <v>93</v>
       </c>
-      <c r="I60" s="78" t="s">
+      <c r="J60" s="10" t="s">
         <v>94</v>
-      </c>
-      <c r="J60" s="10" t="s">
-        <v>95</v>
       </c>
     </row>
     <row r="61" ht="15.75" spans="1:14">
@@ -3411,7 +3412,7 @@
       <c r="A63" s="10"/>
       <c r="F63" s="10"/>
       <c r="G63" s="83" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="H63" s="83"/>
       <c r="I63" s="83"/>
@@ -3424,7 +3425,7 @@
       <c r="A64" s="10"/>
       <c r="F64" s="10"/>
       <c r="G64" s="10" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="H64" s="10"/>
       <c r="I64" s="10"/>
@@ -3438,7 +3439,7 @@
       <c r="A65" s="10"/>
       <c r="F65" s="10"/>
       <c r="G65" s="10" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="H65" s="10"/>
       <c r="I65" s="10"/>
@@ -3452,7 +3453,7 @@
       <c r="A66" s="10"/>
       <c r="F66" s="10"/>
       <c r="G66" s="10" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="H66" s="10"/>
       <c r="I66" s="10"/>
@@ -3465,7 +3466,7 @@
       <c r="A67" s="80"/>
       <c r="F67" s="10"/>
       <c r="G67" s="84" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="H67" s="84"/>
       <c r="I67" s="84"/>
@@ -3479,7 +3480,7 @@
       <c r="A68" s="10"/>
       <c r="F68" s="10"/>
       <c r="G68" s="10" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="H68" s="10"/>
       <c r="I68" s="10"/>
@@ -3492,7 +3493,7 @@
       <c r="A69" s="10"/>
       <c r="F69" s="10"/>
       <c r="G69" s="10" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="H69" s="10"/>
       <c r="I69" s="10"/>
@@ -3506,7 +3507,7 @@
       <c r="A70" s="10"/>
       <c r="F70" s="10"/>
       <c r="G70" s="10" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="H70" s="10"/>
       <c r="I70" s="10"/>
@@ -3520,7 +3521,7 @@
       <c r="A71" s="10"/>
       <c r="F71" s="10"/>
       <c r="G71" s="10" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="H71" s="10"/>
       <c r="I71" s="10"/>
@@ -3807,37 +3808,37 @@
     <row r="2" s="1" customFormat="1" ht="19.5" spans="1:15">
       <c r="A2" s="4"/>
       <c r="B2" s="5" t="s">
+        <v>95</v>
+      </c>
+      <c r="C2" s="5" t="s">
         <v>96</v>
       </c>
-      <c r="C2" s="5" t="s">
+      <c r="D2" s="5" t="s">
         <v>97</v>
       </c>
-      <c r="D2" s="5" t="s">
+      <c r="E2" s="5" t="s">
         <v>98</v>
       </c>
-      <c r="E2" s="5" t="s">
+      <c r="F2" s="5" t="s">
         <v>99</v>
       </c>
-      <c r="F2" s="5" t="s">
+      <c r="G2" s="5" t="s">
         <v>100</v>
       </c>
-      <c r="G2" s="5" t="s">
+      <c r="H2" s="5" t="s">
         <v>101</v>
       </c>
-      <c r="H2" s="5" t="s">
+      <c r="I2" s="5" t="s">
         <v>102</v>
       </c>
-      <c r="I2" s="5" t="s">
+      <c r="J2" s="5" t="s">
         <v>103</v>
       </c>
-      <c r="J2" s="5" t="s">
+      <c r="K2" s="5" t="s">
         <v>104</v>
       </c>
-      <c r="K2" s="5" t="s">
+      <c r="L2" s="5" t="s">
         <v>105</v>
-      </c>
-      <c r="L2" s="5" t="s">
-        <v>106</v>
       </c>
       <c r="M2" s="5"/>
       <c r="N2" s="5"/>
@@ -3848,37 +3849,37 @@
         <v>2</v>
       </c>
       <c r="B3" s="7" t="s">
+        <v>106</v>
+      </c>
+      <c r="C3" s="7" t="s">
+        <v>106</v>
+      </c>
+      <c r="D3" s="7" t="s">
         <v>107</v>
       </c>
-      <c r="C3" s="7" t="s">
-        <v>107</v>
-      </c>
-      <c r="D3" s="7" t="s">
+      <c r="E3" s="7" t="s">
         <v>108</v>
       </c>
-      <c r="E3" s="7" t="s">
+      <c r="F3" s="7" t="s">
+        <v>106</v>
+      </c>
+      <c r="G3" s="7" t="s">
+        <v>106</v>
+      </c>
+      <c r="H3" s="7" t="s">
         <v>109</v>
       </c>
-      <c r="F3" s="7" t="s">
-        <v>107</v>
-      </c>
-      <c r="G3" s="7" t="s">
-        <v>107</v>
-      </c>
-      <c r="H3" s="7" t="s">
+      <c r="I3" s="7" t="s">
         <v>110</v>
       </c>
-      <c r="I3" s="7" t="s">
-        <v>111</v>
-      </c>
       <c r="J3" s="7" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="K3" s="7" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="L3" s="7" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="M3" s="7"/>
       <c r="N3" s="7"/>
@@ -3889,37 +3890,37 @@
         <v>3</v>
       </c>
       <c r="B4" s="7" t="s">
+        <v>109</v>
+      </c>
+      <c r="C4" s="7" t="s">
+        <v>106</v>
+      </c>
+      <c r="D4" s="7" t="s">
+        <v>109</v>
+      </c>
+      <c r="E4" s="7" t="s">
         <v>110</v>
       </c>
-      <c r="C4" s="7" t="s">
-        <v>107</v>
-      </c>
-      <c r="D4" s="7" t="s">
+      <c r="F4" s="7" t="s">
+        <v>109</v>
+      </c>
+      <c r="G4" s="7" t="s">
+        <v>109</v>
+      </c>
+      <c r="H4" s="7" t="s">
+        <v>106</v>
+      </c>
+      <c r="I4" s="7" t="s">
         <v>110</v>
       </c>
-      <c r="E4" s="7" t="s">
-        <v>111</v>
-      </c>
-      <c r="F4" s="7" t="s">
-        <v>110</v>
-      </c>
-      <c r="G4" s="7" t="s">
-        <v>110</v>
-      </c>
-      <c r="H4" s="7" t="s">
-        <v>107</v>
-      </c>
-      <c r="I4" s="7" t="s">
-        <v>111</v>
-      </c>
       <c r="J4" s="7" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="K4" s="7" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="L4" s="7" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="M4" s="7"/>
       <c r="N4" s="7"/>
@@ -3930,35 +3931,35 @@
         <v>4</v>
       </c>
       <c r="B5" s="8" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="C5" s="7" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="D5" s="7"/>
       <c r="E5" s="7" t="s">
+        <v>110</v>
+      </c>
+      <c r="F5" s="8" t="s">
         <v>111</v>
       </c>
-      <c r="F5" s="8" t="s">
+      <c r="G5" s="7" t="s">
+        <v>109</v>
+      </c>
+      <c r="H5" s="7" t="s">
+        <v>109</v>
+      </c>
+      <c r="I5" s="7" t="s">
+        <v>110</v>
+      </c>
+      <c r="J5" s="7" t="s">
+        <v>109</v>
+      </c>
+      <c r="K5" s="9" t="s">
         <v>112</v>
       </c>
-      <c r="G5" s="7" t="s">
-        <v>110</v>
-      </c>
-      <c r="H5" s="7" t="s">
-        <v>110</v>
-      </c>
-      <c r="I5" s="7" t="s">
-        <v>111</v>
-      </c>
-      <c r="J5" s="7" t="s">
-        <v>110</v>
-      </c>
-      <c r="K5" s="9" t="s">
-        <v>113</v>
-      </c>
       <c r="L5" s="7" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="M5" s="7"/>
       <c r="N5" s="7"/>
@@ -3969,33 +3970,33 @@
         <v>5</v>
       </c>
       <c r="B6" s="7" t="s">
+        <v>109</v>
+      </c>
+      <c r="C6" s="8" t="s">
+        <v>111</v>
+      </c>
+      <c r="D6" s="7" t="s">
+        <v>109</v>
+      </c>
+      <c r="E6" s="7" t="s">
         <v>110</v>
       </c>
-      <c r="C6" s="8" t="s">
-        <v>112</v>
-      </c>
-      <c r="D6" s="7" t="s">
-        <v>110</v>
-      </c>
-      <c r="E6" s="7" t="s">
+      <c r="F6" s="7" t="s">
+        <v>109</v>
+      </c>
+      <c r="G6" s="8" t="s">
         <v>111</v>
       </c>
-      <c r="F6" s="7" t="s">
-        <v>110</v>
-      </c>
-      <c r="G6" s="8" t="s">
-        <v>112</v>
-      </c>
       <c r="H6" s="7" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="I6" s="7"/>
       <c r="J6" s="7" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="K6" s="7"/>
       <c r="L6" s="7" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="M6" s="7"/>
       <c r="N6" s="7"/>
@@ -4006,37 +4007,37 @@
         <v>6</v>
       </c>
       <c r="B7" s="7" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="C7" s="7" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="D7" s="7" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="E7" s="7" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="F7" s="7" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="G7" s="7" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="H7" s="7" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="I7" s="7" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="J7" s="7" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="K7" s="7" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="L7" s="7" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="M7" s="7"/>
       <c r="N7" s="7"/>
@@ -4048,30 +4049,30 @@
       </c>
       <c r="B8" s="7"/>
       <c r="C8" s="7" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="D8" s="7"/>
       <c r="E8" s="7" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="F8" s="7"/>
       <c r="G8" s="7" t="s">
+        <v>109</v>
+      </c>
+      <c r="H8" s="7" t="s">
+        <v>109</v>
+      </c>
+      <c r="I8" s="7" t="s">
         <v>110</v>
       </c>
-      <c r="H8" s="7" t="s">
-        <v>110</v>
-      </c>
-      <c r="I8" s="7" t="s">
-        <v>111</v>
-      </c>
       <c r="J8" s="7" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="K8" s="7" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="L8" s="7" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="M8" s="7"/>
       <c r="N8" s="7"/>
@@ -4085,7 +4086,7 @@
       <c r="C9" s="7"/>
       <c r="D9" s="7"/>
       <c r="E9" s="7" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="F9" s="7"/>
       <c r="G9" s="7"/>
@@ -4103,24 +4104,24 @@
         <v>9</v>
       </c>
       <c r="B10" s="7" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="C10" s="7"/>
       <c r="D10" s="7" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="E10" s="7" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="F10" s="7"/>
       <c r="G10" s="7"/>
       <c r="H10" s="7"/>
       <c r="I10" s="7" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="J10" s="7"/>
       <c r="K10" s="7" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="L10" s="7"/>
       <c r="M10" s="7"/>
@@ -4132,35 +4133,35 @@
         <v>10</v>
       </c>
       <c r="B11" s="7" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="C11" s="7" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="D11" s="7" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="E11" s="7" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="F11" s="7" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="G11" s="7" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="H11" s="7" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="I11" s="7" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="J11" s="7"/>
       <c r="K11" s="7" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="L11" s="7" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="M11" s="7"/>
       <c r="N11" s="7"/>

</xml_diff>

<commit_message>
Design+Dev: Added automatic Status Effect descriptions on Abilities.
</commit_message>
<xml_diff>
--- a/Design/Tables.xlsx
+++ b/Design/Tables.xlsx
@@ -2264,7 +2264,10 @@
       <c r="F8" s="17">
         <v>-3</v>
       </c>
-      <c r="G8"/>
+      <c r="G8">
+        <f>2*5.5</f>
+        <v>11</v>
+      </c>
       <c r="H8" s="22"/>
       <c r="K8" s="21"/>
     </row>
@@ -2287,10 +2290,7 @@
       <c r="F9" s="27">
         <v>0</v>
       </c>
-      <c r="G9">
-        <f>7*3.5</f>
-        <v>24.5</v>
-      </c>
+      <c r="G9"/>
       <c r="H9" s="20"/>
       <c r="J9" s="28"/>
       <c r="K9" s="21"/>
@@ -2359,10 +2359,7 @@
       <c r="F12" s="33">
         <v>-3</v>
       </c>
-      <c r="G12" s="10">
-        <f>18+6</f>
-        <v>24</v>
-      </c>
+      <c r="G12" s="10"/>
       <c r="H12" s="21"/>
       <c r="I12" s="21"/>
       <c r="J12" s="21"/>
@@ -2387,10 +2384,7 @@
       <c r="F13" s="13">
         <v>3</v>
       </c>
-      <c r="G13" s="10">
-        <f>6*4.5</f>
-        <v>27</v>
-      </c>
+      <c r="G13" s="10"/>
       <c r="H13" s="21"/>
       <c r="I13" s="21"/>
       <c r="J13" s="21"/>
@@ -2415,10 +2409,7 @@
       <c r="F14" s="33">
         <v>5.5</v>
       </c>
-      <c r="G14" s="10">
-        <f>6*3.5</f>
-        <v>21</v>
-      </c>
+      <c r="G14" s="10"/>
       <c r="H14" s="21"/>
       <c r="I14" s="21"/>
       <c r="J14" s="21"/>

</xml_diff>

<commit_message>
Design: Finished Lightning Font. It's alright.
</commit_message>
<xml_diff>
--- a/Design/Tables.xlsx
+++ b/Design/Tables.xlsx
@@ -2264,10 +2264,7 @@
       <c r="F8" s="17">
         <v>-3</v>
       </c>
-      <c r="G8">
-        <f>2*5.5</f>
-        <v>11</v>
-      </c>
+      <c r="G8"/>
       <c r="H8" s="22"/>
       <c r="K8" s="21"/>
     </row>
@@ -2336,7 +2333,10 @@
       <c r="F11" s="17">
         <v>-2</v>
       </c>
-      <c r="G11"/>
+      <c r="G11">
+        <f>11+4.5</f>
+        <v>15.5</v>
+      </c>
       <c r="H11" s="22"/>
       <c r="K11" s="21"/>
     </row>

</xml_diff>

<commit_message>
Design: Worked on Wizard. Decent.
</commit_message>
<xml_diff>
--- a/Design/Tables.xlsx
+++ b/Design/Tables.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="20475" windowHeight="12300"/>
+    <workbookView windowWidth="20475" windowHeight="12900"/>
   </bookViews>
   <sheets>
     <sheet name="Standard" sheetId="3" r:id="rId1"/>
@@ -33,7 +33,7 @@
     <t>Action Points</t>
   </si>
   <si>
-    <t>Charges</t>
+    <t>Mana</t>
   </si>
   <si>
     <t>Damage (3.5 Armor)</t>
@@ -2311,6 +2311,10 @@
       <c r="F10" s="17">
         <v>-1</v>
       </c>
+      <c r="G10">
+        <f>27+2*4.5</f>
+        <v>36</v>
+      </c>
       <c r="H10" s="22"/>
       <c r="K10" s="21"/>
     </row>
@@ -2334,8 +2338,8 @@
         <v>-2</v>
       </c>
       <c r="G11">
-        <f>11+4.5</f>
-        <v>15.5</v>
+        <f>18.5+4.5</f>
+        <v>23</v>
       </c>
       <c r="H11" s="22"/>
       <c r="K11" s="21"/>
@@ -2359,7 +2363,10 @@
       <c r="F12" s="33">
         <v>-3</v>
       </c>
-      <c r="G12" s="10"/>
+      <c r="G12" s="10">
+        <f>9*2.5</f>
+        <v>22.5</v>
+      </c>
       <c r="H12" s="21"/>
       <c r="I12" s="21"/>
       <c r="J12" s="21"/>

</xml_diff>